<commit_message>
problems of review tab rendering, and export file fidelity seem fixed
</commit_message>
<xml_diff>
--- a/tests/test_outputs/full_export_20260228.xlsx
+++ b/tests/test_outputs/full_export_20260228.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:CR28"/>
+  <dimension ref="A1:CF23"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -582,255 +582,195 @@
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>raw_F_stat</t>
+          <t>raw_beta</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
         <is>
+          <t>raw_se_beta</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
           <t>raw_p_value</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
-        <is>
-          <t>raw_n_control</t>
-        </is>
-      </c>
       <c r="AW1" s="1" t="inlineStr">
         <is>
-          <t>raw_n_treatment</t>
+          <t>raw_multiple_predictors</t>
         </is>
       </c>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>raw_mean_control</t>
+          <t>raw_beta_type</t>
         </is>
       </c>
       <c r="AY1" s="1" t="inlineStr">
         <is>
-          <t>raw_mean_treatment</t>
+          <t>raw_n_predictors</t>
         </is>
       </c>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
-          <t>raw_chi_square_stat</t>
+          <t>raw_group_a_df</t>
         </is>
       </c>
       <c r="BA1" s="1" t="inlineStr">
         <is>
-          <t>raw_var_value_control</t>
+          <t>raw_group_a_F_stat</t>
         </is>
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
-          <t>raw_var_statistic_type</t>
+          <t>raw_group_a_t_stat</t>
         </is>
       </c>
       <c r="BC1" s="1" t="inlineStr">
         <is>
-          <t>raw_control_description</t>
+          <t>raw_group_a_p_value</t>
         </is>
       </c>
       <c r="BD1" s="1" t="inlineStr">
         <is>
-          <t>raw_use_small_sd_approx</t>
+          <t>raw_group_a_n_control</t>
         </is>
       </c>
       <c r="BE1" s="1" t="inlineStr">
         <is>
-          <t>raw_var_value_treatment</t>
+          <t>raw_group_a_n_treatment</t>
         </is>
       </c>
       <c r="BF1" s="1" t="inlineStr">
         <is>
-          <t>raw_treatment_description</t>
+          <t>raw_group_a_mean_control</t>
         </is>
       </c>
       <c r="BG1" s="1" t="inlineStr">
         <is>
-          <t>raw_beta</t>
+          <t>raw_group_a_study_design</t>
         </is>
       </c>
       <c r="BH1" s="1" t="inlineStr">
         <is>
-          <t>raw_se_beta</t>
+          <t>raw_group_a_mean_treatment</t>
         </is>
       </c>
       <c r="BI1" s="1" t="inlineStr">
         <is>
-          <t>raw_multiple_predictors</t>
+          <t>raw_group_a_chi_square_stat</t>
         </is>
       </c>
       <c r="BJ1" s="1" t="inlineStr">
         <is>
-          <t>raw_beta_type</t>
+          <t>raw_group_a_var_value_control</t>
         </is>
       </c>
       <c r="BK1" s="1" t="inlineStr">
         <is>
-          <t>raw_n_predictors</t>
+          <t>raw_group_a_var_statistic_type</t>
         </is>
       </c>
       <c r="BL1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_df</t>
+          <t>raw_group_a_control_description</t>
         </is>
       </c>
       <c r="BM1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_F_stat</t>
+          <t>raw_group_a_use_small_sd_approx</t>
         </is>
       </c>
       <c r="BN1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_t_stat</t>
+          <t>raw_group_a_var_value_treatment</t>
         </is>
       </c>
       <c r="BO1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_p_value</t>
+          <t>raw_group_a_treatment_description</t>
         </is>
       </c>
       <c r="BP1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_n_control</t>
+          <t>raw_group_b_df</t>
         </is>
       </c>
       <c r="BQ1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_n_treatment</t>
+          <t>raw_group_b_F_stat</t>
         </is>
       </c>
       <c r="BR1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_mean_control</t>
+          <t>raw_group_b_t_stat</t>
         </is>
       </c>
       <c r="BS1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_study_design</t>
+          <t>raw_group_b_p_value</t>
         </is>
       </c>
       <c r="BT1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_mean_treatment</t>
+          <t>raw_group_b_n_control</t>
         </is>
       </c>
       <c r="BU1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_chi_square_stat</t>
+          <t>raw_group_b_n_treatment</t>
         </is>
       </c>
       <c r="BV1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_var_value_control</t>
+          <t>raw_group_b_mean_control</t>
         </is>
       </c>
       <c r="BW1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_var_statistic_type</t>
+          <t>raw_group_b_study_design</t>
         </is>
       </c>
       <c r="BX1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_control_description</t>
+          <t>raw_group_b_mean_treatment</t>
         </is>
       </c>
       <c r="BY1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_use_small_sd_approx</t>
+          <t>raw_group_b_chi_square_stat</t>
         </is>
       </c>
       <c r="BZ1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_var_value_treatment</t>
+          <t>raw_group_b_var_value_control</t>
         </is>
       </c>
       <c r="CA1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_a_treatment_description</t>
+          <t>raw_group_b_var_statistic_type</t>
         </is>
       </c>
       <c r="CB1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_b_df</t>
+          <t>raw_group_b_control_description</t>
         </is>
       </c>
       <c r="CC1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_b_F_stat</t>
+          <t>raw_group_b_use_small_sd_approx</t>
         </is>
       </c>
       <c r="CD1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_b_t_stat</t>
+          <t>raw_group_b_var_value_treatment</t>
         </is>
       </c>
       <c r="CE1" s="1" t="inlineStr">
         <is>
-          <t>raw_group_b_p_value</t>
+          <t>raw_group_b_treatment_description</t>
         </is>
       </c>
       <c r="CF1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_n_control</t>
-        </is>
-      </c>
-      <c r="CG1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_n_treatment</t>
-        </is>
-      </c>
-      <c r="CH1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_mean_control</t>
-        </is>
-      </c>
-      <c r="CI1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_study_design</t>
-        </is>
-      </c>
-      <c r="CJ1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_mean_treatment</t>
-        </is>
-      </c>
-      <c r="CK1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_chi_square_stat</t>
-        </is>
-      </c>
-      <c r="CL1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_var_value_control</t>
-        </is>
-      </c>
-      <c r="CM1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_var_statistic_type</t>
-        </is>
-      </c>
-      <c r="CN1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_control_description</t>
-        </is>
-      </c>
-      <c r="CO1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_use_small_sd_approx</t>
-        </is>
-      </c>
-      <c r="CP1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_var_value_treatment</t>
-        </is>
-      </c>
-      <c r="CQ1" s="1" t="inlineStr">
-        <is>
-          <t>raw_group_b_treatment_description</t>
-        </is>
-      </c>
-      <c r="CR1" s="1" t="inlineStr">
         <is>
           <t>raw_interaction_pathway</t>
         </is>
@@ -1027,7 +967,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-02-28T12:14:50+00:00</t>
+          <t>2026-03-01T11:52:42+00:00</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1118,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-02-28T12:14:50+00:00</t>
+          <t>2026-03-01T11:52:42+00:00</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1157,34 +1097,103 @@
       <c r="R5" t="inlineStr">
         <is>
           <t>Paris</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>29c4acf0-94b3-4952-b829-10937bcf18e8</t>
+        </is>
+      </c>
+      <c r="V5">
+        <v>0.8</v>
+      </c>
+      <c r="W5">
+        <v>1.09861228866811</v>
+      </c>
+      <c r="X5">
+        <v>0.05882352941176471</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>calculated</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="AH5" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>correlation</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>Observational</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Ind. health or growth</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="AP5" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>Continuous</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4f8fa6f3-7345-494c-a01e-fdd0d6a6e0f0</t>
+          <t>6b26fc7f-966b-4fe8-8065-d5d00cdecdd8</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>study_site_2</t>
         </is>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Soil microbial community responses to nitrogen enrichment in alpine meadows</t>
+          <t>Sexual selection and mate choice in socially monogamous passerine birds</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Okonkwo CE; Svensson AB; Pires LM</t>
+          <t>Valente EF; Costa PA; Dumont R</t>
         </is>
       </c>
       <c r="F6">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>10.1890/15-1432.1</t>
+          <t>10.1098/rspb.2017.2389</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1199,12 +1208,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-02-28T12:19:44+00:00</t>
+          <t>2026-03-01T11:52:42+00:00</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Toronto, Golden Horseshoe, Ontario, Canada; 43.6535; -79.3839; 324211</t>
+          <t>Paris, Ile-de-France, Metropolitan France, France; 48.8589; 2.32; 7444</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1214,12 +1223,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Forest</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>invited reviewer test</t>
+          <t>frn</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1229,15 +1238,131 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>simple_group</t>
+          <t>study_site</t>
         </is>
       </c>
       <c r="Q6">
-        <v>1</v>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>2026-02-22</t>
+        <v>2</v>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Interaction pathway B</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>c72701cb-7fe6-4331-a857-2acf31ca2772</t>
+        </is>
+      </c>
+      <c r="V6">
+        <v>-0.2737345791026131</v>
+      </c>
+      <c r="W6">
+        <v>-0.2808964681192619</v>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>calculated_relative</t>
+        </is>
+      </c>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>interaction</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>Observational</t>
+        </is>
+      </c>
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Ind. health or growth</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP6" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="AQ6" t="inlineStr">
+        <is>
+          <t>Categorical</t>
+        </is>
+      </c>
+      <c r="BD6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="BF6" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="BG6" t="inlineStr">
+        <is>
+          <t>control_treatment</t>
+        </is>
+      </c>
+      <c r="BH6" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="BJ6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="BM6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BN6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="BR6" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="BW6" t="inlineStr">
+        <is>
+          <t>control_treatment</t>
+        </is>
+      </c>
+      <c r="CC6" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="CF6" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1247,11 +1372,6 @@
           <t>4f8fa6f3-7345-494c-a01e-fdd0d6a6e0f0</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
-        </is>
-      </c>
       <c r="C7">
         <v>4</v>
       </c>
@@ -1285,7 +1405,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-02-28T12:19:44+00:00</t>
+          <t>2026-03-01T11:21:49+00:00</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1315,43 +1435,48 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q7">
         <v>1</v>
       </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Interaction path B</t>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2026-02-22</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
+          <t>4f8fa6f3-7345-494c-a01e-fdd0d6a6e0f0</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>study_site_1</t>
         </is>
       </c>
       <c r="C8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Freshwater fish diversity responses to dam removal across temperate watersheds</t>
+          <t>Soil microbial community responses to nitrogen enrichment in alpine meadows</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Huang JX; Torres MM; Eriksen S</t>
+          <t>Okonkwo CE; Svensson AB; Pires LM</t>
         </is>
       </c>
       <c r="F8">
-        <v>2020</v>
+        <v>2016</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10.1007/s10750-020-04321-y</t>
+          <t>10.1890/15-1432.1</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1366,12 +1491,17 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
+          <t>2026-03-01T11:21:49+00:00</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Toronto, Golden Horseshoe, Ontario, Canada; 43.6535; -79.3839; 324211</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>lon_min=-40; lon_max=40; lat_min=0; lat_max=20</t>
+          <t>lon_min=; lon_max=; lat_min=; lat_max=</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1379,6 +1509,11 @@
           <t>Grassland</t>
         </is>
       </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>invited reviewer test</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1386,15 +1521,159 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>simple_group</t>
+          <t>study_site</t>
         </is>
       </c>
       <c r="Q8">
         <v>1</v>
       </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Interaction path B</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>60011ce2-35d1-40ce-b0ee-e2f611f46281</t>
+        </is>
+      </c>
+      <c r="V8">
+        <v>-0.4700130862035674</v>
+      </c>
+      <c r="W8">
+        <v>-0.5100871333106207</v>
+      </c>
+      <c r="X8">
+        <v>0.05405405405405406</v>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>calculated_relative</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>interaction</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>Experimental (ex-situ)</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Pop. size</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Proportion</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>Continuous</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>control_treatment</t>
+        </is>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="BN8" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="BT8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="BU8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>control_treatment</t>
+        </is>
+      </c>
+      <c r="BX8" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="BZ8" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="CA8" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="CC8" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="CD8" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="CF8" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1404,11 +1683,6 @@
           <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
-        </is>
-      </c>
       <c r="C9">
         <v>5</v>
       </c>
@@ -1442,7 +1716,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
+          <t>2026-03-01T11:27:57+00:00</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1462,76 +1736,15 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q9">
         <v>1</v>
       </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>test interaction path A</t>
-        </is>
-      </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>d6d07672-3dcd-474c-931c-9d6376d479ca</t>
-        </is>
-      </c>
-      <c r="V9">
-        <v>0.1621424235993525</v>
-      </c>
-      <c r="W9">
-        <v>0.1635861840335697</v>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>calculated</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="AI9" t="inlineStr">
-        <is>
-          <t>interaction</t>
-        </is>
-      </c>
-      <c r="AJ9" t="inlineStr">
-        <is>
-          <t>Experimental (ex-situ)</t>
-        </is>
-      </c>
-      <c r="AN9" t="inlineStr">
-        <is>
-          <t>Ind. behaviour</t>
-        </is>
-      </c>
-      <c r="AO9" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AP9" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="AQ9" t="inlineStr">
-        <is>
-          <t>Categorical</t>
-        </is>
-      </c>
-      <c r="CR9" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
@@ -1579,7 +1792,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
+          <t>2026-03-01T11:27:57+00:00</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1607,66 +1820,49 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>test interaction path A</t>
+          <t>Correlation test</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>7a896a01-9251-472c-a3d6-73ad75ce97a1</t>
+          <t>ab07313d-1edb-4992-b116-fd70fc4ab40f</t>
         </is>
       </c>
       <c r="V10">
-        <v>0.2452557357939863</v>
+        <v>0.8</v>
       </c>
       <c r="W10">
-        <v>0.2503586145588892</v>
+        <v>1.09861228866811</v>
+      </c>
+      <c r="X10">
+        <v>0.05882352941176471</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
           <t>calculated</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG10" t="inlineStr">
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
         <is>
           <t>0.8</t>
         </is>
       </c>
       <c r="AI10" t="inlineStr">
         <is>
-          <t>control_treatment</t>
-        </is>
-      </c>
-      <c r="AJ10" t="inlineStr">
-        <is>
-          <t>Experimental (ex-situ)</t>
-        </is>
-      </c>
-      <c r="AN10" t="inlineStr">
-        <is>
-          <t>Ind. behaviour</t>
+          <t>correlation</t>
         </is>
       </c>
       <c r="AO10" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP10" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="AQ10" t="inlineStr">
-        <is>
-          <t>Categorical</t>
-        </is>
-      </c>
-      <c r="BD10" t="inlineStr">
         <is>
           <t>FALSE</t>
         </is>
@@ -1680,7 +1876,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>study_site_1</t>
+          <t>study_site_2</t>
         </is>
       </c>
       <c r="C11">
@@ -1716,7 +1912,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
+          <t>2026-03-01T11:27:57+00:00</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
@@ -1740,16 +1936,16 @@
         </is>
       </c>
       <c r="Q11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>test interaction path A</t>
+          <t>Interaction pathway A</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>7b055485-cfd7-4dd0-bb8f-7016c59f8f6a</t>
+          <t>72256061-2d89-4069-83a2-5299ec4d61b6</t>
         </is>
       </c>
       <c r="V11">
@@ -1780,7 +1976,7 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>Observational</t>
+          <t>Simulation</t>
         </is>
       </c>
       <c r="AN11" t="inlineStr">
@@ -1803,7 +1999,7 @@
           <t>Continuous</t>
         </is>
       </c>
-      <c r="CR11" t="inlineStr">
+      <c r="CF11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
@@ -1812,33 +2008,28 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
+          <t>a9080bd1-ec0f-4308-aca5-cb2e2123e1e8</t>
         </is>
       </c>
       <c r="C12">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Freshwater fish diversity responses to dam removal across temperate watersheds</t>
+          <t>Plant trait plasticity mediates competitive outcomes under drought stress in grasslands</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Huang JX; Torres MM; Eriksen S</t>
+          <t>Ferreira AB; Marchetti DG; Klein R</t>
         </is>
       </c>
       <c r="F12">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>10.1007/s10750-020-04321-y</t>
+          <t>10.1111/nph.17208</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1853,12 +2044,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>lon_min=-40; lon_max=40; lat_min=0; lat_max=20</t>
+          <t>2026-02-28T09:27:26+00:00</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1866,6 +2057,11 @@
           <t>Grassland</t>
         </is>
       </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
       <c r="O12" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -1873,109 +2069,48 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q12">
         <v>1</v>
       </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>test interaction path A</t>
-        </is>
-      </c>
-      <c r="U12" t="inlineStr">
-        <is>
-          <t>bfc60512-8706-42e0-bcf0-2f079b79a038</t>
-        </is>
-      </c>
-      <c r="V12">
-        <v>0.1621424235993525</v>
-      </c>
-      <c r="W12">
-        <v>0.1635861840335697</v>
-      </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>calculated</t>
-        </is>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="AG12" t="inlineStr">
-        <is>
-          <t>0.9</t>
-        </is>
-      </c>
-      <c r="AI12" t="inlineStr">
-        <is>
-          <t>interaction</t>
-        </is>
-      </c>
-      <c r="AJ12" t="inlineStr">
-        <is>
-          <t>Experimental (ex-situ)</t>
-        </is>
-      </c>
-      <c r="AN12" t="inlineStr">
-        <is>
-          <t>Ind. behaviour</t>
-        </is>
-      </c>
-      <c r="AO12" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="AP12" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="AQ12" t="inlineStr">
-        <is>
-          <t>Categorical</t>
-        </is>
-      </c>
-      <c r="CR12" t="inlineStr">
-        <is>
-          <t>A</t>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
+          <t>a9080bd1-ec0f-4308-aca5-cb2e2123e1e8</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>study_site_2</t>
+          <t>study_site_1</t>
         </is>
       </c>
       <c r="C13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Freshwater fish diversity responses to dam removal across temperate watersheds</t>
+          <t>Plant trait plasticity mediates competitive outcomes under drought stress in grasslands</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Huang JX; Torres MM; Eriksen S</t>
+          <t>Ferreira AB; Marchetti DG; Klein R</t>
         </is>
       </c>
       <c r="F13">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>10.1007/s10750-020-04321-y</t>
+          <t>10.1111/nph.17208</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1990,12 +2125,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>lon_min=-40; lon_max=40; lat_min=0; lat_max=20</t>
+          <t>2026-02-28T09:27:26+00:00</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -2003,6 +2138,11 @@
           <t>Grassland</t>
         </is>
       </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
       <c r="O13" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2014,105 +2154,34 @@
         </is>
       </c>
       <c r="Q13">
-        <v>2</v>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>Test effect size 2</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>72256061-2d89-4069-83a2-5299ec4d61b6</t>
-        </is>
-      </c>
-      <c r="V13">
-        <v>0.2452557357939863</v>
-      </c>
-      <c r="W13">
-        <v>0.2503586145588892</v>
-      </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>calculated</t>
-        </is>
-      </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG13" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="AI13" t="inlineStr">
-        <is>
-          <t>control_treatment</t>
-        </is>
-      </c>
-      <c r="AJ13" t="inlineStr">
-        <is>
-          <t>Experimental (ex-situ)</t>
-        </is>
-      </c>
-      <c r="AN13" t="inlineStr">
-        <is>
-          <t>Ind. behaviour</t>
-        </is>
-      </c>
-      <c r="AO13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP13" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="AQ13" t="inlineStr">
-        <is>
-          <t>Categorical</t>
-        </is>
-      </c>
-      <c r="BD13" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>study_site_2</t>
+          <t>bb15055d-5902-4cdc-858b-0e19fb32777f</t>
         </is>
       </c>
       <c r="C14">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Freshwater fish diversity responses to dam removal across temperate watersheds</t>
+          <t>Population-level effects of light pollution on nocturnal insect communities</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Huang JX; Torres MM; Eriksen S</t>
+          <t>Thompson LD; O'Brien KA; Mwangi PK</t>
         </is>
       </c>
       <c r="F14">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>10.1007/s10750-020-04321-y</t>
+          <t>10.1098/rsbl.2019.0367</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2127,12 +2196,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>lon_min=-40; lon_max=40; lat_min=0; lat_max=20</t>
+          <t>2026-02-28T09:27:29+00:00</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -2140,6 +2209,11 @@
           <t>Grassland</t>
         </is>
       </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
       <c r="O14" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2147,109 +2221,43 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q14">
-        <v>2</v>
-      </c>
-      <c r="R14" t="inlineStr">
-        <is>
-          <t>Test effect size 2</t>
-        </is>
-      </c>
-      <c r="U14" t="inlineStr">
-        <is>
-          <t>7e563b92-0209-46ca-b750-36d3d0fe1c08</t>
-        </is>
-      </c>
-      <c r="V14">
-        <v>0.2452557357939863</v>
-      </c>
-      <c r="W14">
-        <v>0.2503586145588892</v>
-      </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>calculated</t>
-        </is>
-      </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG14" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="AI14" t="inlineStr">
-        <is>
-          <t>control_treatment</t>
-        </is>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>Experimental (ex-situ)</t>
-        </is>
-      </c>
-      <c r="AN14" t="inlineStr">
-        <is>
-          <t>Ind. behaviour</t>
-        </is>
-      </c>
-      <c r="AO14" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP14" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="AQ14" t="inlineStr">
-        <is>
-          <t>Categorical</t>
-        </is>
-      </c>
-      <c r="BD14" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
+          <t>bb15055d-5902-4cdc-858b-0e19fb32777f</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>study_site_2</t>
+          <t>study_site_1</t>
         </is>
       </c>
       <c r="C15">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Freshwater fish diversity responses to dam removal across temperate watersheds</t>
+          <t>Population-level effects of light pollution on nocturnal insect communities</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Huang JX; Torres MM; Eriksen S</t>
+          <t>Thompson LD; O'Brien KA; Mwangi PK</t>
         </is>
       </c>
       <c r="F15">
-        <v>2020</v>
+        <v>2019</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>10.1007/s10750-020-04321-y</t>
+          <t>10.1098/rsbl.2019.0367</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2264,12 +2272,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>lon_min=-40; lon_max=40; lat_min=0; lat_max=20</t>
+          <t>2026-02-28T09:27:29+00:00</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2277,6 +2285,11 @@
           <t>Grassland</t>
         </is>
       </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Scotland</t>
+        </is>
+      </c>
       <c r="O15" t="inlineStr">
         <is>
           <t>FALSE</t>
@@ -2288,108 +2301,34 @@
         </is>
       </c>
       <c r="Q15">
-        <v>2</v>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Test effect size 2</t>
-        </is>
-      </c>
-      <c r="U15" t="inlineStr">
-        <is>
-          <t>378c724c-f62e-46d5-9be1-343063060858</t>
-        </is>
-      </c>
-      <c r="V15">
-        <v>0.8</v>
-      </c>
-      <c r="W15">
-        <v>1.09861228866811</v>
-      </c>
-      <c r="X15">
-        <v>0.05882352941176471</v>
-      </c>
-      <c r="Y15" t="inlineStr">
-        <is>
-          <t>calculated</t>
-        </is>
-      </c>
-      <c r="AB15" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="AF15" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
-      </c>
-      <c r="AH15" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="AI15" t="inlineStr">
-        <is>
-          <t>correlation</t>
-        </is>
-      </c>
-      <c r="AJ15" t="inlineStr">
-        <is>
-          <t>Experimental (ex-situ)</t>
-        </is>
-      </c>
-      <c r="AN15" t="inlineStr">
-        <is>
-          <t>Ind. behaviour</t>
-        </is>
-      </c>
-      <c r="AO15" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP15" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="AQ15" t="inlineStr">
-        <is>
-          <t>Categorical</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>fe938548-ee91-4d96-a3b1-48f452e33e9e</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>study_site_2</t>
+          <t>c284b312-98fe-45a7-9bb5-09261ed497d1</t>
         </is>
       </c>
       <c r="C16">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Freshwater fish diversity responses to dam removal across temperate watersheds</t>
+          <t>Herbivore-mediated nutrient cycling in semi-arid savanna ecosystems</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Huang JX; Torres MM; Eriksen S</t>
+          <t>Joubert MN; Pieterse AC; van der Berg J</t>
         </is>
       </c>
       <c r="F16">
-        <v>2020</v>
+        <v>2018</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>10.1007/s10750-020-04321-y</t>
+          <t>10.1111/1365-2745.13024</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2404,17 +2343,22 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-02-28T15:25:37+00:00</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>lon_min=-40; lon_max=40; lat_min=0; lat_max=20</t>
+          <t>2026-02-28T09:28:05+00:00</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Cairo, Egypt; 30.0444; 31.2357; 5466227</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Wetland</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -2424,104 +2368,48 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q16">
-        <v>2</v>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Test effect size 2</t>
-        </is>
-      </c>
-      <c r="U16" t="inlineStr">
-        <is>
-          <t>40fe7803-2e61-4a7f-94fc-a1e81ccfee19</t>
-        </is>
-      </c>
-      <c r="V16">
-        <v>0.2452557357939863</v>
-      </c>
-      <c r="W16">
-        <v>0.2503586145588892</v>
-      </c>
-      <c r="Y16" t="inlineStr">
-        <is>
-          <t>calculated</t>
-        </is>
-      </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="AG16" t="inlineStr">
-        <is>
-          <t>0.8</t>
-        </is>
-      </c>
-      <c r="AI16" t="inlineStr">
-        <is>
-          <t>control_treatment</t>
-        </is>
-      </c>
-      <c r="AJ16" t="inlineStr">
-        <is>
-          <t>Experimental (ex-situ)</t>
-        </is>
-      </c>
-      <c r="AN16" t="inlineStr">
-        <is>
-          <t>Ind. behaviour</t>
-        </is>
-      </c>
-      <c r="AO16" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="AP16" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="AQ16" t="inlineStr">
-        <is>
-          <t>Categorical</t>
-        </is>
-      </c>
-      <c r="BD16" t="inlineStr">
-        <is>
-          <t>FALSE</t>
+        <v>1</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>a9080bd1-ec0f-4308-aca5-cb2e2123e1e8</t>
+          <t>c284b312-98fe-45a7-9bb5-09261ed497d1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>study_site_1</t>
         </is>
       </c>
       <c r="C17">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Plant trait plasticity mediates competitive outcomes under drought stress in grasslands</t>
+          <t>Herbivore-mediated nutrient cycling in semi-arid savanna ecosystems</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ferreira AB; Marchetti DG; Klein R</t>
+          <t>Joubert MN; Pieterse AC; van der Berg J</t>
         </is>
       </c>
       <c r="F17">
-        <v>2021</v>
+        <v>2018</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>10.1111/nph.17208</t>
+          <t>10.1111/1365-2745.13024</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2536,22 +2424,22 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-02-28T09:27:26+00:00</t>
+          <t>2026-02-28T09:28:05+00:00</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
+          <t>Cairo, Egypt; 30.0444; 31.2357; 5466227</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Wetland</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -2561,48 +2449,38 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>simple_group</t>
+          <t>study_site</t>
         </is>
       </c>
       <c r="Q17">
         <v>1</v>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>a9080bd1-ec0f-4308-aca5-cb2e2123e1e8</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
+          <t>f255dc8a-e048-49cc-aad5-20bbdf70f5b4</t>
         </is>
       </c>
       <c r="C18">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Plant trait plasticity mediates competitive outcomes under drought stress in grasslands</t>
+          <t>Seed dispersal limitation constrains plant community recovery after tropical forest fragmentation</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ferreira AB; Marchetti DG; Klein R</t>
+          <t>Almeida FS; Ribeiro GH; Neves CT</t>
         </is>
       </c>
       <c r="F18">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>10.1111/nph.17208</t>
+          <t>10.1111/gcb.16157</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2617,22 +2495,22 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-02-28T09:27:26+00:00</t>
+          <t>2026-02-28T09:28:47+00:00</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
+          <t>Iceland; 64.9842; -18.1059; 299133; MultiPolygon; -25.0135; 65.5045; -25.0079; 65.4708; -24.9887; 65.4379; -24.4824; 64.7928; -23.7161; 63.6161; -23.6902; 63.5848; -23.6531; 63.5559; -23.6058; 63.5302; -23.5496; 63.5083; -23.4861; 63.4908; -23.4171; 63.4783; -23.3444; 63.4711; -23.2701; 63.4693; -23.1961; 63.473; -23.1245; 63.4822; -22.9863; 63.5055; -22.5; 63.4173; -20.774; 63.1019; -20.6951; 63.0905; -20.613; 63.0859; -20.5304; 63.0884; -19.0873; 63.1853; -18.7041; 63.185; -18.6405; 63.187; -18.5781; 63.193; -18.0646; 63.2592; -17.9667; 63.2776; -17.7678; 63.3278; -17.7098; 63.3452; -17.6585; 63.3664; -17.591; 63.399; -17.3177; 63.5463; -16.5809; 63.5876; -16.5117; 63.5937; -16.4455; 63.6046; -16.384; 63.62; -15.9349; 63.7523; -15.8562; 63.7813; -15.6952; 63.8557; -14.77; 64.0538; -14.705; 64.0704; -14.2054; 64.2218; -14.143; 64.2442; -13.793; 64.3932; -13.671; 64.4519; -13.6426; 64.469; -13.6153; 64.4534; -13.5739; 64.4357; -13.5109; 64.4157; -13.4897; 64.4104; -13.441; 64.4005; -13.416; 64.3965; -13.3664; 64.3907; -13.3379; 64.3884; -13.2862; 64.3863; -13.2578; 64.3862; -13.2054; 64.388; -13.178; 64.39; -13.1266; 64.3958; -13.1008; 64.3997; -13.052; 64.4094; -13.0287; 64.4151; -12.984; 64.4283; -12.9637; 64.4355; -12.9246; 64.4521; -12.8775; 64.4788; -12.8628; 64.4894; -12.8412; 64.5085; -12.83; 64.5211; -12.817; 64.5404; -12.8104; 64.5548; -12.8055; 64.5736; -12.8046; 64.5895; -12.8071; 64.6071; -12.813; 64.6241; -12.8218; 64.6401; -12.8352; 64.6575; -12.8492; 64.6715; -12.8708; 64.6887; -12.8886; 64.7005; -12.9185; 64.7169; -12.939; 64.7263; -12.9771; 64.741; -13.0446; 64.7604; -13.1191; 64.7744; -13.1983; 64.7827; -13.2196; 64.7833; -13.2053; 64.7938; -13.1328; 64.838; -13.0828; 64.8768; -13.0662; 64.894; -13.0437; 64.9236; -13.0322; 64.9544; -13.0138; 65.0538; -13.0134; 65.0826; -13.031; 65.1902; -13.1236; 65.5252; -13.1359; 65.5523; -13.1572; 65.5785; -14.063; 66.4484; -14.1044; 66.479; -14.1587; 66.5063; -14.2241; 66.5294; -14.2987; 66.5475; -14.3802; 66.5601; -15.8898; 66.7267; -16.0151; 66.7333; -16.184; 66.7335; -16.2977; 66.7285; -16.6492; 66.696; -16.7327; 66.685; -16.8101; 66.6684; -16.8788; 66.6467; -17.3761; 66.4565; -17.5468; 66.4292; -17.5259; 66.444; -17.4973; 66.4761; -17.4827; 66.5096; -17.4808; 66.5592; -17.4956; 66.5912; -17.5189; 66.6195; -17.55; 66.6444; -17.5809; 66.665; -17.6304; 66.6926; -17.6864; 66.7154; -17.7304; 66.7291; -17.8096; 66.7473; -17.8959; 66.7595; -17.9863; 66.7653; -18.078; 66.7644; -18.1677; 66.757; -18.2524; 66.7432; -18.3296; 66.7237; -18.3952; 66.6995; -18.4487; 66.671; -18.4886; 66.6393; -18.5136; 66.6052; -18.5187; 66.5857; -18.525; 66.574; -18.5279; 66.5383; -18.5147; 66.5029; -18.5008; 66.4866; -18.4924; 66.4728; -18.4581; 66.4423; -18.4136; 66.4155; -18.3591; 66.3919; -18.3171; 66.3769; -18.8; 66.3851; -18.8604; 66.3845; -20.1192; 66.3368; -22.1606; 66.6292; -22.2041; 66.6386; -22.2962; 66.6543; -22.3748; 66.6626; -22.4558; 66.6656; -22.5; 66.6642; -22.5442; 66.6629; -22.5969; 66.657; -22.878; 66.6662; -22.977; 66.6655; -23.0737; 66.657; -23.1641; 66.6411; -23.3815; 66.5918; -23.4683; 66.5668; -23.5396; 66.5349; -24.1866; 66.1666; -24.2216; 66.1429; -24.5265; 65.8973; -24.9484; 65.6014; -24.9834; 65.5708; -25.0053; 65.5382; -25.0135; 65.5045; -19.1995; 67.151; -19.1994; 67.149; -19.1993; 67.147; -19.1992; 67.145; -19.199; 67.143; -19.1987; 67.141; -19.1984; 67.139; -19.198; 67.137; -19.1976; 67.135; -19.1972; 67.133; -19.1967; 67.131; -19.1961; 67.129; -19.1955; 67.127; -19.1948; 67.125; -19.1941; 67.123; -19.1933; 67.121; -19.1925; 67.119; -19.1916; 67.117; -19.1907; 67.115; -19.1897; 67.113; -19.1886; 67.111; -19.1875; 67.109; -19.1864; 67.107; -19.1852; 67.105; -19.1839; 67.103; -19.1826; 67.101; -19.1812; 67.099; -19.1798; 67.097; -19.1784; 67.095; -19.177; 67.093; -19.1755; 67.091; -19.1739; 67.089; -19.1722; 67.087; -19.1705; 67.085; -19.1688; 67.083; -19.167; 67.081; -19.1651; 67.079; -19.1631; 67.077; -19.1611; 67.075; -19.1591; 67.073; -19.1569; 67.071; -19.1547; 67.069; -19.1525; 67.067; -19.1502; 67.065; -19.1478; 67.063; -19.1453; 67.061; -19.1428; 67.059; -19.1415; 67.058; -19.1401; 67.057; -19.1388; 67.056; -19.1375; 67.055; -19.1361; 67.054; -19.1347; 67.053; -19.1333; 67.052; -19.1319; 67.051; -19.1304; 67.05; -19.129; 67.049; -19.1275; 67.048; -19.126; 67.047; -19.1245; 67.046; -19.1229; 67.045; -19.1214; 67.044; -19.1198; 67.043; -19.1182; 67.042; -19.1165; 67.041; -19.1149; 67.04; -19.1132; 67.039; -19.1115; 67.038; -19.1098; 67.037; -19.1081; 67.036; -19.1063; 67.035; -19.1046; 67.034; -19.1028; 67.033; -19.1009; 67.032; -19.0991; 67.031; -19.0972; 67.03; -19.0953; 67.029; -19.0934; 67.028; -19.0914; 67.027; -19.0895; 67.026; -19.0875; 67.025; -19.0854; 67.024; -19.0834; 67.023; -19.0813; 67.022; -19.0792; 67.021; -19.0771; 67.02; -19.0749; 67.019; -19.0727; 67.018; -19.0705; 67.017; -19.0683; 67.016; -19.066; 67.015; -19.0637; 67.014; -19.0613; 67.013; -19.059; 67.012; -19.0566; 67.011; -19.0541; 67.01; -19.0516; 67.009; -19.0491; 67.008; -19.0466; 67.007; -19.044; 67.006; -19.0414; 67.005; -19.0388; 67.004; -19.0361; 67.003; -19.0333; 67.002; -19.0306; 67.001; -19.0278; 67; -19.0249; 66.999; -19.022; 66.998; -19.0191; 66.997; -19.0161; 66.996; -19.013; 66.995; -19.01; 66.994; -19.0068; 66.993; -19.0037; 66.992; -19.0004; 66.991; -18.9971; 66.99; -18.9938; 66.989; -18.9904; 66.988; -18.9869; 66.987; -18.9834; 66.986; -18.9798; 66.985; -18.9762; 66.984; -18.9725; 66.983; -18.9687; 66.982; -18.9648; 66.981; -18.9609; 66.98; -18.9569; 66.979; -18.9528; 66.978; -18.9486; 66.977; -18.9443; 66.976; -18.9399; 66.975; -18.9355; 66.974; -18.9309; 66.973; -18.9262; 66.972; -18.9213; 66.971; -18.9164; 66.97; -18.9113; 66.969; -18.9061; 66.968; -18.9007; 66.967; -18.8952; 66.966; -18.8895; 66.965; -18.8835; 66.964; -18.8774; 66.963; -18.871; 66.962; -18.8644; 66.961; -18.8575; 66.96; -18.8503; 66.959; -18.8427; 66.958; -18.8346; 66.957; -18.8261; 66.956; -18.817; 66.955; -18.8072; 66.954; -18.7965; 66.953; -18.7846; 66.952; -18.7711; 66.951; -18.755; 66.95; -18.734; 66.949; -18.6888; 66.948; -18.6751; 66.948; -18.6299; 66.949; -18.6089; 66.95; -18.5928; 66.951; -18.5793; 66.952; -18.5674; 66.953; -18.5567; 66.954; -18.5469; 66.955; -18.5378; 66.956; -18.5293; 66.957; -18.5212; 66.958; -18.5136; 66.959; -18.5064; 66.96; -18.4995; 66.961; -18.4929; 66.962; -18.4865; 66.963; -18.4804; 66.964; -18.4744; 66.965; -18.4687; 66.966; -18.4632; 66.967; -18.4578; 66.968; -18.4526; 66.969; -18.4475; 66.97; -18.4425; 66.971; -18.4377; 66.972; -18.433; 66.973; -18.4284; 66.974; -18.424; 66.975; -18.4196; 66.976; -18.4153; 66.977; -18.4111; 66.978; -18.407; 66.979; -18.403; 66.98; -18.3991; 66.981; -18.3952; 66.982; -18.3914; 66.983; -18.3877; 66.984; -18.3841; 66.985; -18.3805; 66.986; -18.3769; 66.987; -18.3735; 66.988; -18.37; 66.989; -18.3666; 66.99; -18.3633; 66.991; -18.36; 66.992; -18.3567; 66.993; -18.3536; 66.994; -18.3504; 66.995; -18.3474; 66.996; -18.3443; 66.997; -18.3413; 66.998; -18.3384; 66.999; -18.3355; 67; -18.3327; 67.001; -18.3298; 67.002; -18.3271; 67.003; -18.3243; 67.004; -18.3216; 67.005; -18.3189; 67.006; -18.3162; 67.007; -18.3136; 67.008; -18.3111; 67.009; -18.3085; 67.01; -18.306; 67.011; -18.3035; 67.012; -18.3011; 67.013; -18.2987; 67.014; -18.2963; 67.015; -18.294; 67.016; -18.2917; 67.017; -18.2894; 67.018; -18.2871; 67.019; -18.2849; 67.02; -18.2827; 67.021; -18.2806; 67.022; -18.2784; 67.023; -18.2763; 67.024; -18.2743; 67.025; -18.2722; 67.026; -18.2702; 67.027; -18.2682; 67.028; -18.2662; 67.029; -18.2643; 67.03; -18.2623; 67.031; -18.2604; 67.032; -18.2586; 67.033; -18.2567; 67.034; -18.2549; 67.035; -18.2531; 67.036; -18.2513; 67.037; -18.2496; 67.038; -18.2478; 67.039; -18.2461; 67.04; -18.2444; 67.041; -18.2427; 67.042; -18.2411; 67.043; -18.2395; 67.044; -18.2379; 67.045; -18.2363; 67.046; -18.2347; 67.047; -18.2332; 67.048; -18.2317; 67.049; -18.2302; 67.05; -18.2287; 67.051; -18.2272; 67.052; -18.2258; 67.053; -18.2243; 67.054; -18.2229; 67.055; -18.2215; 67.056; -18.2202; 67.057; -18.2188; 67.058; -18.2175; 67.059; -18.2162; 67.06; -18.2149; 67.061; -18.2124; 67.063; -18.2099; 67.065; -18.2075; 67.067; -18.2052; 67.069; -18.2029; 67.071; -18.2007; 67.073; -18.1986; 67.075; -18.1965; 67.077; -18.1945; 67.079; -18.1925; 67.081; -18.1907; 67.083; -18.1889; 67.085; -18.1871; 67.087; -18.1854; 67.089; -18.1838; 67.091; -18.1822; 67.093; -18.1807; 67.095; -18.1792; 67.097; -18.1778; 67.099; -18.1764; 67.101; -18.1751; 67.103; -18.1739; 67.105; -18.1727; 67.107; -18.1716; 67.109; -18.1705; 67.111; -18.1695; 67.113; -18.1686; 67.115; -18.1676; 67.117; -18.1668; 67.119; -18.166; 67.121; -18.1652; 67.123; -18.1645; 67.125; -18.1639; 67.127; -18.1633; 67.129; -18.1628; 67.131; -18.1623; 67.133; -18.1618; 67.135; -18.1615; 67.137; -18.1611; 67.139; -18.1609; 67.141; -18.1606; 67.143; -18.1605; 67.145; -18.1603; 67.147; -18.1603; 67.149; -18.1602; 67.151; -18.1603; 67.153; -18.1603; 67.155; -18.1605; 67.157; -18.1607; 67.159; -18.1609; 67.161; -18.1612; 67.163; -18.1615; 67.165; -18.1619; 67.167; -18.1624; 67.169; -18.1629; 67.171; -18.1634; 67.173; -18.164; 67.175; -18.1647; 67.177; -18.1654; 67.179; -18.1661; 67.181; -18.167; 67.183; -18.1678; 67.185; -18.1687; 67.187; -18.1697; 67.189; -18.1707; 67.191; -18.1718; 67.193; -18.173; 67.195; -18.1742; 67.197; -18.1754; 67.199; -18.1766; 67.201; -18.1779; 67.203; -18.1793; 67.205; -18.1807; 67.207; -18.1822; 67.209; -18.1837; 67.211; -18.1853; 67.213; -18.187; 67.215; -18.1887; 67.217; -18.1905; 67.219; -18.1923; 67.221; -18.1943; 67.223; -18.1962; 67.225; -18.1983; 67.227; -18.2004; 67.229; -18.2025; 67.231; -18.2048; 67.233; -18.2071; 67.235; -18.2094; 67.237; -18.2119; 67.239; -18.2144; 67.241; -18.2157; 67.242; -18.217; 67.243; -18.2183; 67.244; -18.2196; 67.245; -18.221; 67.246; -18.2223; 67.247; -18.2237; 67.248; -18.2251; 67.249; -18.2266; 67.25; -18.228; 67.251; -18.2295; 67.252; -18.231; 67.253; -18.2325; 67.254; -18.234; 67.255; -18.2356; 67.256; -18.2371; 67.257; -18.2387; 67.258; -18.2404; 67.259; -18.242; 67.26; -18.2436; 67.261; -18.2453; 67.262; -18.247; 67.263; -18.2488; 67.264; -18.2505; 67.265; -18.2523; 67.266; -18.2541; 67.267; -18.2559; 67.268; -18.2577; 67.269; -18.2596; 67.27; -18.2615; 67.271; -18.2634; 67.272; -18.2653; 67.273; -18.2673; 67.274; -18.2693; 67.275; -18.2713; 67.276; -18.2734; 67.277; -18.2754; 67.278; -18.2775; 67.279; -18.2797; 67.28; -18.2818; 67.281; -18.284; 67.282; -18.2862; 67.283; -18.2885; 67.284; -18.2907; 67.285; -18.293; 67.286; -18.2954; 67.287; -18.2978; 67.288; -18.3002; 67.289; -18.3026; 67.29; -18.3051; 67.291; -18.3076; 67.292; -18.3101; 67.293; -18.3127; 67.294; -18.3153; 67.295; -18.318; 67.296; -18.3206; 67.297; -18.3234; 67.298; -18.3262; 67.299; -18.329; 67.3; -18.3318; 67.301; -18.3347; 67.302; -18.3377; 67.303; -18.3407; 67.304; -18.3437; 67.305; -18.3468; 67.306; -18.3499; 67.307; -18.3531; 67.308; -18.3563; 67.309; -18.3595; 67.31; -18.3628; 67.311; -18.3662; 67.312; -18.3696; 67.313; -18.373; 67.314; -18.3766; 67.315; -18.3802; 67.316; -18.3838; 67.317; -18.3876; 67.318; -18.3914; 67.319; -18.3952; 67.32; -18.3992; 67.321; -18.4032; 67.322; -18.4073; 67.323; -18.4116; 67.324; -18.4159; 67.325; -18.4203; 67.326; -18.4248; 67.327; -18.4294; 67.328; -18.4341; 67.329; -18.4389; 67.33; -18.4439; 67.331; -18.449; 67.332; -18.4543; 67.333; -18.4597; 67.334; -18.4653; 67.335; -18.471; 67.336; -18.477; 67.337; -18.4831; 67.338; -18.4896; 67.339; -18.4962; 67.34; -18.5032; 67.341; -18.5105; 67.342; -18.5181; 67.343; -18.5262; 67.344; -18.5348; 67.345; -18.5439; 67.346; -18.5538; 67.347; -18.5646; 67.348; -18.5766; 67.349; -18.5902; 67.35; -18.6065; 67.351; -18.6277; 67.352; -18.6732; 67.353; -18.6879; 67.353; -18.7334; 67.352; -18.7546; 67.351; -18.7708; 67.35; -18.7845; 67.349; -18.7964; 67.348; -18.8072; 67.347; -18.8171; 67.346; -18.8263; 67.345; -18.8348; 67.344; -18.8429; 67.343; -18.8506; 67.342; -18.8579; 67.341; -18.8648; 67.34; -18.8715; 67.339; -18.8779; 67.338; -18.8841; 67.337; -18.89; 67.336; -18.8958; 67.335; -18.9014; 67.334; -18.9068; 67.333; -18.912; 67.332; -18.9171; 67.331; -18.9221; 67.33; -18.927; 67.329; -18.9317; 67.328; -18.9363; 67.327; -18.9408; 67.326; -18.9452; 67.325; -18.9495; 67.324; -18.9537; 67.323; -18.9578; 67.322; -18.9619; 67.321; -18.9658; 67.32; -18.9697; 67.319; -18.9735; 67.318; -18.9772; 67.317; -18.9809; 67.316; -18.9845; 67.315; -18.988; 67.314; -18.9915; 67.313; -18.9949; 67.312; -18.9982; 67.311; -19.0015; 67.31; -19.0048; 67.309; -19.008; 67.308; -19.0111; 67.307; -19.0142; 67.306; -19.0172; 67.305; -19.0202; 67.304; -19.0232; 67.303; -19.0261; 67.302; -19.0289; 67.301; -19.0317; 67.3; -19.0345; 67.299; -19.0372; 67.298; -19.0399; 67.297; -19.0426; 67.296; -19.0452; 67.295; -19.0478; 67.294; -19.0503; 67.293; -19.0528; 67.292; -19.0553; 67.291; -19.0577; 67.29; -19.0601; 67.289; -19.0625; 67.288; -19.0648; 67.287; -19.0671; 67.286; -19.0694; 67.285; -19.0717; 67.284; -19.0739; 67.283; -19.0761; 67.282; -19.0782; 67.281; -19.0803; 67.28; -19.0824; 67.279; -19.0845; 67.278; -19.0866; 67.277; -19.0886; 67.276; -19.0906; 67.275; -19.0925; 67.274; -19.0945; 67.273; -19.0964; 67.272; -19.0983; 67.271; -19.1002; 67.27; -19.102; 67.269; -19.1038; 67.268; -19.1056; 67.267; -19.1074; 67.266; -19.1091; 67.265; -19.1108; 67.264; -19.1125; 67.263; -19.1142; 67.262; -19.1159; 67.261; -19.1175; 67.26; -19.1191; 67.259; -19.1207; 67.258; -19.1223; 67.257; -19.1239; 67.256; -19.1254; 67.255; -19.1269; 67.254; -19.1284; 67.253; -19.1299; 67.252; -19.1314; 67.251; -19.1329; 67.25; -19.1343; 67.249; -19.1357; 67.248; -19.1372; 67.247; -19.1385; 67.246; -19.1399; 67.245; -19.1413; 67.244; -19.1426; 67.243; -19.1439; 67.242; -19.1452; 67.241; -19.1478; 67.239; -19.1502; 67.237; -19.1526; 67.235; -19.155; 67.233; -19.1572; 67.231; -19.1594; 67.229; -19.1616; 67.227; -19.1636; 67.225; -19.1656; 67.223; -19.1676; 67.221; -19.1695; 67.219; -19.1713; 67.217; -19.173; 67.215; -19.1747; 67.213; -19.1763; 67.211; -19.1779; 67.209; -19.1794; 67.207; -19.1809; 67.205; -19.1823; 67.203; -19.1836; 67.201; -19.1849; 67.199; -19.1861; 67.197; -19.1873; 67.195; -19.1884; 67.193; -19.1895; 67.191; -19.1905; 67.189; -19.1914; 67.187; -19.1923; 67.185; -19.1932; 67.183; -19.1939; 67.181; -19.1947; 67.179; -19.1954; 67.177; -19.196; 67.175; -19.1966; 67.173; -19.1971; 67.171; -19.1976; 67.169; -19.198; 67.167; -19.1983; 67.165; -19.1987; 67.163; -19.1989; 67.161; -19.1991; 67.159; -19.1993; 67.157; -19.1994; 67.155; -19.1995; 67.153; -19.1995; 67.151</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Forest</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -2642,38 +2520,48 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q18">
         <v>1</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>bb15055d-5902-4cdc-858b-0e19fb32777f</t>
+          <t>f255dc8a-e048-49cc-aad5-20bbdf70f5b4</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>study_site_1</t>
         </is>
       </c>
       <c r="C19">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Population-level effects of light pollution on nocturnal insect communities</t>
+          <t>Seed dispersal limitation constrains plant community recovery after tropical forest fragmentation</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Thompson LD; O'Brien KA; Mwangi PK</t>
+          <t>Almeida FS; Ribeiro GH; Neves CT</t>
         </is>
       </c>
       <c r="F19">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>10.1098/rsbl.2019.0367</t>
+          <t>10.1111/gcb.16157</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2688,22 +2576,22 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-02-28T09:27:29+00:00</t>
+          <t>2026-02-28T09:28:47+00:00</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
+          <t>Iceland; 64.9842; -18.1059; 299133; MultiPolygon; -25.0135; 65.5045; -25.0079; 65.4708; -24.9887; 65.4379; -24.4824; 64.7928; -23.7161; 63.6161; -23.6902; 63.5848; -23.6531; 63.5559; -23.6058; 63.5302; -23.5496; 63.5083; -23.4861; 63.4908; -23.4171; 63.4783; -23.3444; 63.4711; -23.2701; 63.4693; -23.1961; 63.473; -23.1245; 63.4822; -22.9863; 63.5055; -22.5; 63.4173; -20.774; 63.1019; -20.6951; 63.0905; -20.613; 63.0859; -20.5304; 63.0884; -19.0873; 63.1853; -18.7041; 63.185; -18.6405; 63.187; -18.5781; 63.193; -18.0646; 63.2592; -17.9667; 63.2776; -17.7678; 63.3278; -17.7098; 63.3452; -17.6585; 63.3664; -17.591; 63.399; -17.3177; 63.5463; -16.5809; 63.5876; -16.5117; 63.5937; -16.4455; 63.6046; -16.384; 63.62; -15.9349; 63.7523; -15.8562; 63.7813; -15.6952; 63.8557; -14.77; 64.0538; -14.705; 64.0704; -14.2054; 64.2218; -14.143; 64.2442; -13.793; 64.3932; -13.671; 64.4519; -13.6426; 64.469; -13.6153; 64.4534; -13.5739; 64.4357; -13.5109; 64.4157; -13.4897; 64.4104; -13.441; 64.4005; -13.416; 64.3965; -13.3664; 64.3907; -13.3379; 64.3884; -13.2862; 64.3863; -13.2578; 64.3862; -13.2054; 64.388; -13.178; 64.39; -13.1266; 64.3958; -13.1008; 64.3997; -13.052; 64.4094; -13.0287; 64.4151; -12.984; 64.4283; -12.9637; 64.4355; -12.9246; 64.4521; -12.8775; 64.4788; -12.8628; 64.4894; -12.8412; 64.5085; -12.83; 64.5211; -12.817; 64.5404; -12.8104; 64.5548; -12.8055; 64.5736; -12.8046; 64.5895; -12.8071; 64.6071; -12.813; 64.6241; -12.8218; 64.6401; -12.8352; 64.6575; -12.8492; 64.6715; -12.8708; 64.6887; -12.8886; 64.7005; -12.9185; 64.7169; -12.939; 64.7263; -12.9771; 64.741; -13.0446; 64.7604; -13.1191; 64.7744; -13.1983; 64.7827; -13.2196; 64.7833; -13.2053; 64.7938; -13.1328; 64.838; -13.0828; 64.8768; -13.0662; 64.894; -13.0437; 64.9236; -13.0322; 64.9544; -13.0138; 65.0538; -13.0134; 65.0826; -13.031; 65.1902; -13.1236; 65.5252; -13.1359; 65.5523; -13.1572; 65.5785; -14.063; 66.4484; -14.1044; 66.479; -14.1587; 66.5063; -14.2241; 66.5294; -14.2987; 66.5475; -14.3802; 66.5601; -15.8898; 66.7267; -16.0151; 66.7333; -16.184; 66.7335; -16.2977; 66.7285; -16.6492; 66.696; -16.7327; 66.685; -16.8101; 66.6684; -16.8788; 66.6467; -17.3761; 66.4565; -17.5468; 66.4292; -17.5259; 66.444; -17.4973; 66.4761; -17.4827; 66.5096; -17.4808; 66.5592; -17.4956; 66.5912; -17.5189; 66.6195; -17.55; 66.6444; -17.5809; 66.665; -17.6304; 66.6926; -17.6864; 66.7154; -17.7304; 66.7291; -17.8096; 66.7473; -17.8959; 66.7595; -17.9863; 66.7653; -18.078; 66.7644; -18.1677; 66.757; -18.2524; 66.7432; -18.3296; 66.7237; -18.3952; 66.6995; -18.4487; 66.671; -18.4886; 66.6393; -18.5136; 66.6052; -18.5187; 66.5857; -18.525; 66.574; -18.5279; 66.5383; -18.5147; 66.5029; -18.5008; 66.4866; -18.4924; 66.4728; -18.4581; 66.4423; -18.4136; 66.4155; -18.3591; 66.3919; -18.3171; 66.3769; -18.8; 66.3851; -18.8604; 66.3845; -20.1192; 66.3368; -22.1606; 66.6292; -22.2041; 66.6386; -22.2962; 66.6543; -22.3748; 66.6626; -22.4558; 66.6656; -22.5; 66.6642; -22.5442; 66.6629; -22.5969; 66.657; -22.878; 66.6662; -22.977; 66.6655; -23.0737; 66.657; -23.1641; 66.6411; -23.3815; 66.5918; -23.4683; 66.5668; -23.5396; 66.5349; -24.1866; 66.1666; -24.2216; 66.1429; -24.5265; 65.8973; -24.9484; 65.6014; -24.9834; 65.5708; -25.0053; 65.5382; -25.0135; 65.5045; -19.1995; 67.151; -19.1994; 67.149; -19.1993; 67.147; -19.1992; 67.145; -19.199; 67.143; -19.1987; 67.141; -19.1984; 67.139; -19.198; 67.137; -19.1976; 67.135; -19.1972; 67.133; -19.1967; 67.131; -19.1961; 67.129; -19.1955; 67.127; -19.1948; 67.125; -19.1941; 67.123; -19.1933; 67.121; -19.1925; 67.119; -19.1916; 67.117; -19.1907; 67.115; -19.1897; 67.113; -19.1886; 67.111; -19.1875; 67.109; -19.1864; 67.107; -19.1852; 67.105; -19.1839; 67.103; -19.1826; 67.101; -19.1812; 67.099; -19.1798; 67.097; -19.1784; 67.095; -19.177; 67.093; -19.1755; 67.091; -19.1739; 67.089; -19.1722; 67.087; -19.1705; 67.085; -19.1688; 67.083; -19.167; 67.081; -19.1651; 67.079; -19.1631; 67.077; -19.1611; 67.075; -19.1591; 67.073; -19.1569; 67.071; -19.1547; 67.069; -19.1525; 67.067; -19.1502; 67.065; -19.1478; 67.063; -19.1453; 67.061; -19.1428; 67.059; -19.1415; 67.058; -19.1401; 67.057; -19.1388; 67.056; -19.1375; 67.055; -19.1361; 67.054; -19.1347; 67.053; -19.1333; 67.052; -19.1319; 67.051; -19.1304; 67.05; -19.129; 67.049; -19.1275; 67.048; -19.126; 67.047; -19.1245; 67.046; -19.1229; 67.045; -19.1214; 67.044; -19.1198; 67.043; -19.1182; 67.042; -19.1165; 67.041; -19.1149; 67.04; -19.1132; 67.039; -19.1115; 67.038; -19.1098; 67.037; -19.1081; 67.036; -19.1063; 67.035; -19.1046; 67.034; -19.1028; 67.033; -19.1009; 67.032; -19.0991; 67.031; -19.0972; 67.03; -19.0953; 67.029; -19.0934; 67.028; -19.0914; 67.027; -19.0895; 67.026; -19.0875; 67.025; -19.0854; 67.024; -19.0834; 67.023; -19.0813; 67.022; -19.0792; 67.021; -19.0771; 67.02; -19.0749; 67.019; -19.0727; 67.018; -19.0705; 67.017; -19.0683; 67.016; -19.066; 67.015; -19.0637; 67.014; -19.0613; 67.013; -19.059; 67.012; -19.0566; 67.011; -19.0541; 67.01; -19.0516; 67.009; -19.0491; 67.008; -19.0466; 67.007; -19.044; 67.006; -19.0414; 67.005; -19.0388; 67.004; -19.0361; 67.003; -19.0333; 67.002; -19.0306; 67.001; -19.0278; 67; -19.0249; 66.999; -19.022; 66.998; -19.0191; 66.997; -19.0161; 66.996; -19.013; 66.995; -19.01; 66.994; -19.0068; 66.993; -19.0037; 66.992; -19.0004; 66.991; -18.9971; 66.99; -18.9938; 66.989; -18.9904; 66.988; -18.9869; 66.987; -18.9834; 66.986; -18.9798; 66.985; -18.9762; 66.984; -18.9725; 66.983; -18.9687; 66.982; -18.9648; 66.981; -18.9609; 66.98; -18.9569; 66.979; -18.9528; 66.978; -18.9486; 66.977; -18.9443; 66.976; -18.9399; 66.975; -18.9355; 66.974; -18.9309; 66.973; -18.9262; 66.972; -18.9213; 66.971; -18.9164; 66.97; -18.9113; 66.969; -18.9061; 66.968; -18.9007; 66.967; -18.8952; 66.966; -18.8895; 66.965; -18.8835; 66.964; -18.8774; 66.963; -18.871; 66.962; -18.8644; 66.961; -18.8575; 66.96; -18.8503; 66.959; -18.8427; 66.958; -18.8346; 66.957; -18.8261; 66.956; -18.817; 66.955; -18.8072; 66.954; -18.7965; 66.953; -18.7846; 66.952; -18.7711; 66.951; -18.755; 66.95; -18.734; 66.949; -18.6888; 66.948; -18.6751; 66.948; -18.6299; 66.949; -18.6089; 66.95; -18.5928; 66.951; -18.5793; 66.952; -18.5674; 66.953; -18.5567; 66.954; -18.5469; 66.955; -18.5378; 66.956; -18.5293; 66.957; -18.5212; 66.958; -18.5136; 66.959; -18.5064; 66.96; -18.4995; 66.961; -18.4929; 66.962; -18.4865; 66.963; -18.4804; 66.964; -18.4744; 66.965; -18.4687; 66.966; -18.4632; 66.967; -18.4578; 66.968; -18.4526; 66.969; -18.4475; 66.97; -18.4425; 66.971; -18.4377; 66.972; -18.433; 66.973; -18.4284; 66.974; -18.424; 66.975; -18.4196; 66.976; -18.4153; 66.977; -18.4111; 66.978; -18.407; 66.979; -18.403; 66.98; -18.3991; 66.981; -18.3952; 66.982; -18.3914; 66.983; -18.3877; 66.984; -18.3841; 66.985; -18.3805; 66.986; -18.3769; 66.987; -18.3735; 66.988; -18.37; 66.989; -18.3666; 66.99; -18.3633; 66.991; -18.36; 66.992; -18.3567; 66.993; -18.3536; 66.994; -18.3504; 66.995; -18.3474; 66.996; -18.3443; 66.997; -18.3413; 66.998; -18.3384; 66.999; -18.3355; 67; -18.3327; 67.001; -18.3298; 67.002; -18.3271; 67.003; -18.3243; 67.004; -18.3216; 67.005; -18.3189; 67.006; -18.3162; 67.007; -18.3136; 67.008; -18.3111; 67.009; -18.3085; 67.01; -18.306; 67.011; -18.3035; 67.012; -18.3011; 67.013; -18.2987; 67.014; -18.2963; 67.015; -18.294; 67.016; -18.2917; 67.017; -18.2894; 67.018; -18.2871; 67.019; -18.2849; 67.02; -18.2827; 67.021; -18.2806; 67.022; -18.2784; 67.023; -18.2763; 67.024; -18.2743; 67.025; -18.2722; 67.026; -18.2702; 67.027; -18.2682; 67.028; -18.2662; 67.029; -18.2643; 67.03; -18.2623; 67.031; -18.2604; 67.032; -18.2586; 67.033; -18.2567; 67.034; -18.2549; 67.035; -18.2531; 67.036; -18.2513; 67.037; -18.2496; 67.038; -18.2478; 67.039; -18.2461; 67.04; -18.2444; 67.041; -18.2427; 67.042; -18.2411; 67.043; -18.2395; 67.044; -18.2379; 67.045; -18.2363; 67.046; -18.2347; 67.047; -18.2332; 67.048; -18.2317; 67.049; -18.2302; 67.05; -18.2287; 67.051; -18.2272; 67.052; -18.2258; 67.053; -18.2243; 67.054; -18.2229; 67.055; -18.2215; 67.056; -18.2202; 67.057; -18.2188; 67.058; -18.2175; 67.059; -18.2162; 67.06; -18.2149; 67.061; -18.2124; 67.063; -18.2099; 67.065; -18.2075; 67.067; -18.2052; 67.069; -18.2029; 67.071; -18.2007; 67.073; -18.1986; 67.075; -18.1965; 67.077; -18.1945; 67.079; -18.1925; 67.081; -18.1907; 67.083; -18.1889; 67.085; -18.1871; 67.087; -18.1854; 67.089; -18.1838; 67.091; -18.1822; 67.093; -18.1807; 67.095; -18.1792; 67.097; -18.1778; 67.099; -18.1764; 67.101; -18.1751; 67.103; -18.1739; 67.105; -18.1727; 67.107; -18.1716; 67.109; -18.1705; 67.111; -18.1695; 67.113; -18.1686; 67.115; -18.1676; 67.117; -18.1668; 67.119; -18.166; 67.121; -18.1652; 67.123; -18.1645; 67.125; -18.1639; 67.127; -18.1633; 67.129; -18.1628; 67.131; -18.1623; 67.133; -18.1618; 67.135; -18.1615; 67.137; -18.1611; 67.139; -18.1609; 67.141; -18.1606; 67.143; -18.1605; 67.145; -18.1603; 67.147; -18.1603; 67.149; -18.1602; 67.151; -18.1603; 67.153; -18.1603; 67.155; -18.1605; 67.157; -18.1607; 67.159; -18.1609; 67.161; -18.1612; 67.163; -18.1615; 67.165; -18.1619; 67.167; -18.1624; 67.169; -18.1629; 67.171; -18.1634; 67.173; -18.164; 67.175; -18.1647; 67.177; -18.1654; 67.179; -18.1661; 67.181; -18.167; 67.183; -18.1678; 67.185; -18.1687; 67.187; -18.1697; 67.189; -18.1707; 67.191; -18.1718; 67.193; -18.173; 67.195; -18.1742; 67.197; -18.1754; 67.199; -18.1766; 67.201; -18.1779; 67.203; -18.1793; 67.205; -18.1807; 67.207; -18.1822; 67.209; -18.1837; 67.211; -18.1853; 67.213; -18.187; 67.215; -18.1887; 67.217; -18.1905; 67.219; -18.1923; 67.221; -18.1943; 67.223; -18.1962; 67.225; -18.1983; 67.227; -18.2004; 67.229; -18.2025; 67.231; -18.2048; 67.233; -18.2071; 67.235; -18.2094; 67.237; -18.2119; 67.239; -18.2144; 67.241; -18.2157; 67.242; -18.217; 67.243; -18.2183; 67.244; -18.2196; 67.245; -18.221; 67.246; -18.2223; 67.247; -18.2237; 67.248; -18.2251; 67.249; -18.2266; 67.25; -18.228; 67.251; -18.2295; 67.252; -18.231; 67.253; -18.2325; 67.254; -18.234; 67.255; -18.2356; 67.256; -18.2371; 67.257; -18.2387; 67.258; -18.2404; 67.259; -18.242; 67.26; -18.2436; 67.261; -18.2453; 67.262; -18.247; 67.263; -18.2488; 67.264; -18.2505; 67.265; -18.2523; 67.266; -18.2541; 67.267; -18.2559; 67.268; -18.2577; 67.269; -18.2596; 67.27; -18.2615; 67.271; -18.2634; 67.272; -18.2653; 67.273; -18.2673; 67.274; -18.2693; 67.275; -18.2713; 67.276; -18.2734; 67.277; -18.2754; 67.278; -18.2775; 67.279; -18.2797; 67.28; -18.2818; 67.281; -18.284; 67.282; -18.2862; 67.283; -18.2885; 67.284; -18.2907; 67.285; -18.293; 67.286; -18.2954; 67.287; -18.2978; 67.288; -18.3002; 67.289; -18.3026; 67.29; -18.3051; 67.291; -18.3076; 67.292; -18.3101; 67.293; -18.3127; 67.294; -18.3153; 67.295; -18.318; 67.296; -18.3206; 67.297; -18.3234; 67.298; -18.3262; 67.299; -18.329; 67.3; -18.3318; 67.301; -18.3347; 67.302; -18.3377; 67.303; -18.3407; 67.304; -18.3437; 67.305; -18.3468; 67.306; -18.3499; 67.307; -18.3531; 67.308; -18.3563; 67.309; -18.3595; 67.31; -18.3628; 67.311; -18.3662; 67.312; -18.3696; 67.313; -18.373; 67.314; -18.3766; 67.315; -18.3802; 67.316; -18.3838; 67.317; -18.3876; 67.318; -18.3914; 67.319; -18.3952; 67.32; -18.3992; 67.321; -18.4032; 67.322; -18.4073; 67.323; -18.4116; 67.324; -18.4159; 67.325; -18.4203; 67.326; -18.4248; 67.327; -18.4294; 67.328; -18.4341; 67.329; -18.4389; 67.33; -18.4439; 67.331; -18.449; 67.332; -18.4543; 67.333; -18.4597; 67.334; -18.4653; 67.335; -18.471; 67.336; -18.477; 67.337; -18.4831; 67.338; -18.4896; 67.339; -18.4962; 67.34; -18.5032; 67.341; -18.5105; 67.342; -18.5181; 67.343; -18.5262; 67.344; -18.5348; 67.345; -18.5439; 67.346; -18.5538; 67.347; -18.5646; 67.348; -18.5766; 67.349; -18.5902; 67.35; -18.6065; 67.351; -18.6277; 67.352; -18.6732; 67.353; -18.6879; 67.353; -18.7334; 67.352; -18.7546; 67.351; -18.7708; 67.35; -18.7845; 67.349; -18.7964; 67.348; -18.8072; 67.347; -18.8171; 67.346; -18.8263; 67.345; -18.8348; 67.344; -18.8429; 67.343; -18.8506; 67.342; -18.8579; 67.341; -18.8648; 67.34; -18.8715; 67.339; -18.8779; 67.338; -18.8841; 67.337; -18.89; 67.336; -18.8958; 67.335; -18.9014; 67.334; -18.9068; 67.333; -18.912; 67.332; -18.9171; 67.331; -18.9221; 67.33; -18.927; 67.329; -18.9317; 67.328; -18.9363; 67.327; -18.9408; 67.326; -18.9452; 67.325; -18.9495; 67.324; -18.9537; 67.323; -18.9578; 67.322; -18.9619; 67.321; -18.9658; 67.32; -18.9697; 67.319; -18.9735; 67.318; -18.9772; 67.317; -18.9809; 67.316; -18.9845; 67.315; -18.988; 67.314; -18.9915; 67.313; -18.9949; 67.312; -18.9982; 67.311; -19.0015; 67.31; -19.0048; 67.309; -19.008; 67.308; -19.0111; 67.307; -19.0142; 67.306; -19.0172; 67.305; -19.0202; 67.304; -19.0232; 67.303; -19.0261; 67.302; -19.0289; 67.301; -19.0317; 67.3; -19.0345; 67.299; -19.0372; 67.298; -19.0399; 67.297; -19.0426; 67.296; -19.0452; 67.295; -19.0478; 67.294; -19.0503; 67.293; -19.0528; 67.292; -19.0553; 67.291; -19.0577; 67.29; -19.0601; 67.289; -19.0625; 67.288; -19.0648; 67.287; -19.0671; 67.286; -19.0694; 67.285; -19.0717; 67.284; -19.0739; 67.283; -19.0761; 67.282; -19.0782; 67.281; -19.0803; 67.28; -19.0824; 67.279; -19.0845; 67.278; -19.0866; 67.277; -19.0886; 67.276; -19.0906; 67.275; -19.0925; 67.274; -19.0945; 67.273; -19.0964; 67.272; -19.0983; 67.271; -19.1002; 67.27; -19.102; 67.269; -19.1038; 67.268; -19.1056; 67.267; -19.1074; 67.266; -19.1091; 67.265; -19.1108; 67.264; -19.1125; 67.263; -19.1142; 67.262; -19.1159; 67.261; -19.1175; 67.26; -19.1191; 67.259; -19.1207; 67.258; -19.1223; 67.257; -19.1239; 67.256; -19.1254; 67.255; -19.1269; 67.254; -19.1284; 67.253; -19.1299; 67.252; -19.1314; 67.251; -19.1329; 67.25; -19.1343; 67.249; -19.1357; 67.248; -19.1372; 67.247; -19.1385; 67.246; -19.1399; 67.245; -19.1413; 67.244; -19.1426; 67.243; -19.1439; 67.242; -19.1452; 67.241; -19.1478; 67.239; -19.1502; 67.237; -19.1526; 67.235; -19.155; 67.233; -19.1572; 67.231; -19.1594; 67.229; -19.1616; 67.227; -19.1636; 67.225; -19.1656; 67.223; -19.1676; 67.221; -19.1695; 67.219; -19.1713; 67.217; -19.173; 67.215; -19.1747; 67.213; -19.1763; 67.211; -19.1779; 67.209; -19.1794; 67.207; -19.1809; 67.205; -19.1823; 67.203; -19.1836; 67.201; -19.1849; 67.199; -19.1861; 67.197; -19.1873; 67.195; -19.1884; 67.193; -19.1895; 67.191; -19.1905; 67.189; -19.1914; 67.187; -19.1923; 67.185; -19.1932; 67.183; -19.1939; 67.181; -19.1947; 67.179; -19.1954; 67.177; -19.196; 67.175; -19.1966; 67.173; -19.1971; 67.171; -19.1976; 67.169; -19.198; 67.167; -19.1983; 67.165; -19.1987; 67.163; -19.1989; 67.161; -19.1991; 67.159; -19.1993; 67.157; -19.1994; 67.155; -19.1995; 67.153; -19.1995; 67.151</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Forest</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -2713,7 +2601,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>simple_group</t>
+          <t>study_site</t>
         </is>
       </c>
       <c r="Q19">
@@ -2723,33 +2611,28 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>bb15055d-5902-4cdc-858b-0e19fb32777f</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
+          <t>96dc0855-1faa-4b76-b276-825d9bc6a8fe</t>
         </is>
       </c>
       <c r="C20">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Population-level effects of light pollution on nocturnal insect communities</t>
+          <t>Range shifts of montane mammals under projected warming in the Andes</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Thompson LD; O'Brien KA; Mwangi PK</t>
+          <t>Gutierrez MJ; Blanco VF; Quispe RR</t>
         </is>
       </c>
       <c r="F20">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10.1098/rsbl.2019.0367</t>
+          <t>10.1111/geb.13094</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2764,22 +2647,22 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-02-28T09:27:29+00:00</t>
+          <t>2026-02-28T09:29:11+00:00</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>City of Edinburgh, Scotland, United Kingdom; 55.9533; -3.1884; 1920901</t>
+          <t>Honolulu County, Hawaii, United States; 21.4682; -157.9605; 3861844; MultiPolygon; -178.4436; 28.419; -178.4405; 28.4052; -178.4332; 28.3978; -178.4159; 28.3801; -178.4137; 28.375; -178.4141; 28.375; -178.4153; 28.375; -178.4157; 28.375; -178.4123; 28.3633; -178.4115; 28.3607; -178.3956; 28.3419; -178.3867; 28.3391; -178.375; 28.3354; -178.375; 28.3358; -178.375; 28.3371; -178.375; 28.3375; -178.3489; 28.3347; -178.3417; 28.3339; -178.3014; 28.3283; -178.2889; 28.3288; -178.2719; 28.3353; -178.2703; 28.3359; -178.2575; 28.3428; -178.25; 28.3494; -178.25; 28.349; -178.25; 28.3476; -178.25; 28.3472; -178.2461; 28.3524; -178.2389; 28.362; -178.2357; 28.369; -178.233; 28.375; -178.2338; 28.375; -178.2363; 28.375; -178.2371; 28.375; -178.2325; 28.3836; -178.2311; 28.3937; -178.2305; 28.3977; -178.2322; 28.4273; -178.2378; 28.4529; -178.2385; 28.4562; -178.25; 28.4682; -178.25; 28.4679; -178.25; 28.467; -178.25; 28.4667; -178.256; 28.4751; -178.257; 28.4765; -178.2712; 28.4886; -178.2801; 28.4944; -178.2888; 28.5; -178.2873; 28.5; -178.2826; 28.5; -178.2811; 28.5; -178.2915; 28.5072; -178.2979; 28.5102; -178.3043; 28.5133; -178.3151; 28.5163; -178.3337; 28.5172; -178.3405; 28.5173; -178.3558; 28.5146; -178.3606; 28.5138; -178.375; 28.5101; -178.375; 28.5096; -178.375; 28.5083; -178.375; 28.5078; -178.3773; 28.5063; -178.3813; 28.5036; -178.3842; 28.5016; -178.3864; 28.5; -178.3883; 28.5; -178.3939; 28.5; -178.3958; 28.5; -178.4118; 28.4837; -178.4168; 28.4782; -178.4276; 28.4661; -178.4383; 28.4441; -178.4436; 28.419; -176.0434; 27.7959; -176.0429; 27.7784; -176.0396; 27.7582; -176.0344; 27.75; -176.0293; 27.7427; -176.0249; 27.738; -176.0235; 27.7367; -176.0055; 27.7203; -176; 27.7161; -176; 27.7147; -176; 27.7107; -176; 27.7093; -175.9763; 27.6969; -175.9696; 27.6934; -175.9395; 27.6882; -175.8988; 27.6983; -175.8952; 27.6992; -175.875; 27.7102; -175.875; 27.7098; -175.875; 27.7088; -175.875; 27.7084; -175.8649; 27.7145; -175.845; 27.7285; -175.8175; 27.723; -175.8029; 27.7235; -175.7791; 27.7257; -175.75; 27.7333; -175.75; 27.7323; -175.7461; 27.7327; -175.7341; 27.7389; -175.7262; 27.75; -175.7248; 27.7526; -175.6784; 27.8432; -175.6766; 27.8468; -175.6665; 27.875; -175.6663; 27.875; -175.6658; 27.875; -175.6656; 27.875; -175.6641; 27.8941; -175.6645; 27.9061; -175.6648; 27.9144; -175.6701; 27.9416; -175.6815; 27.9586; -175.7044; 27.9827; -175.7078; 27.9847; -175.7349; 28; -175.736; 28; -175.739; 28; -175.74; 28; -175.7411; 28.0003; -175.7444; 28.001; -175.7445; 28.001; -175.7455; 28.0013; -175.7457; 28.0014; -175.7463; 28.0016; -175.7466; 28.0016; -175.75; 28.003; -175.7544; 28.004; -175.7697; 28.0075; -175.7786; 28.0081; -175.7863; 28.0086; -175.7868; 28.0086; -175.7999; 28.0082; -175.806; 28.0073; -175.8067; 28.0072; -175.8101; 28.0059; -175.8174; 28.0022; -175.8231; 28; -175.8579; 27.9821; -175.875; 27.9733; -175.875; 27.9738; -175.875; 27.9754; -175.875; 27.9759; -175.9044; 27.9606; -175.9088; 27.9583; -175.9357; 27.9406; -175.9505; 27.9362; -175.9663; 27.9299; -175.9814; 27.9132; -175.9847; 27.9065; -175.9876; 27.9005; -175.9921; 27.8895; -175.9938; 27.875; -175.9931; 27.875; -175.9913; 27.875; -175.9907; 27.875; -175.9889; 27.8619; -175.9782; 27.848; -175.9735; 27.8449; -175.9558; 27.8331; -175.9395; 27.8275; -175.9254; 27.8234; -175.921; 27.8214; -175.9243; 27.8137; -175.9325; 27.8145; -175.9388; 27.8186; -175.9645; 27.827; -175.9746; 27.8302; -175.9832; 27.8314; -175.9907; 27.8326; -176; 27.8305; -176; 27.8315; -176; 27.8344; -176; 27.8353; -176.0062; 27.8326; -176.0108; 27.8303; -176.025; 27.8216; -176.0268; 27.8195; -176.0287; 27.8173; -176.0366; 27.8071; -176.0426; 27.7981; -176.0434; 27.7959; -174.0675; 26.0525; -174.0659; 26.0394; -174.0599; 26.0227; -174.0592; 26.0207; -174.0461; 26.0023; -174.0431; 26; -174.042; 26; -174.0387; 26; -174.0375; 26; -174.0309; 25.9957; -174.0272; 25.9933; -174.0079; 25.9905; -174.0064; 25.9903; -174; 25.9902; -174; 25.9907; -174; 25.9923; -174; 25.9929; -173.9959; 25.994; -173.9918; 25.9951; -173.9845; 25.9976; -173.984; 25.9979; -173.9803; 26; -173.9796; 26; -173.9777; 26; -173.977; 26; -173.9649; 26.0066; -173.9431; 26.0107; -173.9428; 26.0107; -173.926; 26.0196; -173.9131; 26.036; -173.9034; 26.0601; -173.9038; 26.0668; -173.9085; 26.0819; -173.9134; 26.0994; -173.914; 26.1005; -173.9186; 26.1097; -173.926; 26.1172; -173.9291; 26.1201; -173.9389; 26.125; -173.9361; 26.125; -173.9503; 26.1332; -173.9579; 26.1357; -173.9696; 26.1354; -173.9814; 26.1332; -173.9919; 26.1366; -174; 26.1369; -174; 26.1355; -174.0007; 26.1357; -174.0028; 26.1363; -174.0035; 26.1365; -174.0071; 26.1371; -174.0109; 26.1366; -174.011; 26.1366; -174.0189; 26.134; -174.0311; 26.1291; -174.0318; 26.1287; -174.0383; 26.125; -174.0379; 26.125; -174.037; 26.125; -174.0366; 26.125; -174.0407; 26.1226; -174.0496; 26.1166; -174.0525; 26.113; -174.0548; 26.1077; -174.0556; 26.1053; -174.0591; 26.0942; -174.0615; 26.082; -174.0674; 26.0596; -174.0675; 26.0525; -171.8096; 25.7813; -171.8081; 25.7729; -171.807; 25.7671; -171.8004; 25.75; -171.8006; 25.75; -171.797; 25.7405; -171.7947; 25.7386; -171.7829; 25.7283; -171.7702; 25.7182; -171.7626; 25.7148; -171.7553; 25.7115; -171.75; 25.7103; -171.75; 25.7101; -171.75; 25.7094; -171.75; 25.7092; -171.7375; 25.7065; -171.7314; 25.7075; -171.7184; 25.7095; -171.6998; 25.7169; -171.6869; 25.7279; -171.6829; 25.7333; -171.6805; 25.7368; -171.6777; 25.75; -171.669; 25.7777; -171.6679; 25.7812; -171.6694; 25.7939; -171.6766; 25.8109; -171.6883; 25.8238; -171.7106; 25.8332; -171.7211; 25.8339; -171.7315; 25.8346; -171.75; 25.8379; -171.7681; 25.8337; -171.7719; 25.8314; -171.7729; 25.8308; -171.787; 25.8223; -171.8001; 25.8058; -171.8065; 25.7934; -171.8096; 25.7813; -170.6849; 25.5064; -170.6848; 25.5048; -170.6847; 25.5031; -170.6846; 25.5014; -170.6843; 25.4998; -170.6841; 25.4981; -170.6837; 25.4965; -170.6833; 25.4949; -170.6828; 25.4932; -170.6823; 25.4916; -170.6817; 25.4901; -170.6811; 25.4885; -170.6804; 25.4869; -170.6797; 25.4854; -170.6789; 25.4839; -170.6781; 25.4824; -170.6772; 25.4809; -170.6762; 25.4795; -170.6752; 25.4781; -170.6741; 25.4767; -170.673; 25.4754; -170.6719; 25.4741; -170.6707; 25.4729; -170.6694; 25.4716; -170.6681; 25.4704; -170.6674; 25.4698; -170.6663; 25.4689; -170.665; 25.4678; -170.6635; 25.4668; -170.6621; 25.4657; -170.6606; 25.4648; -170.6591; 25.4638; -170.6575; 25.4629; -170.6559; 25.4621; -170.6543; 25.4613; -170.6526; 25.4606; -170.6509; 25.4599; -170.6492; 25.4593; -170.6475; 25.4587; -170.6458; 25.4582; -170.644; 25.4577; -170.6422; 25.4573; -170.6404; 25.4569; -170.6386; 25.4566; -170.6368; 25.4563; -170.635; 25.4561; -170.6331; 25.456; -170.6313; 25.4559; -170.6295; 25.4558; -170.6276; 25.4558; -170.6258; 25.4559; -170.6239; 25.456; -170.6221; 25.4562; -170.6203; 25.4564; -170.6185; 25.4567; -170.6167; 25.4571; -170.6149; 25.4575; -170.6131; 25.4579; -170.6113; 25.4584; -170.6096; 25.459; -170.6079; 25.4596; -170.6062; 25.4602; -170.6045; 25.461; -170.6029; 25.4617; -170.6013; 25.4625; -170.5997; 25.4634; -170.5982; 25.4643; -170.5967; 25.4652; -170.5952; 25.4662; -170.5937; 25.4673; -170.5923; 25.4684; -170.591; 25.4695; -170.5897; 25.4706; -170.5884; 25.4719; -170.5871; 25.4731; -170.5859; 25.4744; -170.5848; 25.4757; -170.5837; 25.477; -170.5827; 25.4784; -170.5817; 25.4798; -170.5807; 25.4812; -170.5798; 25.4827; -170.579; 25.4842; -170.5782; 25.4857; -170.5775; 25.4872; -170.5768; 25.4888; -170.5762; 25.4904; -170.5757; 25.492; -170.5752; 25.4936; -170.5747; 25.4952; -170.5744; 25.4968; -170.5741; 25.4985; -170.5738; 25.5002; -170.5736; 25.5018; -170.5735; 25.5035; -170.5734; 25.5051; -170.5734; 25.5068; -170.5735; 25.5085; -170.5736; 25.5101; -170.5737; 25.5118; -170.574; 25.5135; -170.5743; 25.5151; -170.5746; 25.5168; -170.5751; 25.5184; -170.5755; 25.52; -170.5761; 25.5216; -170.5767; 25.5232; -170.5773; 25.5248; -170.578; 25.5263; -170.5787; 25.5278; -170.5795; 25.5293; -170.5804; 25.5308; -170.5813; 25.5323; -170.5823; 25.5337; -170.5833; 25.5351; -170.5844; 25.5364; -170.5855; 25.5378; -170.5866; 25.5391; -170.5879; 25.5403; -170.5891; 25.5415; -170.5904; 25.5427; -170.5917; 25.5439; -170.5931; 25.545; -170.5945; 25.5461; -170.596; 25.5471; -170.5975; 25.5481; -170.599; 25.549; -170.6005; 25.5499; -170.6021; 25.5507; -170.6038; 25.5515; -170.6054; 25.5523; -170.6071; 25.5529; -170.6088; 25.5536; -170.6105; 25.5542; -170.6122; 25.5547; -170.614; 25.5552; -170.6158; 25.5556; -170.6176; 25.556; -170.6194; 25.5563; -170.6212; 25.5566; -170.623; 25.5568; -170.6249; 25.557; -170.6267; 25.5571; -170.6285; 25.5571; -170.6304; 25.5571; -170.6322; 25.5571; -170.6341; 25.557; -170.6359; 25.5568; -170.6377; 25.5566; -170.6395; 25.5563; -170.6413; 25.556; -170.6431; 25.5556; -170.6449; 25.5551; -170.6467; 25.5546; -170.6484; 25.5541; -170.6501; 25.5535; -170.6518; 25.5528; -170.6535; 25.5522; -170.6551; 25.5514; -170.6567; 25.5506; -170.6583; 25.5497; -170.6599; 25.5489; -170.6614; 25.5479; -170.6629; 25.5469; -170.6644; 25.5459; -170.6658; 25.5448; -170.6671; 25.5437; -170.6685; 25.5425; -170.6697; 25.5413; -170.671; 25.5401; -170.6722; 25.5388; -170.6733; 25.5375; -170.6744; 25.5362; -170.6755; 25.5348; -170.6764; 25.5334; -170.6774; 25.532; -170.6783; 25.5305; -170.6791; 25.529; -170.6799; 25.5275; -170.6807; 25.526; -170.6813; 25.5244; -170.682; 25.5229; -170.6825; 25.5213; -170.683; 25.5197; -170.6835; 25.518; -170.6839; 25.5164; -170.6842; 25.5148; -170.6844; 25.5131; -170.6846; 25.5114; -170.6848; 25.5098; -170.6849; 25.5081; -170.6849; 25.5064; -168.0584; 24.9879; -168.0503; 24.9745; -168.0378; 24.9597; -168.0236; 24.9545; -168; 24.9507; -168; 24.9502; -168; 24.9486; -168; 24.9481; -167.9835; 24.9493; -167.9825; 24.9496; -167.9668; 24.9549; -167.9586; 24.9614; -167.9537; 24.9644; -167.949; 24.9736; -167.9473; 24.9814; -167.9467; 24.9829; -167.9442; 24.9898; -167.9446; 25; -167.9449; 25; -167.946; 25; -167.9463; 25; -167.9479; 25.0095; -167.9499; 25.0157; -167.9524; 25.0235; -167.962; 25.0332; -167.9725; 25.0412; -167.9847; 25.047; -167.9889; 25.049; -168; 25.0522; -168; 25.0503; -168.0017; 25.0502; -168.0064; 25.05; -168.0085; 25.0499; -168.0097; 25.0498; -168.0132; 25.0492; -168.016; 25.0486; -168.0222; 25.0467; -168.027; 25.0448; -168.03; 25.0431; -168.0355; 25.04; -168.0421; 25.0354; -168.0466; 25.0313; -168.0506; 25.0259; -168.0526; 25.0213; -168.0547; 25.0153; -168.0562; 25.0105; -168.0572; 25.0059; -168.058; 25.0026; -168.0582; 25; -168.0584; 24.9879; -166.3865; 23.8464; -166.3845; 23.832; -166.3829; 23.8297; -166.3788; 23.8236; -166.375; 23.8216; -166.375; 23.8222; -166.375; 23.824; -166.375; 23.8246; -166.3692; 23.8155; -166.3573; 23.8066; -166.3563; 23.8059; -166.3368; 23.7996; -166.3226; 23.7991; -166.3136; 23.8037; -166.3192; 23.791; -166.323; 23.7744; -166.3237; 23.771; -166.3202; 23.7585; -166.3167; 23.75; -166.3173; 23.75; -166.3191; 23.75; -166.3197; 23.75; -166.3158; 23.7401; -166.3111; 23.736; -166.3026; 23.7287; -166.286; 23.7181; -166.2668; 23.7134; -166.2656; 23.7131; -166.25; 23.7139; -166.25; 23.7148; -166.25; 23.7173; -166.25; 23.7182; -166.2412; 23.7197; -166.2315; 23.7236; -166.2268; 23.7274; -166.2262; 23.7235; -166.2249; 23.7152; -166.2228; 23.7049; -166.2148; 23.6967; -166.2054; 23.6916; -166.212; 23.6855; -166.224; 23.6725; -166.2299; 23.6544; -166.2302; 23.6526; -166.2323; 23.6416; -166.2288; 23.6318; -166.2248; 23.625; -166.2256; 23.625; -166.2281; 23.625; -166.2289; 23.625; -166.2242; 23.6148; -166.2149; 23.6042; -166.2111; 23.5998; -166.1944; 23.5895; -166.1722; 23.5871; -166.1512; 23.5905; -166.1452; 23.5942; -166.1313; 23.603; -166.125; 23.6093; -166.125; 23.6088; -166.125; 23.6075; -166.125; 23.6071; -166.1214; 23.6088; -166.1206; 23.6093; -166.1168; 23.6113; -166.1126; 23.6166; -166.1118; 23.6202; -166.1107; 23.625; -166.112; 23.625; -166.1158; 23.625; -166.1171; 23.625; -166.1139; 23.6346; -166.1131; 23.637; -166.1138; 23.6523; -166.1175; 23.6641; -166.1177; 23.6646; -166.125; 23.6707; -166.125; 23.6714; -166.125; 23.6734; -166.125; 23.6741; -166.1279; 23.6776; -166.1307; 23.681; -166.133; 23.6847; -166.1288; 23.6876; -166.125; 23.6901; -166.125; 23.6893; -166.125; 23.6869; -166.125; 23.6861; -166.1145; 23.6962; -166.1135; 23.6971; -166.1059; 23.7135; -166.1046; 23.7289; -166.106; 23.7379; -166.1068; 23.7425; -166.1133; 23.75; -166.1135; 23.75; -166.1143; 23.75; -166.1146; 23.75; -166.1167; 23.7542; -166.1166; 23.7548; -166.1165; 23.7574; -166.1169; 23.7617; -166.1185; 23.7667; -166.1212; 23.7692; -166.125; 23.7729; -166.125; 23.7715; -166.125; 23.7675; -166.125; 23.7661; -166.1294; 23.7702; -166.1368; 23.7785; -166.1426; 23.7844; -166.143; 23.7845; -166.1482; 23.7855; -166.1502; 23.7997; -166.1535; 23.8189; -166.1649; 23.8354; -166.1697; 23.8374; -166.1683; 23.8401; -166.1653; 23.8496; -166.1648; 23.851; -166.1655; 23.8648; -166.1683; 23.875; -166.1678; 23.875; -166.1664; 23.875; -166.1659; 23.875; -166.1704; 23.8885; -166.1752; 23.894; -166.1823; 23.9023; -166.2043; 23.9172; -166.2293; 23.927; -166.2331; 23.9285; -166.25; 23.9324; -166.25; 23.9289; -166.2647; 23.9285; -166.2785; 23.9259; -166.288; 23.9242; -166.2884; 23.929; -166.3071; 23.9249; -166.3247; 23.918; -166.3301; 23.9083; -166.3514; 23.9029; -166.352; 23.9025; -166.3656; 23.8942; -166.375; 23.8854; -166.375; 23.886; -166.375; 23.8877; -166.375; 23.8883; -166.3776; 23.8862; -166.3805; 23.884; -166.3822; 23.8782; -166.3822; 23.8781; -166.3833; 23.875; -166.3819; 23.875; -166.384; 23.8656; -166.3843; 23.8637; -166.3865; 23.8464; -164.7649; 23.575; -164.7647; 23.5664; -164.7626; 23.5585; -164.7591; 23.5527; -164.7576; 23.5502; -164.7531; 23.5453; -164.75; 23.5411; -164.75; 23.5401; -164.75; 23.5371; -164.75; 23.5361; -164.7394; 23.5302; -164.723; 23.5218; -164.7013; 23.517; -164.6963; 23.517; -164.6852; 23.5171; -164.6733; 23.5211; -164.6639; 23.527; -164.654; 23.5352; -164.6453; 23.5515; -164.64; 23.5761; -164.6446; 23.5945; -164.6541; 23.6071; -164.6688; 23.6166; -164.6826; 23.6228; -164.6889; 23.6234; -164.6974; 23.6233; -164.7023; 23.6233; -164.7098; 23.6232; -164.7246; 23.6211; -164.7401; 23.6144; -164.75; 23.6051; -164.7538; 23.6035; -164.7555; 23.6017; -164.7581; 23.599; -164.7603; 23.5951; -164.7612; 23.5935; -164.7635; 23.5867; -164.7648; 23.5817; -164.7649; 23.575; -161.9876; 23.0699; -161.9872; 23.0567; -161.9854; 23.0411; -161.9761; 23.0256; -161.9552; 23.0092; -161.9319; 23.0053; -161.9311; 23.0054; -161.8942; 23.0094; -161.875; 23.0201; -161.875; 23.0199; -161.875; 23.0194; -161.875; 23.0192; -161.8714; 23.0235; -161.8686; 23.0277; -161.8665; 23.0328; -161.8655; 23.034; -161.8633; 23.0366; -161.8608; 23.0444; -161.8589; 23.0526; -161.8581; 23.0608; -161.8589; 23.0681; -161.86; 23.0757; -161.863; 23.0851; -161.863; 23.0852; -161.8677; 23.0911; -161.8704; 23.0954; -161.8736; 23.0969; -161.875; 23.0975; -161.875; 23.0984; -161.875; 23.1008; -161.875; 23.1016; -161.8876; 23.1104; -161.9194; 23.114; -161.9311; 23.113; -161.9447; 23.1119; -161.9654; 23.105; -161.9825; 23.0913; -161.9876; 23.0699; -158.3447; 21.5777; -158.3441; 21.5698; -158.3422; 21.5643; -158.3401; 21.5611; -158.3396; 21.5603; -158.3351; 21.554; -158.3287; 21.546; -158.3176; 21.5391; -158.3173; 21.5389; -158.2987; 21.5247; -158.3001; 21.5097; -158.301; 21.5; -158.3012; 21.4984; -158.3014; 21.4968; -158.2933; 21.4968; -158.2902; 21.4968; -158.2915; 21.4894; -158.2906; 21.4794; -158.2905; 21.4784; -158.2903; 21.476; -158.2901; 21.4756; -158.2898; 21.4747; -158.2879; 21.4702; -158.2859; 21.4652; -158.2814; 21.4572; -158.2813; 21.457; -158.2786; 21.4529; -158.2764; 21.4496; -158.2762; 21.4493; -158.275; 21.4482; -158.2683; 21.442; -158.268; 21.4414; -158.2662; 21.4379; -158.2638; 21.433; -158.2637; 21.433; -158.2576; 21.4255; -158.2529; 21.4223; -158.252; 21.4217; -158.249; 21.4197; -158.2473; 21.419; -158.2465; 21.4165; -158.2458; 21.4145; -158.2414; 21.4122; -158.2401; 21.4115; -158.24; 21.4114; -158.2397; 21.4097; -158.2388; 21.4049; -158.2386; 21.4032; -158.2371; 21.3977; -158.2356; 21.3894; -158.2352; 21.3887; -158.2319; 21.3811; -158.2289; 21.3756; -158.2283; 21.375; -158.2222; 21.3682; -158.2178; 21.3645; -158.2126; 21.3618; -158.2066; 21.359; -158.2045; 21.3583; -158.2014; 21.3572; -158.1933; 21.3544; -158.1902; 21.3538; -158.1888; 21.3535; -158.1887; 21.3535; -158.1886; 21.3534; -158.1886; 21.3533; -158.187; 21.3511; -158.1833; 21.3459; -158.1827; 21.344; -158.182; 21.3412; -158.1768; 21.3208; -158.1644; 21.2723; -158.1612; 21.2674; -158.1596; 21.2634; -158.1576; 21.2611; -158.1541; 21.2566; -158.15; 21.2525; -158.1493; 21.2517; -158.1468; 21.25; -158.1445; 21.2484; -158.1423; 21.2468; -158.1421; 21.2468; -158.1348; 21.2424; -158.1223; 21.2386; -158.1101; 21.2371; -158.0916; 21.2379; -158.0849; 21.2393; -158.0769; 21.241; -158.0725; 21.2419; -158.0598; 21.2413; -158.0526; 21.2421; -158.0492; 21.2425; -158.0444; 21.2429; -158.039; 21.2432; -158.0326; 21.2445; -158.0281; 21.2468; -158.0272; 21.2478; -158.0257; 21.2483; -158.0241; 21.2485; -158.022; 21.2487; -158.0191; 21.2487; -158.0183; 21.2487; -158.0134; 21.2492; -158.0094; 21.2492; -158.0045; 21.2492; -158.0044; 21.2492; -158.0001; 21.2496; -157.9995; 21.2496; -157.997; 21.2496; -157.9956; 21.2496; -157.9929; 21.25; -157.9919; 21.2501; -157.9907; 21.25; -157.9898; 21.2499; -157.9878; 21.2496; -157.9873; 21.2497; -157.9866; 21.2499; -157.9859; 21.25; -157.9852; 21.2501; -157.9844; 21.2501; -157.9834; 21.2501; -157.98; 21.2507; -157.9768; 21.2514; -157.9756; 21.2517; -157.9744; 21.252; -157.9727; 21.2526; -157.9723; 21.2527; -157.9707; 21.2533; -157.9707; 21.2533; -157.9683; 21.2543; -157.9667; 21.2553; -157.9653; 21.2565; -157.9652; 21.2565; -157.9636; 21.2577; -157.9614; 21.257; -157.9588; 21.256; -157.9566; 21.2556; -157.9534; 21.2546; -157.9527; 21.2546; -157.9471; 21.2538; -157.942; 21.253; -157.9395; 21.2513; -157.9368; 21.25; -157.9367; 21.2499; -157.9337; 21.2488; -157.9315; 21.2483; -157.9279; 21.248; -157.9251; 21.2478; -157.9225; 21.2478; -157.9201; 21.2473; -157.9199; 21.2472; -157.9174; 21.2475; -157.9156; 21.2475; -157.9135; 21.2475; -157.9118; 21.2478; -157.91; 21.2478; -157.9088; 21.2478; -157.9079; 21.2478; -157.9053; 21.248; -157.9036; 21.2483; -157.9019; 21.2488; -157.9002; 21.2496; -157.8987; 21.2499; -157.898; 21.2488; -157.896; 21.2468; -157.8948; 21.2468; -157.8896; 21.2446; -157.8861; 21.2432; -157.8813; 21.2394; -157.8749; 21.2305; -157.8737; 21.2288; -157.8723; 21.2283; -157.8697; 21.2249; -157.869; 21.2239; -157.8666; 21.2208; -157.8658; 21.2197; -157.8656; 21.2194; -157.8641; 21.218; -157.8591; 21.2131; -157.8589; 21.2131; -157.8568; 21.212; -157.8545; 21.2109; -157.851; 21.2091; -157.8477; 21.2078; -157.8453; 21.207; -157.8387; 21.2045; -157.8291; 21.2009; -157.8281; 21.2008; -157.8213; 21.2002; -157.812; 21.1994; -157.8102; 21.1992; -157.8079; 21.1995; -157.7955; 21.2011; -157.7914; 21.2016; -157.7909; 21.2017; -157.7883; 21.2025; -157.779; 21.2054; -157.776; 21.2064; -157.7746; 21.2068; -157.7714; 21.2078; -157.7705; 21.2083; -157.7693; 21.2091; -157.7683; 21.2096; -157.7654; 21.2113; -157.7644; 21.2119; -157.7636; 21.2124; -157.761; 21.2139; -157.7601; 21.2144; -157.758; 21.2156; -157.7555; 21.2176; -157.7533; 21.2194; -157.7508; 21.22; -157.7473; 21.2209; -157.7453; 21.2217; -157.7411; 21.2179; -157.74; 21.2169; -157.7363; 21.2151; -157.7338; 21.2139; -157.7309; 21.2125; -157.7259; 21.2111; -157.7232; 21.2104; -157.7204; 21.2097; -157.7197; 21.2095; -157.7116; 21.2086; -157.7087; 21.2082; -157.7083; 21.2082; -157.6926; 21.209; -157.6894; 21.2092; -157.6758; 21.2138; -157.6651; 21.2199; -157.6535; 21.2291; -157.6513; 21.232; -157.6481; 21.2362; -157.6459; 21.2406; -157.6405; 21.2433; -157.6389; 21.2441; -157.6341; 21.2468; -157.632; 21.2485; -157.6242; 21.254; -157.6223; 21.2553; -157.6161; 21.2604; -157.6147; 21.2619; -157.6077; 21.2691; -157.6009; 21.2829; -157.6; 21.2866; -157.5979; 21.2951; -157.5973; 21.3107; -157.5976; 21.3138; -157.598; 21.3185; -157.5987; 21.3261; -157.6002; 21.3324; -157.6012; 21.3369; -157.6014; 21.3376; -157.6018; 21.3395; -157.602; 21.3402; -157.6022; 21.3411; -157.6023; 21.3415; -157.6035; 21.3438; -157.6039; 21.3446; -157.6047; 21.3462; -157.6071; 21.3508; -157.6079; 21.3524; -157.6082; 21.3531; -157.6153; 21.3616; -157.6201; 21.3677; -157.6223; 21.3718; -157.6223; 21.3727; -157.6254; 21.3746; -157.626; 21.375; -157.6285; 21.3766; -157.6285; 21.3814; -157.6293; 21.3852; -157.6312; 21.3883; -157.6324; 21.39; -157.6324; 21.3915; -157.6324; 21.3929; -157.6332; 21.3976; -157.6342; 21.4022; -157.6347; 21.4044; -157.6351; 21.4057; -157.6358; 21.4078; -157.6363; 21.4091; -157.6378; 21.4139; -157.6378; 21.414; -157.6382; 21.4161; -157.6386; 21.4178; -157.6409; 21.4226; -157.6409; 21.4228; -157.6425; 21.4264; -157.6456; 21.4302; -157.6464; 21.4313; -157.6486; 21.4341; -157.65; 21.4361; -157.6522; 21.4391; -157.65; 21.4418; -157.6496; 21.4423; -157.6495; 21.4424; -157.6474; 21.4455; -157.6455; 21.4487; -157.6433; 21.4538; -157.6418; 21.4582; -157.6407; 21.4627; -157.6412; 21.4672; -157.6428; 21.4723; -157.6454; 21.4768; -157.6477; 21.4805; -157.6485; 21.4819; -157.65; 21.4842; -157.6505; 21.4851; -157.6536; 21.4889; -157.6557; 21.4919; -157.6557; 21.4921; -157.6567; 21.4929; -157.6588; 21.4947; -157.6599; 21.4958; -157.6609; 21.4968; -157.673; 21.5; -157.6778; 21.5019; -157.6835; 21.5078; -157.6927; 21.5135; -157.7026; 21.5187; -157.7065; 21.5196; -157.7122; 21.5208; -157.7126; 21.5208; -157.7277; 21.5198; -157.7411; 21.5174; -157.7473; 21.5153; -157.7509; 21.5165; -157.7619; 21.5264; -157.765; 21.5293; -157.7683; 21.5324; -157.7737; 21.5373; -157.7744; 21.538; -157.775; 21.5386; -157.7762; 21.5397; -157.7774; 21.541; -157.7774; 21.541; -157.7776; 21.5411; -157.7776; 21.5412; -157.7786; 21.5421; -157.78; 21.5436; -157.781; 21.5446; -157.783; 21.5488; -157.7844; 21.5518; -157.7848; 21.5525; -157.7863; 21.5555; -157.7868; 21.5562; -157.7881; 21.5582; -157.7884; 21.5585; -157.7886; 21.5589; -157.7902; 21.5615; -157.7912; 21.5646; -157.7917; 21.5654; -157.7933; 21.5682; -157.7937; 21.5719; -157.7952; 21.5761; -157.7971; 21.581; -157.7986; 21.5852; -157.7991; 21.5859; -157.802; 21.5901; -157.8035; 21.5916; -157.8043; 21.5924; -157.8049; 21.5931; -157.8066; 21.5945; -157.8074; 21.5952; -157.8082; 21.5959; -157.8098; 21.5973; -157.8106; 21.5978; -157.8116; 21.5983; -157.8142; 21.5998; -157.817; 21.6021; -157.8186; 21.6034; -157.8245; 21.6071; -157.8319; 21.6113; -157.8341; 21.6124; -157.8343; 21.6125; -157.8372; 21.6137; -157.8394; 21.6162; -157.8403; 21.6173; -157.8432; 21.6207; -157.8441; 21.6218; -157.8474; 21.6314; -157.8515; 21.6427; -157.8538; 21.6492; -157.8542; 21.6503; -157.8602; 21.6655; -157.8617; 21.6681; -157.865; 21.6741; -157.8655; 21.675; -157.8664; 21.6765; -157.8708; 21.6835; -157.8722; 21.6859; -157.8763; 21.6962; -157.8768; 21.697; -157.8814; 21.7052; -157.8847; 21.7079; -157.8881; 21.71; -157.8914; 21.7121; -157.8942; 21.7148; -157.8964; 21.7183; -157.8981; 21.721; -157.9; 21.7227; -157.9004; 21.7231; -157.9004; 21.7231; -157.9053; 21.7255; -157.9092; 21.728; -157.9105; 21.7293; -157.9139; 21.7329; -157.9219; 21.7414; -157.9242; 21.7435; -157.9279; 21.746; -157.9302; 21.7468; -157.9316; 21.7482; -157.9418; 21.7546; -157.9551; 21.7586; -157.9783; 21.763; -157.9917; 21.763; -157.9972; 21.7616; -158.0082; 21.7553; -158.024; 21.7468; -158.0251; 21.7462; -158.0309; 21.7431; -158.0353; 21.7431; -158.0405; 21.742; -158.0449; 21.7409; -158.0501; 21.7399; -158.0571; 21.7355; -158.0623; 21.7301; -158.0676; 21.7247; -158.0719; 21.7192; -158.0789; 21.716; -158.0818; 21.7139; -158.0833; 21.7127; -158.0885; 21.7095; -158.0886; 21.7095; -158.0955; 21.703; -158.0998; 21.6975; -158.1033; 21.6921; -158.104; 21.6909; -158.1068; 21.6856; -158.1078; 21.6838; -158.1089; 21.6819; -158.1103; 21.6791; -158.1116; 21.6759; -158.1124; 21.6739; -158.1127; 21.6731; -158.1129; 21.6726; -158.1135; 21.6708; -158.1138; 21.67; -158.1143; 21.6687; -158.1147; 21.6672; -158.1165; 21.665; -158.1173; 21.6639; -158.1182; 21.6623; -158.119; 21.6607; -158.1202; 21.6573; -158.1206; 21.6638; -158.1213; 21.6646; -158.1222; 21.6657; -158.1261; 21.6635; -158.1281; 21.6625; -158.1283; 21.6623; -158.1334; 21.6586; -158.1342; 21.658; -158.1351; 21.6571; -158.1392; 21.6532; -158.1445; 21.6469; -158.1488; 21.642; -158.1555; 21.6397; -158.1665; 21.636; -158.175; 21.632; -158.187; 21.6326; -158.1996; 21.6345; -158.215; 21.6331; -158.2302; 21.6308; -158.2472; 21.6311; -158.2677; 21.6281; -158.2782; 21.6278; -158.2896; 21.6254; -158.3019; 21.6218; -158.3097; 21.6218; -158.3119; 21.6218; -158.3197; 21.6173; -158.3242; 21.6157; -158.3277; 21.6118; -158.3299; 21.6094; -158.335; 21.6046; -158.3395; 21.5967; -158.3421; 21.5912; -158.3447; 21.5832; -158.3447; 21.5777</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Grassland</t>
+          <t>Wetland</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2789,38 +2672,48 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q20">
         <v>1</v>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>c284b312-98fe-45a7-9bb5-09261ed497d1</t>
+          <t>96dc0855-1faa-4b76-b276-825d9bc6a8fe</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>study_site_1</t>
         </is>
       </c>
       <c r="C21">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Herbivore-mediated nutrient cycling in semi-arid savanna ecosystems</t>
+          <t>Range shifts of montane mammals under projected warming in the Andes</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Joubert MN; Pieterse AC; van der Berg J</t>
+          <t>Gutierrez MJ; Blanco VF; Quispe RR</t>
         </is>
       </c>
       <c r="F21">
-        <v>2018</v>
+        <v>2020</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>10.1111/1365-2745.13024</t>
+          <t>10.1111/geb.13094</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2835,12 +2728,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-02-28T09:28:05+00:00</t>
+          <t>2026-02-28T09:29:11+00:00</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Cairo, Egypt; 30.0444; 31.2357; 5466227</t>
+          <t>Honolulu County, Hawaii, United States; 21.4682; -157.9605; 3861844; MultiPolygon; -178.4436; 28.419; -178.4405; 28.4052; -178.4332; 28.3978; -178.4159; 28.3801; -178.4137; 28.375; -178.4141; 28.375; -178.4153; 28.375; -178.4157; 28.375; -178.4123; 28.3633; -178.4115; 28.3607; -178.3956; 28.3419; -178.3867; 28.3391; -178.375; 28.3354; -178.375; 28.3358; -178.375; 28.3371; -178.375; 28.3375; -178.3489; 28.3347; -178.3417; 28.3339; -178.3014; 28.3283; -178.2889; 28.3288; -178.2719; 28.3353; -178.2703; 28.3359; -178.2575; 28.3428; -178.25; 28.3494; -178.25; 28.349; -178.25; 28.3476; -178.25; 28.3472; -178.2461; 28.3524; -178.2389; 28.362; -178.2357; 28.369; -178.233; 28.375; -178.2338; 28.375; -178.2363; 28.375; -178.2371; 28.375; -178.2325; 28.3836; -178.2311; 28.3937; -178.2305; 28.3977; -178.2322; 28.4273; -178.2378; 28.4529; -178.2385; 28.4562; -178.25; 28.4682; -178.25; 28.4679; -178.25; 28.467; -178.25; 28.4667; -178.256; 28.4751; -178.257; 28.4765; -178.2712; 28.4886; -178.2801; 28.4944; -178.2888; 28.5; -178.2873; 28.5; -178.2826; 28.5; -178.2811; 28.5; -178.2915; 28.5072; -178.2979; 28.5102; -178.3043; 28.5133; -178.3151; 28.5163; -178.3337; 28.5172; -178.3405; 28.5173; -178.3558; 28.5146; -178.3606; 28.5138; -178.375; 28.5101; -178.375; 28.5096; -178.375; 28.5083; -178.375; 28.5078; -178.3773; 28.5063; -178.3813; 28.5036; -178.3842; 28.5016; -178.3864; 28.5; -178.3883; 28.5; -178.3939; 28.5; -178.3958; 28.5; -178.4118; 28.4837; -178.4168; 28.4782; -178.4276; 28.4661; -178.4383; 28.4441; -178.4436; 28.419; -176.0434; 27.7959; -176.0429; 27.7784; -176.0396; 27.7582; -176.0344; 27.75; -176.0293; 27.7427; -176.0249; 27.738; -176.0235; 27.7367; -176.0055; 27.7203; -176; 27.7161; -176; 27.7147; -176; 27.7107; -176; 27.7093; -175.9763; 27.6969; -175.9696; 27.6934; -175.9395; 27.6882; -175.8988; 27.6983; -175.8952; 27.6992; -175.875; 27.7102; -175.875; 27.7098; -175.875; 27.7088; -175.875; 27.7084; -175.8649; 27.7145; -175.845; 27.7285; -175.8175; 27.723; -175.8029; 27.7235; -175.7791; 27.7257; -175.75; 27.7333; -175.75; 27.7323; -175.7461; 27.7327; -175.7341; 27.7389; -175.7262; 27.75; -175.7248; 27.7526; -175.6784; 27.8432; -175.6766; 27.8468; -175.6665; 27.875; -175.6663; 27.875; -175.6658; 27.875; -175.6656; 27.875; -175.6641; 27.8941; -175.6645; 27.9061; -175.6648; 27.9144; -175.6701; 27.9416; -175.6815; 27.9586; -175.7044; 27.9827; -175.7078; 27.9847; -175.7349; 28; -175.736; 28; -175.739; 28; -175.74; 28; -175.7411; 28.0003; -175.7444; 28.001; -175.7445; 28.001; -175.7455; 28.0013; -175.7457; 28.0014; -175.7463; 28.0016; -175.7466; 28.0016; -175.75; 28.003; -175.7544; 28.004; -175.7697; 28.0075; -175.7786; 28.0081; -175.7863; 28.0086; -175.7868; 28.0086; -175.7999; 28.0082; -175.806; 28.0073; -175.8067; 28.0072; -175.8101; 28.0059; -175.8174; 28.0022; -175.8231; 28; -175.8579; 27.9821; -175.875; 27.9733; -175.875; 27.9738; -175.875; 27.9754; -175.875; 27.9759; -175.9044; 27.9606; -175.9088; 27.9583; -175.9357; 27.9406; -175.9505; 27.9362; -175.9663; 27.9299; -175.9814; 27.9132; -175.9847; 27.9065; -175.9876; 27.9005; -175.9921; 27.8895; -175.9938; 27.875; -175.9931; 27.875; -175.9913; 27.875; -175.9907; 27.875; -175.9889; 27.8619; -175.9782; 27.848; -175.9735; 27.8449; -175.9558; 27.8331; -175.9395; 27.8275; -175.9254; 27.8234; -175.921; 27.8214; -175.9243; 27.8137; -175.9325; 27.8145; -175.9388; 27.8186; -175.9645; 27.827; -175.9746; 27.8302; -175.9832; 27.8314; -175.9907; 27.8326; -176; 27.8305; -176; 27.8315; -176; 27.8344; -176; 27.8353; -176.0062; 27.8326; -176.0108; 27.8303; -176.025; 27.8216; -176.0268; 27.8195; -176.0287; 27.8173; -176.0366; 27.8071; -176.0426; 27.7981; -176.0434; 27.7959; -174.0675; 26.0525; -174.0659; 26.0394; -174.0599; 26.0227; -174.0592; 26.0207; -174.0461; 26.0023; -174.0431; 26; -174.042; 26; -174.0387; 26; -174.0375; 26; -174.0309; 25.9957; -174.0272; 25.9933; -174.0079; 25.9905; -174.0064; 25.9903; -174; 25.9902; -174; 25.9907; -174; 25.9923; -174; 25.9929; -173.9959; 25.994; -173.9918; 25.9951; -173.9845; 25.9976; -173.984; 25.9979; -173.9803; 26; -173.9796; 26; -173.9777; 26; -173.977; 26; -173.9649; 26.0066; -173.9431; 26.0107; -173.9428; 26.0107; -173.926; 26.0196; -173.9131; 26.036; -173.9034; 26.0601; -173.9038; 26.0668; -173.9085; 26.0819; -173.9134; 26.0994; -173.914; 26.1005; -173.9186; 26.1097; -173.926; 26.1172; -173.9291; 26.1201; -173.9389; 26.125; -173.9361; 26.125; -173.9503; 26.1332; -173.9579; 26.1357; -173.9696; 26.1354; -173.9814; 26.1332; -173.9919; 26.1366; -174; 26.1369; -174; 26.1355; -174.0007; 26.1357; -174.0028; 26.1363; -174.0035; 26.1365; -174.0071; 26.1371; -174.0109; 26.1366; -174.011; 26.1366; -174.0189; 26.134; -174.0311; 26.1291; -174.0318; 26.1287; -174.0383; 26.125; -174.0379; 26.125; -174.037; 26.125; -174.0366; 26.125; -174.0407; 26.1226; -174.0496; 26.1166; -174.0525; 26.113; -174.0548; 26.1077; -174.0556; 26.1053; -174.0591; 26.0942; -174.0615; 26.082; -174.0674; 26.0596; -174.0675; 26.0525; -171.8096; 25.7813; -171.8081; 25.7729; -171.807; 25.7671; -171.8004; 25.75; -171.8006; 25.75; -171.797; 25.7405; -171.7947; 25.7386; -171.7829; 25.7283; -171.7702; 25.7182; -171.7626; 25.7148; -171.7553; 25.7115; -171.75; 25.7103; -171.75; 25.7101; -171.75; 25.7094; -171.75; 25.7092; -171.7375; 25.7065; -171.7314; 25.7075; -171.7184; 25.7095; -171.6998; 25.7169; -171.6869; 25.7279; -171.6829; 25.7333; -171.6805; 25.7368; -171.6777; 25.75; -171.669; 25.7777; -171.6679; 25.7812; -171.6694; 25.7939; -171.6766; 25.8109; -171.6883; 25.8238; -171.7106; 25.8332; -171.7211; 25.8339; -171.7315; 25.8346; -171.75; 25.8379; -171.7681; 25.8337; -171.7719; 25.8314; -171.7729; 25.8308; -171.787; 25.8223; -171.8001; 25.8058; -171.8065; 25.7934; -171.8096; 25.7813; -170.6849; 25.5064; -170.6848; 25.5048; -170.6847; 25.5031; -170.6846; 25.5014; -170.6843; 25.4998; -170.6841; 25.4981; -170.6837; 25.4965; -170.6833; 25.4949; -170.6828; 25.4932; -170.6823; 25.4916; -170.6817; 25.4901; -170.6811; 25.4885; -170.6804; 25.4869; -170.6797; 25.4854; -170.6789; 25.4839; -170.6781; 25.4824; -170.6772; 25.4809; -170.6762; 25.4795; -170.6752; 25.4781; -170.6741; 25.4767; -170.673; 25.4754; -170.6719; 25.4741; -170.6707; 25.4729; -170.6694; 25.4716; -170.6681; 25.4704; -170.6674; 25.4698; -170.6663; 25.4689; -170.665; 25.4678; -170.6635; 25.4668; -170.6621; 25.4657; -170.6606; 25.4648; -170.6591; 25.4638; -170.6575; 25.4629; -170.6559; 25.4621; -170.6543; 25.4613; -170.6526; 25.4606; -170.6509; 25.4599; -170.6492; 25.4593; -170.6475; 25.4587; -170.6458; 25.4582; -170.644; 25.4577; -170.6422; 25.4573; -170.6404; 25.4569; -170.6386; 25.4566; -170.6368; 25.4563; -170.635; 25.4561; -170.6331; 25.456; -170.6313; 25.4559; -170.6295; 25.4558; -170.6276; 25.4558; -170.6258; 25.4559; -170.6239; 25.456; -170.6221; 25.4562; -170.6203; 25.4564; -170.6185; 25.4567; -170.6167; 25.4571; -170.6149; 25.4575; -170.6131; 25.4579; -170.6113; 25.4584; -170.6096; 25.459; -170.6079; 25.4596; -170.6062; 25.4602; -170.6045; 25.461; -170.6029; 25.4617; -170.6013; 25.4625; -170.5997; 25.4634; -170.5982; 25.4643; -170.5967; 25.4652; -170.5952; 25.4662; -170.5937; 25.4673; -170.5923; 25.4684; -170.591; 25.4695; -170.5897; 25.4706; -170.5884; 25.4719; -170.5871; 25.4731; -170.5859; 25.4744; -170.5848; 25.4757; -170.5837; 25.477; -170.5827; 25.4784; -170.5817; 25.4798; -170.5807; 25.4812; -170.5798; 25.4827; -170.579; 25.4842; -170.5782; 25.4857; -170.5775; 25.4872; -170.5768; 25.4888; -170.5762; 25.4904; -170.5757; 25.492; -170.5752; 25.4936; -170.5747; 25.4952; -170.5744; 25.4968; -170.5741; 25.4985; -170.5738; 25.5002; -170.5736; 25.5018; -170.5735; 25.5035; -170.5734; 25.5051; -170.5734; 25.5068; -170.5735; 25.5085; -170.5736; 25.5101; -170.5737; 25.5118; -170.574; 25.5135; -170.5743; 25.5151; -170.5746; 25.5168; -170.5751; 25.5184; -170.5755; 25.52; -170.5761; 25.5216; -170.5767; 25.5232; -170.5773; 25.5248; -170.578; 25.5263; -170.5787; 25.5278; -170.5795; 25.5293; -170.5804; 25.5308; -170.5813; 25.5323; -170.5823; 25.5337; -170.5833; 25.5351; -170.5844; 25.5364; -170.5855; 25.5378; -170.5866; 25.5391; -170.5879; 25.5403; -170.5891; 25.5415; -170.5904; 25.5427; -170.5917; 25.5439; -170.5931; 25.545; -170.5945; 25.5461; -170.596; 25.5471; -170.5975; 25.5481; -170.599; 25.549; -170.6005; 25.5499; -170.6021; 25.5507; -170.6038; 25.5515; -170.6054; 25.5523; -170.6071; 25.5529; -170.6088; 25.5536; -170.6105; 25.5542; -170.6122; 25.5547; -170.614; 25.5552; -170.6158; 25.5556; -170.6176; 25.556; -170.6194; 25.5563; -170.6212; 25.5566; -170.623; 25.5568; -170.6249; 25.557; -170.6267; 25.5571; -170.6285; 25.5571; -170.6304; 25.5571; -170.6322; 25.5571; -170.6341; 25.557; -170.6359; 25.5568; -170.6377; 25.5566; -170.6395; 25.5563; -170.6413; 25.556; -170.6431; 25.5556; -170.6449; 25.5551; -170.6467; 25.5546; -170.6484; 25.5541; -170.6501; 25.5535; -170.6518; 25.5528; -170.6535; 25.5522; -170.6551; 25.5514; -170.6567; 25.5506; -170.6583; 25.5497; -170.6599; 25.5489; -170.6614; 25.5479; -170.6629; 25.5469; -170.6644; 25.5459; -170.6658; 25.5448; -170.6671; 25.5437; -170.6685; 25.5425; -170.6697; 25.5413; -170.671; 25.5401; -170.6722; 25.5388; -170.6733; 25.5375; -170.6744; 25.5362; -170.6755; 25.5348; -170.6764; 25.5334; -170.6774; 25.532; -170.6783; 25.5305; -170.6791; 25.529; -170.6799; 25.5275; -170.6807; 25.526; -170.6813; 25.5244; -170.682; 25.5229; -170.6825; 25.5213; -170.683; 25.5197; -170.6835; 25.518; -170.6839; 25.5164; -170.6842; 25.5148; -170.6844; 25.5131; -170.6846; 25.5114; -170.6848; 25.5098; -170.6849; 25.5081; -170.6849; 25.5064; -168.0584; 24.9879; -168.0503; 24.9745; -168.0378; 24.9597; -168.0236; 24.9545; -168; 24.9507; -168; 24.9502; -168; 24.9486; -168; 24.9481; -167.9835; 24.9493; -167.9825; 24.9496; -167.9668; 24.9549; -167.9586; 24.9614; -167.9537; 24.9644; -167.949; 24.9736; -167.9473; 24.9814; -167.9467; 24.9829; -167.9442; 24.9898; -167.9446; 25; -167.9449; 25; -167.946; 25; -167.9463; 25; -167.9479; 25.0095; -167.9499; 25.0157; -167.9524; 25.0235; -167.962; 25.0332; -167.9725; 25.0412; -167.9847; 25.047; -167.9889; 25.049; -168; 25.0522; -168; 25.0503; -168.0017; 25.0502; -168.0064; 25.05; -168.0085; 25.0499; -168.0097; 25.0498; -168.0132; 25.0492; -168.016; 25.0486; -168.0222; 25.0467; -168.027; 25.0448; -168.03; 25.0431; -168.0355; 25.04; -168.0421; 25.0354; -168.0466; 25.0313; -168.0506; 25.0259; -168.0526; 25.0213; -168.0547; 25.0153; -168.0562; 25.0105; -168.0572; 25.0059; -168.058; 25.0026; -168.0582; 25; -168.0584; 24.9879; -166.3865; 23.8464; -166.3845; 23.832; -166.3829; 23.8297; -166.3788; 23.8236; -166.375; 23.8216; -166.375; 23.8222; -166.375; 23.824; -166.375; 23.8246; -166.3692; 23.8155; -166.3573; 23.8066; -166.3563; 23.8059; -166.3368; 23.7996; -166.3226; 23.7991; -166.3136; 23.8037; -166.3192; 23.791; -166.323; 23.7744; -166.3237; 23.771; -166.3202; 23.7585; -166.3167; 23.75; -166.3173; 23.75; -166.3191; 23.75; -166.3197; 23.75; -166.3158; 23.7401; -166.3111; 23.736; -166.3026; 23.7287; -166.286; 23.7181; -166.2668; 23.7134; -166.2656; 23.7131; -166.25; 23.7139; -166.25; 23.7148; -166.25; 23.7173; -166.25; 23.7182; -166.2412; 23.7197; -166.2315; 23.7236; -166.2268; 23.7274; -166.2262; 23.7235; -166.2249; 23.7152; -166.2228; 23.7049; -166.2148; 23.6967; -166.2054; 23.6916; -166.212; 23.6855; -166.224; 23.6725; -166.2299; 23.6544; -166.2302; 23.6526; -166.2323; 23.6416; -166.2288; 23.6318; -166.2248; 23.625; -166.2256; 23.625; -166.2281; 23.625; -166.2289; 23.625; -166.2242; 23.6148; -166.2149; 23.6042; -166.2111; 23.5998; -166.1944; 23.5895; -166.1722; 23.5871; -166.1512; 23.5905; -166.1452; 23.5942; -166.1313; 23.603; -166.125; 23.6093; -166.125; 23.6088; -166.125; 23.6075; -166.125; 23.6071; -166.1214; 23.6088; -166.1206; 23.6093; -166.1168; 23.6113; -166.1126; 23.6166; -166.1118; 23.6202; -166.1107; 23.625; -166.112; 23.625; -166.1158; 23.625; -166.1171; 23.625; -166.1139; 23.6346; -166.1131; 23.637; -166.1138; 23.6523; -166.1175; 23.6641; -166.1177; 23.6646; -166.125; 23.6707; -166.125; 23.6714; -166.125; 23.6734; -166.125; 23.6741; -166.1279; 23.6776; -166.1307; 23.681; -166.133; 23.6847; -166.1288; 23.6876; -166.125; 23.6901; -166.125; 23.6893; -166.125; 23.6869; -166.125; 23.6861; -166.1145; 23.6962; -166.1135; 23.6971; -166.1059; 23.7135; -166.1046; 23.7289; -166.106; 23.7379; -166.1068; 23.7425; -166.1133; 23.75; -166.1135; 23.75; -166.1143; 23.75; -166.1146; 23.75; -166.1167; 23.7542; -166.1166; 23.7548; -166.1165; 23.7574; -166.1169; 23.7617; -166.1185; 23.7667; -166.1212; 23.7692; -166.125; 23.7729; -166.125; 23.7715; -166.125; 23.7675; -166.125; 23.7661; -166.1294; 23.7702; -166.1368; 23.7785; -166.1426; 23.7844; -166.143; 23.7845; -166.1482; 23.7855; -166.1502; 23.7997; -166.1535; 23.8189; -166.1649; 23.8354; -166.1697; 23.8374; -166.1683; 23.8401; -166.1653; 23.8496; -166.1648; 23.851; -166.1655; 23.8648; -166.1683; 23.875; -166.1678; 23.875; -166.1664; 23.875; -166.1659; 23.875; -166.1704; 23.8885; -166.1752; 23.894; -166.1823; 23.9023; -166.2043; 23.9172; -166.2293; 23.927; -166.2331; 23.9285; -166.25; 23.9324; -166.25; 23.9289; -166.2647; 23.9285; -166.2785; 23.9259; -166.288; 23.9242; -166.2884; 23.929; -166.3071; 23.9249; -166.3247; 23.918; -166.3301; 23.9083; -166.3514; 23.9029; -166.352; 23.9025; -166.3656; 23.8942; -166.375; 23.8854; -166.375; 23.886; -166.375; 23.8877; -166.375; 23.8883; -166.3776; 23.8862; -166.3805; 23.884; -166.3822; 23.8782; -166.3822; 23.8781; -166.3833; 23.875; -166.3819; 23.875; -166.384; 23.8656; -166.3843; 23.8637; -166.3865; 23.8464; -164.7649; 23.575; -164.7647; 23.5664; -164.7626; 23.5585; -164.7591; 23.5527; -164.7576; 23.5502; -164.7531; 23.5453; -164.75; 23.5411; -164.75; 23.5401; -164.75; 23.5371; -164.75; 23.5361; -164.7394; 23.5302; -164.723; 23.5218; -164.7013; 23.517; -164.6963; 23.517; -164.6852; 23.5171; -164.6733; 23.5211; -164.6639; 23.527; -164.654; 23.5352; -164.6453; 23.5515; -164.64; 23.5761; -164.6446; 23.5945; -164.6541; 23.6071; -164.6688; 23.6166; -164.6826; 23.6228; -164.6889; 23.6234; -164.6974; 23.6233; -164.7023; 23.6233; -164.7098; 23.6232; -164.7246; 23.6211; -164.7401; 23.6144; -164.75; 23.6051; -164.7538; 23.6035; -164.7555; 23.6017; -164.7581; 23.599; -164.7603; 23.5951; -164.7612; 23.5935; -164.7635; 23.5867; -164.7648; 23.5817; -164.7649; 23.575; -161.9876; 23.0699; -161.9872; 23.0567; -161.9854; 23.0411; -161.9761; 23.0256; -161.9552; 23.0092; -161.9319; 23.0053; -161.9311; 23.0054; -161.8942; 23.0094; -161.875; 23.0201; -161.875; 23.0199; -161.875; 23.0194; -161.875; 23.0192; -161.8714; 23.0235; -161.8686; 23.0277; -161.8665; 23.0328; -161.8655; 23.034; -161.8633; 23.0366; -161.8608; 23.0444; -161.8589; 23.0526; -161.8581; 23.0608; -161.8589; 23.0681; -161.86; 23.0757; -161.863; 23.0851; -161.863; 23.0852; -161.8677; 23.0911; -161.8704; 23.0954; -161.8736; 23.0969; -161.875; 23.0975; -161.875; 23.0984; -161.875; 23.1008; -161.875; 23.1016; -161.8876; 23.1104; -161.9194; 23.114; -161.9311; 23.113; -161.9447; 23.1119; -161.9654; 23.105; -161.9825; 23.0913; -161.9876; 23.0699; -158.3447; 21.5777; -158.3441; 21.5698; -158.3422; 21.5643; -158.3401; 21.5611; -158.3396; 21.5603; -158.3351; 21.554; -158.3287; 21.546; -158.3176; 21.5391; -158.3173; 21.5389; -158.2987; 21.5247; -158.3001; 21.5097; -158.301; 21.5; -158.3012; 21.4984; -158.3014; 21.4968; -158.2933; 21.4968; -158.2902; 21.4968; -158.2915; 21.4894; -158.2906; 21.4794; -158.2905; 21.4784; -158.2903; 21.476; -158.2901; 21.4756; -158.2898; 21.4747; -158.2879; 21.4702; -158.2859; 21.4652; -158.2814; 21.4572; -158.2813; 21.457; -158.2786; 21.4529; -158.2764; 21.4496; -158.2762; 21.4493; -158.275; 21.4482; -158.2683; 21.442; -158.268; 21.4414; -158.2662; 21.4379; -158.2638; 21.433; -158.2637; 21.433; -158.2576; 21.4255; -158.2529; 21.4223; -158.252; 21.4217; -158.249; 21.4197; -158.2473; 21.419; -158.2465; 21.4165; -158.2458; 21.4145; -158.2414; 21.4122; -158.2401; 21.4115; -158.24; 21.4114; -158.2397; 21.4097; -158.2388; 21.4049; -158.2386; 21.4032; -158.2371; 21.3977; -158.2356; 21.3894; -158.2352; 21.3887; -158.2319; 21.3811; -158.2289; 21.3756; -158.2283; 21.375; -158.2222; 21.3682; -158.2178; 21.3645; -158.2126; 21.3618; -158.2066; 21.359; -158.2045; 21.3583; -158.2014; 21.3572; -158.1933; 21.3544; -158.1902; 21.3538; -158.1888; 21.3535; -158.1887; 21.3535; -158.1886; 21.3534; -158.1886; 21.3533; -158.187; 21.3511; -158.1833; 21.3459; -158.1827; 21.344; -158.182; 21.3412; -158.1768; 21.3208; -158.1644; 21.2723; -158.1612; 21.2674; -158.1596; 21.2634; -158.1576; 21.2611; -158.1541; 21.2566; -158.15; 21.2525; -158.1493; 21.2517; -158.1468; 21.25; -158.1445; 21.2484; -158.1423; 21.2468; -158.1421; 21.2468; -158.1348; 21.2424; -158.1223; 21.2386; -158.1101; 21.2371; -158.0916; 21.2379; -158.0849; 21.2393; -158.0769; 21.241; -158.0725; 21.2419; -158.0598; 21.2413; -158.0526; 21.2421; -158.0492; 21.2425; -158.0444; 21.2429; -158.039; 21.2432; -158.0326; 21.2445; -158.0281; 21.2468; -158.0272; 21.2478; -158.0257; 21.2483; -158.0241; 21.2485; -158.022; 21.2487; -158.0191; 21.2487; -158.0183; 21.2487; -158.0134; 21.2492; -158.0094; 21.2492; -158.0045; 21.2492; -158.0044; 21.2492; -158.0001; 21.2496; -157.9995; 21.2496; -157.997; 21.2496; -157.9956; 21.2496; -157.9929; 21.25; -157.9919; 21.2501; -157.9907; 21.25; -157.9898; 21.2499; -157.9878; 21.2496; -157.9873; 21.2497; -157.9866; 21.2499; -157.9859; 21.25; -157.9852; 21.2501; -157.9844; 21.2501; -157.9834; 21.2501; -157.98; 21.2507; -157.9768; 21.2514; -157.9756; 21.2517; -157.9744; 21.252; -157.9727; 21.2526; -157.9723; 21.2527; -157.9707; 21.2533; -157.9707; 21.2533; -157.9683; 21.2543; -157.9667; 21.2553; -157.9653; 21.2565; -157.9652; 21.2565; -157.9636; 21.2577; -157.9614; 21.257; -157.9588; 21.256; -157.9566; 21.2556; -157.9534; 21.2546; -157.9527; 21.2546; -157.9471; 21.2538; -157.942; 21.253; -157.9395; 21.2513; -157.9368; 21.25; -157.9367; 21.2499; -157.9337; 21.2488; -157.9315; 21.2483; -157.9279; 21.248; -157.9251; 21.2478; -157.9225; 21.2478; -157.9201; 21.2473; -157.9199; 21.2472; -157.9174; 21.2475; -157.9156; 21.2475; -157.9135; 21.2475; -157.9118; 21.2478; -157.91; 21.2478; -157.9088; 21.2478; -157.9079; 21.2478; -157.9053; 21.248; -157.9036; 21.2483; -157.9019; 21.2488; -157.9002; 21.2496; -157.8987; 21.2499; -157.898; 21.2488; -157.896; 21.2468; -157.8948; 21.2468; -157.8896; 21.2446; -157.8861; 21.2432; -157.8813; 21.2394; -157.8749; 21.2305; -157.8737; 21.2288; -157.8723; 21.2283; -157.8697; 21.2249; -157.869; 21.2239; -157.8666; 21.2208; -157.8658; 21.2197; -157.8656; 21.2194; -157.8641; 21.218; -157.8591; 21.2131; -157.8589; 21.2131; -157.8568; 21.212; -157.8545; 21.2109; -157.851; 21.2091; -157.8477; 21.2078; -157.8453; 21.207; -157.8387; 21.2045; -157.8291; 21.2009; -157.8281; 21.2008; -157.8213; 21.2002; -157.812; 21.1994; -157.8102; 21.1992; -157.8079; 21.1995; -157.7955; 21.2011; -157.7914; 21.2016; -157.7909; 21.2017; -157.7883; 21.2025; -157.779; 21.2054; -157.776; 21.2064; -157.7746; 21.2068; -157.7714; 21.2078; -157.7705; 21.2083; -157.7693; 21.2091; -157.7683; 21.2096; -157.7654; 21.2113; -157.7644; 21.2119; -157.7636; 21.2124; -157.761; 21.2139; -157.7601; 21.2144; -157.758; 21.2156; -157.7555; 21.2176; -157.7533; 21.2194; -157.7508; 21.22; -157.7473; 21.2209; -157.7453; 21.2217; -157.7411; 21.2179; -157.74; 21.2169; -157.7363; 21.2151; -157.7338; 21.2139; -157.7309; 21.2125; -157.7259; 21.2111; -157.7232; 21.2104; -157.7204; 21.2097; -157.7197; 21.2095; -157.7116; 21.2086; -157.7087; 21.2082; -157.7083; 21.2082; -157.6926; 21.209; -157.6894; 21.2092; -157.6758; 21.2138; -157.6651; 21.2199; -157.6535; 21.2291; -157.6513; 21.232; -157.6481; 21.2362; -157.6459; 21.2406; -157.6405; 21.2433; -157.6389; 21.2441; -157.6341; 21.2468; -157.632; 21.2485; -157.6242; 21.254; -157.6223; 21.2553; -157.6161; 21.2604; -157.6147; 21.2619; -157.6077; 21.2691; -157.6009; 21.2829; -157.6; 21.2866; -157.5979; 21.2951; -157.5973; 21.3107; -157.5976; 21.3138; -157.598; 21.3185; -157.5987; 21.3261; -157.6002; 21.3324; -157.6012; 21.3369; -157.6014; 21.3376; -157.6018; 21.3395; -157.602; 21.3402; -157.6022; 21.3411; -157.6023; 21.3415; -157.6035; 21.3438; -157.6039; 21.3446; -157.6047; 21.3462; -157.6071; 21.3508; -157.6079; 21.3524; -157.6082; 21.3531; -157.6153; 21.3616; -157.6201; 21.3677; -157.6223; 21.3718; -157.6223; 21.3727; -157.6254; 21.3746; -157.626; 21.375; -157.6285; 21.3766; -157.6285; 21.3814; -157.6293; 21.3852; -157.6312; 21.3883; -157.6324; 21.39; -157.6324; 21.3915; -157.6324; 21.3929; -157.6332; 21.3976; -157.6342; 21.4022; -157.6347; 21.4044; -157.6351; 21.4057; -157.6358; 21.4078; -157.6363; 21.4091; -157.6378; 21.4139; -157.6378; 21.414; -157.6382; 21.4161; -157.6386; 21.4178; -157.6409; 21.4226; -157.6409; 21.4228; -157.6425; 21.4264; -157.6456; 21.4302; -157.6464; 21.4313; -157.6486; 21.4341; -157.65; 21.4361; -157.6522; 21.4391; -157.65; 21.4418; -157.6496; 21.4423; -157.6495; 21.4424; -157.6474; 21.4455; -157.6455; 21.4487; -157.6433; 21.4538; -157.6418; 21.4582; -157.6407; 21.4627; -157.6412; 21.4672; -157.6428; 21.4723; -157.6454; 21.4768; -157.6477; 21.4805; -157.6485; 21.4819; -157.65; 21.4842; -157.6505; 21.4851; -157.6536; 21.4889; -157.6557; 21.4919; -157.6557; 21.4921; -157.6567; 21.4929; -157.6588; 21.4947; -157.6599; 21.4958; -157.6609; 21.4968; -157.673; 21.5; -157.6778; 21.5019; -157.6835; 21.5078; -157.6927; 21.5135; -157.7026; 21.5187; -157.7065; 21.5196; -157.7122; 21.5208; -157.7126; 21.5208; -157.7277; 21.5198; -157.7411; 21.5174; -157.7473; 21.5153; -157.7509; 21.5165; -157.7619; 21.5264; -157.765; 21.5293; -157.7683; 21.5324; -157.7737; 21.5373; -157.7744; 21.538; -157.775; 21.5386; -157.7762; 21.5397; -157.7774; 21.541; -157.7774; 21.541; -157.7776; 21.5411; -157.7776; 21.5412; -157.7786; 21.5421; -157.78; 21.5436; -157.781; 21.5446; -157.783; 21.5488; -157.7844; 21.5518; -157.7848; 21.5525; -157.7863; 21.5555; -157.7868; 21.5562; -157.7881; 21.5582; -157.7884; 21.5585; -157.7886; 21.5589; -157.7902; 21.5615; -157.7912; 21.5646; -157.7917; 21.5654; -157.7933; 21.5682; -157.7937; 21.5719; -157.7952; 21.5761; -157.7971; 21.581; -157.7986; 21.5852; -157.7991; 21.5859; -157.802; 21.5901; -157.8035; 21.5916; -157.8043; 21.5924; -157.8049; 21.5931; -157.8066; 21.5945; -157.8074; 21.5952; -157.8082; 21.5959; -157.8098; 21.5973; -157.8106; 21.5978; -157.8116; 21.5983; -157.8142; 21.5998; -157.817; 21.6021; -157.8186; 21.6034; -157.8245; 21.6071; -157.8319; 21.6113; -157.8341; 21.6124; -157.8343; 21.6125; -157.8372; 21.6137; -157.8394; 21.6162; -157.8403; 21.6173; -157.8432; 21.6207; -157.8441; 21.6218; -157.8474; 21.6314; -157.8515; 21.6427; -157.8538; 21.6492; -157.8542; 21.6503; -157.8602; 21.6655; -157.8617; 21.6681; -157.865; 21.6741; -157.8655; 21.675; -157.8664; 21.6765; -157.8708; 21.6835; -157.8722; 21.6859; -157.8763; 21.6962; -157.8768; 21.697; -157.8814; 21.7052; -157.8847; 21.7079; -157.8881; 21.71; -157.8914; 21.7121; -157.8942; 21.7148; -157.8964; 21.7183; -157.8981; 21.721; -157.9; 21.7227; -157.9004; 21.7231; -157.9004; 21.7231; -157.9053; 21.7255; -157.9092; 21.728; -157.9105; 21.7293; -157.9139; 21.7329; -157.9219; 21.7414; -157.9242; 21.7435; -157.9279; 21.746; -157.9302; 21.7468; -157.9316; 21.7482; -157.9418; 21.7546; -157.9551; 21.7586; -157.9783; 21.763; -157.9917; 21.763; -157.9972; 21.7616; -158.0082; 21.7553; -158.024; 21.7468; -158.0251; 21.7462; -158.0309; 21.7431; -158.0353; 21.7431; -158.0405; 21.742; -158.0449; 21.7409; -158.0501; 21.7399; -158.0571; 21.7355; -158.0623; 21.7301; -158.0676; 21.7247; -158.0719; 21.7192; -158.0789; 21.716; -158.0818; 21.7139; -158.0833; 21.7127; -158.0885; 21.7095; -158.0886; 21.7095; -158.0955; 21.703; -158.0998; 21.6975; -158.1033; 21.6921; -158.104; 21.6909; -158.1068; 21.6856; -158.1078; 21.6838; -158.1089; 21.6819; -158.1103; 21.6791; -158.1116; 21.6759; -158.1124; 21.6739; -158.1127; 21.6731; -158.1129; 21.6726; -158.1135; 21.6708; -158.1138; 21.67; -158.1143; 21.6687; -158.1147; 21.6672; -158.1165; 21.665; -158.1173; 21.6639; -158.1182; 21.6623; -158.119; 21.6607; -158.1202; 21.6573; -158.1206; 21.6638; -158.1213; 21.6646; -158.1222; 21.6657; -158.1261; 21.6635; -158.1281; 21.6625; -158.1283; 21.6623; -158.1334; 21.6586; -158.1342; 21.658; -158.1351; 21.6571; -158.1392; 21.6532; -158.1445; 21.6469; -158.1488; 21.642; -158.1555; 21.6397; -158.1665; 21.636; -158.175; 21.632; -158.187; 21.6326; -158.1996; 21.6345; -158.215; 21.6331; -158.2302; 21.6308; -158.2472; 21.6311; -158.2677; 21.6281; -158.2782; 21.6278; -158.2896; 21.6254; -158.3019; 21.6218; -158.3097; 21.6218; -158.3119; 21.6218; -158.3197; 21.6173; -158.3242; 21.6157; -158.3277; 21.6118; -158.3299; 21.6094; -158.335; 21.6046; -158.3395; 21.5967; -158.3421; 21.5912; -158.3447; 21.5832; -158.3447; 21.5777</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2850,7 +2743,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2860,48 +2753,38 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>simple_group</t>
+          <t>study_site</t>
         </is>
       </c>
       <c r="Q21">
         <v>1</v>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>c284b312-98fe-45a7-9bb5-09261ed497d1</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
+          <t>6a2f0c6a-b4f6-430e-8281-e4adbd7de258</t>
         </is>
       </c>
       <c r="C22">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Herbivore-mediated nutrient cycling in semi-arid savanna ecosystems</t>
+          <t>Mycorrhizal network connectivity shapes seedling recruitment under closed canopy</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Joubert MN; Pieterse AC; van der Berg J</t>
+          <t>MacPherson DL; Simard SW; Heinrich BR</t>
         </is>
       </c>
       <c r="F22">
-        <v>2018</v>
+        <v>2021</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10.1111/1365-2745.13024</t>
+          <t>10.1038/s41559-021-01569-0</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2916,22 +2799,22 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-02-28T09:28:05+00:00</t>
+          <t>2026-02-28T09:30:02+00:00</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Cairo, Egypt; 30.0444; 31.2357; 5466227</t>
+          <t>Hobart, City of Hobart, Tasmania, Australia; -42.8825; 147.3281; 10632745</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Wetland</t>
+          <t>Forest</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -2941,38 +2824,48 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>study_site</t>
+          <t>simple_group</t>
         </is>
       </c>
       <c r="Q22">
         <v>1</v>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>f255dc8a-e048-49cc-aad5-20bbdf70f5b4</t>
+          <t>6a2f0c6a-b4f6-430e-8281-e4adbd7de258</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>study_site_1</t>
         </is>
       </c>
       <c r="C23">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Seed dispersal limitation constrains plant community recovery after tropical forest fragmentation</t>
+          <t>Mycorrhizal network connectivity shapes seedling recruitment under closed canopy</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Almeida FS; Ribeiro GH; Neves CT</t>
+          <t>MacPherson DL; Simard SW; Heinrich BR</t>
         </is>
       </c>
       <c r="F23">
-        <v>2022</v>
+        <v>2021</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>10.1111/gcb.16157</t>
+          <t>10.1038/s41559-021-01569-0</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2987,12 +2880,12 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-02-28T09:28:47+00:00</t>
+          <t>2026-02-28T09:30:02+00:00</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Iceland; 64.9842; -18.1059; 299133; MultiPolygon; -25.0135; 65.5045; -25.0079; 65.4708; -24.9887; 65.4379; -24.4824; 64.7928; -23.7161; 63.6161; -23.6902; 63.5848; -23.6531; 63.5559; -23.6058; 63.5302; -23.5496; 63.5083; -23.4861; 63.4908; -23.4171; 63.4783; -23.3444; 63.4711; -23.2701; 63.4693; -23.1961; 63.473; -23.1245; 63.4822; -22.9863; 63.5055; -22.5; 63.4173; -20.774; 63.1019; -20.6951; 63.0905; -20.613; 63.0859; -20.5304; 63.0884; -19.0873; 63.1853; -18.7041; 63.185; -18.6405; 63.187; -18.5781; 63.193; -18.0646; 63.2592; -17.9667; 63.2776; -17.7678; 63.3278; -17.7098; 63.3452; -17.6585; 63.3664; -17.591; 63.399; -17.3177; 63.5463; -16.5809; 63.5876; -16.5117; 63.5937; -16.4455; 63.6046; -16.384; 63.62; -15.9349; 63.7523; -15.8562; 63.7813; -15.6952; 63.8557; -14.77; 64.0538; -14.705; 64.0704; -14.2054; 64.2218; -14.143; 64.2442; -13.793; 64.3932; -13.671; 64.4519; -13.6426; 64.469; -13.6153; 64.4534; -13.5739; 64.4357; -13.5109; 64.4157; -13.4897; 64.4104; -13.441; 64.4005; -13.416; 64.3965; -13.3664; 64.3907; -13.3379; 64.3884; -13.2862; 64.3863; -13.2578; 64.3862; -13.2054; 64.388; -13.178; 64.39; -13.1266; 64.3958; -13.1008; 64.3997; -13.052; 64.4094; -13.0287; 64.4151; -12.984; 64.4283; -12.9637; 64.4355; -12.9246; 64.4521; -12.8775; 64.4788; -12.8628; 64.4894; -12.8412; 64.5085; -12.83; 64.5211; -12.817; 64.5404; -12.8104; 64.5548; -12.8055; 64.5736; -12.8046; 64.5895; -12.8071; 64.6071; -12.813; 64.6241; -12.8218; 64.6401; -12.8352; 64.6575; -12.8492; 64.6715; -12.8708; 64.6887; -12.8886; 64.7005; -12.9185; 64.7169; -12.939; 64.7263; -12.9771; 64.741; -13.0446; 64.7604; -13.1191; 64.7744; -13.1983; 64.7827; -13.2196; 64.7833; -13.2053; 64.7938; -13.1328; 64.838; -13.0828; 64.8768; -13.0662; 64.894; -13.0437; 64.9236; -13.0322; 64.9544; -13.0138; 65.0538; -13.0134; 65.0826; -13.031; 65.1902; -13.1236; 65.5252; -13.1359; 65.5523; -13.1572; 65.5785; -14.063; 66.4484; -14.1044; 66.479; -14.1587; 66.5063; -14.2241; 66.5294; -14.2987; 66.5475; -14.3802; 66.5601; -15.8898; 66.7267; -16.0151; 66.7333; -16.184; 66.7335; -16.2977; 66.7285; -16.6492; 66.696; -16.7327; 66.685; -16.8101; 66.6684; -16.8788; 66.6467; -17.3761; 66.4565; -17.5468; 66.4292; -17.5259; 66.444; -17.4973; 66.4761; -17.4827; 66.5096; -17.4808; 66.5592; -17.4956; 66.5912; -17.5189; 66.6195; -17.55; 66.6444; -17.5809; 66.665; -17.6304; 66.6926; -17.6864; 66.7154; -17.7304; 66.7291; -17.8096; 66.7473; -17.8959; 66.7595; -17.9863; 66.7653; -18.078; 66.7644; -18.1677; 66.757; -18.2524; 66.7432; -18.3296; 66.7237; -18.3952; 66.6995; -18.4487; 66.671; -18.4886; 66.6393; -18.5136; 66.6052; -18.5187; 66.5857; -18.525; 66.574; -18.5279; 66.5383; -18.5147; 66.5029; -18.5008; 66.4866; -18.4924; 66.4728; -18.4581; 66.4423; -18.4136; 66.4155; -18.3591; 66.3919; -18.3171; 66.3769; -18.8; 66.3851; -18.8604; 66.3845; -20.1192; 66.3368; -22.1606; 66.6292; -22.2041; 66.6386; -22.2962; 66.6543; -22.3748; 66.6626; -22.4558; 66.6656; -22.5; 66.6642; -22.5442; 66.6629; -22.5969; 66.657; -22.878; 66.6662; -22.977; 66.6655; -23.0737; 66.657; -23.1641; 66.6411; -23.3815; 66.5918; -23.4683; 66.5668; -23.5396; 66.5349; -24.1866; 66.1666; -24.2216; 66.1429; -24.5265; 65.8973; -24.9484; 65.6014; -24.9834; 65.5708; -25.0053; 65.5382; -25.0135; 65.5045; -19.1995; 67.151; -19.1994; 67.149; -19.1993; 67.147; -19.1992; 67.145; -19.199; 67.143; -19.1987; 67.141; -19.1984; 67.139; -19.198; 67.137; -19.1976; 67.135; -19.1972; 67.133; -19.1967; 67.131; -19.1961; 67.129; -19.1955; 67.127; -19.1948; 67.125; -19.1941; 67.123; -19.1933; 67.121; -19.1925; 67.119; -19.1916; 67.117; -19.1907; 67.115; -19.1897; 67.113; -19.1886; 67.111; -19.1875; 67.109; -19.1864; 67.107; -19.1852; 67.105; -19.1839; 67.103; -19.1826; 67.101; -19.1812; 67.099; -19.1798; 67.097; -19.1784; 67.095; -19.177; 67.093; -19.1755; 67.091; -19.1739; 67.089; -19.1722; 67.087; -19.1705; 67.085; -19.1688; 67.083; -19.167; 67.081; -19.1651; 67.079; -19.1631; 67.077; -19.1611; 67.075; -19.1591; 67.073; -19.1569; 67.071; -19.1547; 67.069; -19.1525; 67.067; -19.1502; 67.065; -19.1478; 67.063; -19.1453; 67.061; -19.1428; 67.059; -19.1415; 67.058; -19.1401; 67.057; -19.1388; 67.056; -19.1375; 67.055; -19.1361; 67.054; -19.1347; 67.053; -19.1333; 67.052; -19.1319; 67.051; -19.1304; 67.05; -19.129; 67.049; -19.1275; 67.048; -19.126; 67.047; -19.1245; 67.046; -19.1229; 67.045; -19.1214; 67.044; -19.1198; 67.043; -19.1182; 67.042; -19.1165; 67.041; -19.1149; 67.04; -19.1132; 67.039; -19.1115; 67.038; -19.1098; 67.037; -19.1081; 67.036; -19.1063; 67.035; -19.1046; 67.034; -19.1028; 67.033; -19.1009; 67.032; -19.0991; 67.031; -19.0972; 67.03; -19.0953; 67.029; -19.0934; 67.028; -19.0914; 67.027; -19.0895; 67.026; -19.0875; 67.025; -19.0854; 67.024; -19.0834; 67.023; -19.0813; 67.022; -19.0792; 67.021; -19.0771; 67.02; -19.0749; 67.019; -19.0727; 67.018; -19.0705; 67.017; -19.0683; 67.016; -19.066; 67.015; -19.0637; 67.014; -19.0613; 67.013; -19.059; 67.012; -19.0566; 67.011; -19.0541; 67.01; -19.0516; 67.009; -19.0491; 67.008; -19.0466; 67.007; -19.044; 67.006; -19.0414; 67.005; -19.0388; 67.004; -19.0361; 67.003; -19.0333; 67.002; -19.0306; 67.001; -19.0278; 67; -19.0249; 66.999; -19.022; 66.998; -19.0191; 66.997; -19.0161; 66.996; -19.013; 66.995; -19.01; 66.994; -19.0068; 66.993; -19.0037; 66.992; -19.0004; 66.991; -18.9971; 66.99; -18.9938; 66.989; -18.9904; 66.988; -18.9869; 66.987; -18.9834; 66.986; -18.9798; 66.985; -18.9762; 66.984; -18.9725; 66.983; -18.9687; 66.982; -18.9648; 66.981; -18.9609; 66.98; -18.9569; 66.979; -18.9528; 66.978; -18.9486; 66.977; -18.9443; 66.976; -18.9399; 66.975; -18.9355; 66.974; -18.9309; 66.973; -18.9262; 66.972; -18.9213; 66.971; -18.9164; 66.97; -18.9113; 66.969; -18.9061; 66.968; -18.9007; 66.967; -18.8952; 66.966; -18.8895; 66.965; -18.8835; 66.964; -18.8774; 66.963; -18.871; 66.962; -18.8644; 66.961; -18.8575; 66.96; -18.8503; 66.959; -18.8427; 66.958; -18.8346; 66.957; -18.8261; 66.956; -18.817; 66.955; -18.8072; 66.954; -18.7965; 66.953; -18.7846; 66.952; -18.7711; 66.951; -18.755; 66.95; -18.734; 66.949; -18.6888; 66.948; -18.6751; 66.948; -18.6299; 66.949; -18.6089; 66.95; -18.5928; 66.951; -18.5793; 66.952; -18.5674; 66.953; -18.5567; 66.954; -18.5469; 66.955; -18.5378; 66.956; -18.5293; 66.957; -18.5212; 66.958; -18.5136; 66.959; -18.5064; 66.96; -18.4995; 66.961; -18.4929; 66.962; -18.4865; 66.963; -18.4804; 66.964; -18.4744; 66.965; -18.4687; 66.966; -18.4632; 66.967; -18.4578; 66.968; -18.4526; 66.969; -18.4475; 66.97; -18.4425; 66.971; -18.4377; 66.972; -18.433; 66.973; -18.4284; 66.974; -18.424; 66.975; -18.4196; 66.976; -18.4153; 66.977; -18.4111; 66.978; -18.407; 66.979; -18.403; 66.98; -18.3991; 66.981; -18.3952; 66.982; -18.3914; 66.983; -18.3877; 66.984; -18.3841; 66.985; -18.3805; 66.986; -18.3769; 66.987; -18.3735; 66.988; -18.37; 66.989; -18.3666; 66.99; -18.3633; 66.991; -18.36; 66.992; -18.3567; 66.993; -18.3536; 66.994; -18.3504; 66.995; -18.3474; 66.996; -18.3443; 66.997; -18.3413; 66.998; -18.3384; 66.999; -18.3355; 67; -18.3327; 67.001; -18.3298; 67.002; -18.3271; 67.003; -18.3243; 67.004; -18.3216; 67.005; -18.3189; 67.006; -18.3162; 67.007; -18.3136; 67.008; -18.3111; 67.009; -18.3085; 67.01; -18.306; 67.011; -18.3035; 67.012; -18.3011; 67.013; -18.2987; 67.014; -18.2963; 67.015; -18.294; 67.016; -18.2917; 67.017; -18.2894; 67.018; -18.2871; 67.019; -18.2849; 67.02; -18.2827; 67.021; -18.2806; 67.022; -18.2784; 67.023; -18.2763; 67.024; -18.2743; 67.025; -18.2722; 67.026; -18.2702; 67.027; -18.2682; 67.028; -18.2662; 67.029; -18.2643; 67.03; -18.2623; 67.031; -18.2604; 67.032; -18.2586; 67.033; -18.2567; 67.034; -18.2549; 67.035; -18.2531; 67.036; -18.2513; 67.037; -18.2496; 67.038; -18.2478; 67.039; -18.2461; 67.04; -18.2444; 67.041; -18.2427; 67.042; -18.2411; 67.043; -18.2395; 67.044; -18.2379; 67.045; -18.2363; 67.046; -18.2347; 67.047; -18.2332; 67.048; -18.2317; 67.049; -18.2302; 67.05; -18.2287; 67.051; -18.2272; 67.052; -18.2258; 67.053; -18.2243; 67.054; -18.2229; 67.055; -18.2215; 67.056; -18.2202; 67.057; -18.2188; 67.058; -18.2175; 67.059; -18.2162; 67.06; -18.2149; 67.061; -18.2124; 67.063; -18.2099; 67.065; -18.2075; 67.067; -18.2052; 67.069; -18.2029; 67.071; -18.2007; 67.073; -18.1986; 67.075; -18.1965; 67.077; -18.1945; 67.079; -18.1925; 67.081; -18.1907; 67.083; -18.1889; 67.085; -18.1871; 67.087; -18.1854; 67.089; -18.1838; 67.091; -18.1822; 67.093; -18.1807; 67.095; -18.1792; 67.097; -18.1778; 67.099; -18.1764; 67.101; -18.1751; 67.103; -18.1739; 67.105; -18.1727; 67.107; -18.1716; 67.109; -18.1705; 67.111; -18.1695; 67.113; -18.1686; 67.115; -18.1676; 67.117; -18.1668; 67.119; -18.166; 67.121; -18.1652; 67.123; -18.1645; 67.125; -18.1639; 67.127; -18.1633; 67.129; -18.1628; 67.131; -18.1623; 67.133; -18.1618; 67.135; -18.1615; 67.137; -18.1611; 67.139; -18.1609; 67.141; -18.1606; 67.143; -18.1605; 67.145; -18.1603; 67.147; -18.1603; 67.149; -18.1602; 67.151; -18.1603; 67.153; -18.1603; 67.155; -18.1605; 67.157; -18.1607; 67.159; -18.1609; 67.161; -18.1612; 67.163; -18.1615; 67.165; -18.1619; 67.167; -18.1624; 67.169; -18.1629; 67.171; -18.1634; 67.173; -18.164; 67.175; -18.1647; 67.177; -18.1654; 67.179; -18.1661; 67.181; -18.167; 67.183; -18.1678; 67.185; -18.1687; 67.187; -18.1697; 67.189; -18.1707; 67.191; -18.1718; 67.193; -18.173; 67.195; -18.1742; 67.197; -18.1754; 67.199; -18.1766; 67.201; -18.1779; 67.203; -18.1793; 67.205; -18.1807; 67.207; -18.1822; 67.209; -18.1837; 67.211; -18.1853; 67.213; -18.187; 67.215; -18.1887; 67.217; -18.1905; 67.219; -18.1923; 67.221; -18.1943; 67.223; -18.1962; 67.225; -18.1983; 67.227; -18.2004; 67.229; -18.2025; 67.231; -18.2048; 67.233; -18.2071; 67.235; -18.2094; 67.237; -18.2119; 67.239; -18.2144; 67.241; -18.2157; 67.242; -18.217; 67.243; -18.2183; 67.244; -18.2196; 67.245; -18.221; 67.246; -18.2223; 67.247; -18.2237; 67.248; -18.2251; 67.249; -18.2266; 67.25; -18.228; 67.251; -18.2295; 67.252; -18.231; 67.253; -18.2325; 67.254; -18.234; 67.255; -18.2356; 67.256; -18.2371; 67.257; -18.2387; 67.258; -18.2404; 67.259; -18.242; 67.26; -18.2436; 67.261; -18.2453; 67.262; -18.247; 67.263; -18.2488; 67.264; -18.2505; 67.265; -18.2523; 67.266; -18.2541; 67.267; -18.2559; 67.268; -18.2577; 67.269; -18.2596; 67.27; -18.2615; 67.271; -18.2634; 67.272; -18.2653; 67.273; -18.2673; 67.274; -18.2693; 67.275; -18.2713; 67.276; -18.2734; 67.277; -18.2754; 67.278; -18.2775; 67.279; -18.2797; 67.28; -18.2818; 67.281; -18.284; 67.282; -18.2862; 67.283; -18.2885; 67.284; -18.2907; 67.285; -18.293; 67.286; -18.2954; 67.287; -18.2978; 67.288; -18.3002; 67.289; -18.3026; 67.29; -18.3051; 67.291; -18.3076; 67.292; -18.3101; 67.293; -18.3127; 67.294; -18.3153; 67.295; -18.318; 67.296; -18.3206; 67.297; -18.3234; 67.298; -18.3262; 67.299; -18.329; 67.3; -18.3318; 67.301; -18.3347; 67.302; -18.3377; 67.303; -18.3407; 67.304; -18.3437; 67.305; -18.3468; 67.306; -18.3499; 67.307; -18.3531; 67.308; -18.3563; 67.309; -18.3595; 67.31; -18.3628; 67.311; -18.3662; 67.312; -18.3696; 67.313; -18.373; 67.314; -18.3766; 67.315; -18.3802; 67.316; -18.3838; 67.317; -18.3876; 67.318; -18.3914; 67.319; -18.3952; 67.32; -18.3992; 67.321; -18.4032; 67.322; -18.4073; 67.323; -18.4116; 67.324; -18.4159; 67.325; -18.4203; 67.326; -18.4248; 67.327; -18.4294; 67.328; -18.4341; 67.329; -18.4389; 67.33; -18.4439; 67.331; -18.449; 67.332; -18.4543; 67.333; -18.4597; 67.334; -18.4653; 67.335; -18.471; 67.336; -18.477; 67.337; -18.4831; 67.338; -18.4896; 67.339; -18.4962; 67.34; -18.5032; 67.341; -18.5105; 67.342; -18.5181; 67.343; -18.5262; 67.344; -18.5348; 67.345; -18.5439; 67.346; -18.5538; 67.347; -18.5646; 67.348; -18.5766; 67.349; -18.5902; 67.35; -18.6065; 67.351; -18.6277; 67.352; -18.6732; 67.353; -18.6879; 67.353; -18.7334; 67.352; -18.7546; 67.351; -18.7708; 67.35; -18.7845; 67.349; -18.7964; 67.348; -18.8072; 67.347; -18.8171; 67.346; -18.8263; 67.345; -18.8348; 67.344; -18.8429; 67.343; -18.8506; 67.342; -18.8579; 67.341; -18.8648; 67.34; -18.8715; 67.339; -18.8779; 67.338; -18.8841; 67.337; -18.89; 67.336; -18.8958; 67.335; -18.9014; 67.334; -18.9068; 67.333; -18.912; 67.332; -18.9171; 67.331; -18.9221; 67.33; -18.927; 67.329; -18.9317; 67.328; -18.9363; 67.327; -18.9408; 67.326; -18.9452; 67.325; -18.9495; 67.324; -18.9537; 67.323; -18.9578; 67.322; -18.9619; 67.321; -18.9658; 67.32; -18.9697; 67.319; -18.9735; 67.318; -18.9772; 67.317; -18.9809; 67.316; -18.9845; 67.315; -18.988; 67.314; -18.9915; 67.313; -18.9949; 67.312; -18.9982; 67.311; -19.0015; 67.31; -19.0048; 67.309; -19.008; 67.308; -19.0111; 67.307; -19.0142; 67.306; -19.0172; 67.305; -19.0202; 67.304; -19.0232; 67.303; -19.0261; 67.302; -19.0289; 67.301; -19.0317; 67.3; -19.0345; 67.299; -19.0372; 67.298; -19.0399; 67.297; -19.0426; 67.296; -19.0452; 67.295; -19.0478; 67.294; -19.0503; 67.293; -19.0528; 67.292; -19.0553; 67.291; -19.0577; 67.29; -19.0601; 67.289; -19.0625; 67.288; -19.0648; 67.287; -19.0671; 67.286; -19.0694; 67.285; -19.0717; 67.284; -19.0739; 67.283; -19.0761; 67.282; -19.0782; 67.281; -19.0803; 67.28; -19.0824; 67.279; -19.0845; 67.278; -19.0866; 67.277; -19.0886; 67.276; -19.0906; 67.275; -19.0925; 67.274; -19.0945; 67.273; -19.0964; 67.272; -19.0983; 67.271; -19.1002; 67.27; -19.102; 67.269; -19.1038; 67.268; -19.1056; 67.267; -19.1074; 67.266; -19.1091; 67.265; -19.1108; 67.264; -19.1125; 67.263; -19.1142; 67.262; -19.1159; 67.261; -19.1175; 67.26; -19.1191; 67.259; -19.1207; 67.258; -19.1223; 67.257; -19.1239; 67.256; -19.1254; 67.255; -19.1269; 67.254; -19.1284; 67.253; -19.1299; 67.252; -19.1314; 67.251; -19.1329; 67.25; -19.1343; 67.249; -19.1357; 67.248; -19.1372; 67.247; -19.1385; 67.246; -19.1399; 67.245; -19.1413; 67.244; -19.1426; 67.243; -19.1439; 67.242; -19.1452; 67.241; -19.1478; 67.239; -19.1502; 67.237; -19.1526; 67.235; -19.155; 67.233; -19.1572; 67.231; -19.1594; 67.229; -19.1616; 67.227; -19.1636; 67.225; -19.1656; 67.223; -19.1676; 67.221; -19.1695; 67.219; -19.1713; 67.217; -19.173; 67.215; -19.1747; 67.213; -19.1763; 67.211; -19.1779; 67.209; -19.1794; 67.207; -19.1809; 67.205; -19.1823; 67.203; -19.1836; 67.201; -19.1849; 67.199; -19.1861; 67.197; -19.1873; 67.195; -19.1884; 67.193; -19.1895; 67.191; -19.1905; 67.189; -19.1914; 67.187; -19.1923; 67.185; -19.1932; 67.183; -19.1939; 67.181; -19.1947; 67.179; -19.1954; 67.177; -19.196; 67.175; -19.1966; 67.173; -19.1971; 67.171; -19.1976; 67.169; -19.198; 67.167; -19.1983; 67.165; -19.1987; 67.163; -19.1989; 67.161; -19.1991; 67.159; -19.1993; 67.157; -19.1994; 67.155; -19.1995; 67.153; -19.1995; 67.151</t>
+          <t>Hobart, City of Hobart, Tasmania, Australia; -42.8825; 147.3281; 10632745</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -3002,7 +2895,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Iceland</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -3012,395 +2905,10 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>simple_group</t>
+          <t>study_site</t>
         </is>
       </c>
       <c r="Q23">
-        <v>1</v>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>f255dc8a-e048-49cc-aad5-20bbdf70f5b4</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
-        </is>
-      </c>
-      <c r="C24">
-        <v>9</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Seed dispersal limitation constrains plant community recovery after tropical forest fragmentation</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Almeida FS; Ribeiro GH; Neves CT</t>
-        </is>
-      </c>
-      <c r="F24">
-        <v>2022</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>10.1111/gcb.16157</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>reviewed</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>564c9186-f70d-47f2-b285-55baee74f705</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>2026-02-28T09:28:47+00:00</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Iceland; 64.9842; -18.1059; 299133; MultiPolygon; -25.0135; 65.5045; -25.0079; 65.4708; -24.9887; 65.4379; -24.4824; 64.7928; -23.7161; 63.6161; -23.6902; 63.5848; -23.6531; 63.5559; -23.6058; 63.5302; -23.5496; 63.5083; -23.4861; 63.4908; -23.4171; 63.4783; -23.3444; 63.4711; -23.2701; 63.4693; -23.1961; 63.473; -23.1245; 63.4822; -22.9863; 63.5055; -22.5; 63.4173; -20.774; 63.1019; -20.6951; 63.0905; -20.613; 63.0859; -20.5304; 63.0884; -19.0873; 63.1853; -18.7041; 63.185; -18.6405; 63.187; -18.5781; 63.193; -18.0646; 63.2592; -17.9667; 63.2776; -17.7678; 63.3278; -17.7098; 63.3452; -17.6585; 63.3664; -17.591; 63.399; -17.3177; 63.5463; -16.5809; 63.5876; -16.5117; 63.5937; -16.4455; 63.6046; -16.384; 63.62; -15.9349; 63.7523; -15.8562; 63.7813; -15.6952; 63.8557; -14.77; 64.0538; -14.705; 64.0704; -14.2054; 64.2218; -14.143; 64.2442; -13.793; 64.3932; -13.671; 64.4519; -13.6426; 64.469; -13.6153; 64.4534; -13.5739; 64.4357; -13.5109; 64.4157; -13.4897; 64.4104; -13.441; 64.4005; -13.416; 64.3965; -13.3664; 64.3907; -13.3379; 64.3884; -13.2862; 64.3863; -13.2578; 64.3862; -13.2054; 64.388; -13.178; 64.39; -13.1266; 64.3958; -13.1008; 64.3997; -13.052; 64.4094; -13.0287; 64.4151; -12.984; 64.4283; -12.9637; 64.4355; -12.9246; 64.4521; -12.8775; 64.4788; -12.8628; 64.4894; -12.8412; 64.5085; -12.83; 64.5211; -12.817; 64.5404; -12.8104; 64.5548; -12.8055; 64.5736; -12.8046; 64.5895; -12.8071; 64.6071; -12.813; 64.6241; -12.8218; 64.6401; -12.8352; 64.6575; -12.8492; 64.6715; -12.8708; 64.6887; -12.8886; 64.7005; -12.9185; 64.7169; -12.939; 64.7263; -12.9771; 64.741; -13.0446; 64.7604; -13.1191; 64.7744; -13.1983; 64.7827; -13.2196; 64.7833; -13.2053; 64.7938; -13.1328; 64.838; -13.0828; 64.8768; -13.0662; 64.894; -13.0437; 64.9236; -13.0322; 64.9544; -13.0138; 65.0538; -13.0134; 65.0826; -13.031; 65.1902; -13.1236; 65.5252; -13.1359; 65.5523; -13.1572; 65.5785; -14.063; 66.4484; -14.1044; 66.479; -14.1587; 66.5063; -14.2241; 66.5294; -14.2987; 66.5475; -14.3802; 66.5601; -15.8898; 66.7267; -16.0151; 66.7333; -16.184; 66.7335; -16.2977; 66.7285; -16.6492; 66.696; -16.7327; 66.685; -16.8101; 66.6684; -16.8788; 66.6467; -17.3761; 66.4565; -17.5468; 66.4292; -17.5259; 66.444; -17.4973; 66.4761; -17.4827; 66.5096; -17.4808; 66.5592; -17.4956; 66.5912; -17.5189; 66.6195; -17.55; 66.6444; -17.5809; 66.665; -17.6304; 66.6926; -17.6864; 66.7154; -17.7304; 66.7291; -17.8096; 66.7473; -17.8959; 66.7595; -17.9863; 66.7653; -18.078; 66.7644; -18.1677; 66.757; -18.2524; 66.7432; -18.3296; 66.7237; -18.3952; 66.6995; -18.4487; 66.671; -18.4886; 66.6393; -18.5136; 66.6052; -18.5187; 66.5857; -18.525; 66.574; -18.5279; 66.5383; -18.5147; 66.5029; -18.5008; 66.4866; -18.4924; 66.4728; -18.4581; 66.4423; -18.4136; 66.4155; -18.3591; 66.3919; -18.3171; 66.3769; -18.8; 66.3851; -18.8604; 66.3845; -20.1192; 66.3368; -22.1606; 66.6292; -22.2041; 66.6386; -22.2962; 66.6543; -22.3748; 66.6626; -22.4558; 66.6656; -22.5; 66.6642; -22.5442; 66.6629; -22.5969; 66.657; -22.878; 66.6662; -22.977; 66.6655; -23.0737; 66.657; -23.1641; 66.6411; -23.3815; 66.5918; -23.4683; 66.5668; -23.5396; 66.5349; -24.1866; 66.1666; -24.2216; 66.1429; -24.5265; 65.8973; -24.9484; 65.6014; -24.9834; 65.5708; -25.0053; 65.5382; -25.0135; 65.5045; -19.1995; 67.151; -19.1994; 67.149; -19.1993; 67.147; -19.1992; 67.145; -19.199; 67.143; -19.1987; 67.141; -19.1984; 67.139; -19.198; 67.137; -19.1976; 67.135; -19.1972; 67.133; -19.1967; 67.131; -19.1961; 67.129; -19.1955; 67.127; -19.1948; 67.125; -19.1941; 67.123; -19.1933; 67.121; -19.1925; 67.119; -19.1916; 67.117; -19.1907; 67.115; -19.1897; 67.113; -19.1886; 67.111; -19.1875; 67.109; -19.1864; 67.107; -19.1852; 67.105; -19.1839; 67.103; -19.1826; 67.101; -19.1812; 67.099; -19.1798; 67.097; -19.1784; 67.095; -19.177; 67.093; -19.1755; 67.091; -19.1739; 67.089; -19.1722; 67.087; -19.1705; 67.085; -19.1688; 67.083; -19.167; 67.081; -19.1651; 67.079; -19.1631; 67.077; -19.1611; 67.075; -19.1591; 67.073; -19.1569; 67.071; -19.1547; 67.069; -19.1525; 67.067; -19.1502; 67.065; -19.1478; 67.063; -19.1453; 67.061; -19.1428; 67.059; -19.1415; 67.058; -19.1401; 67.057; -19.1388; 67.056; -19.1375; 67.055; -19.1361; 67.054; -19.1347; 67.053; -19.1333; 67.052; -19.1319; 67.051; -19.1304; 67.05; -19.129; 67.049; -19.1275; 67.048; -19.126; 67.047; -19.1245; 67.046; -19.1229; 67.045; -19.1214; 67.044; -19.1198; 67.043; -19.1182; 67.042; -19.1165; 67.041; -19.1149; 67.04; -19.1132; 67.039; -19.1115; 67.038; -19.1098; 67.037; -19.1081; 67.036; -19.1063; 67.035; -19.1046; 67.034; -19.1028; 67.033; -19.1009; 67.032; -19.0991; 67.031; -19.0972; 67.03; -19.0953; 67.029; -19.0934; 67.028; -19.0914; 67.027; -19.0895; 67.026; -19.0875; 67.025; -19.0854; 67.024; -19.0834; 67.023; -19.0813; 67.022; -19.0792; 67.021; -19.0771; 67.02; -19.0749; 67.019; -19.0727; 67.018; -19.0705; 67.017; -19.0683; 67.016; -19.066; 67.015; -19.0637; 67.014; -19.0613; 67.013; -19.059; 67.012; -19.0566; 67.011; -19.0541; 67.01; -19.0516; 67.009; -19.0491; 67.008; -19.0466; 67.007; -19.044; 67.006; -19.0414; 67.005; -19.0388; 67.004; -19.0361; 67.003; -19.0333; 67.002; -19.0306; 67.001; -19.0278; 67; -19.0249; 66.999; -19.022; 66.998; -19.0191; 66.997; -19.0161; 66.996; -19.013; 66.995; -19.01; 66.994; -19.0068; 66.993; -19.0037; 66.992; -19.0004; 66.991; -18.9971; 66.99; -18.9938; 66.989; -18.9904; 66.988; -18.9869; 66.987; -18.9834; 66.986; -18.9798; 66.985; -18.9762; 66.984; -18.9725; 66.983; -18.9687; 66.982; -18.9648; 66.981; -18.9609; 66.98; -18.9569; 66.979; -18.9528; 66.978; -18.9486; 66.977; -18.9443; 66.976; -18.9399; 66.975; -18.9355; 66.974; -18.9309; 66.973; -18.9262; 66.972; -18.9213; 66.971; -18.9164; 66.97; -18.9113; 66.969; -18.9061; 66.968; -18.9007; 66.967; -18.8952; 66.966; -18.8895; 66.965; -18.8835; 66.964; -18.8774; 66.963; -18.871; 66.962; -18.8644; 66.961; -18.8575; 66.96; -18.8503; 66.959; -18.8427; 66.958; -18.8346; 66.957; -18.8261; 66.956; -18.817; 66.955; -18.8072; 66.954; -18.7965; 66.953; -18.7846; 66.952; -18.7711; 66.951; -18.755; 66.95; -18.734; 66.949; -18.6888; 66.948; -18.6751; 66.948; -18.6299; 66.949; -18.6089; 66.95; -18.5928; 66.951; -18.5793; 66.952; -18.5674; 66.953; -18.5567; 66.954; -18.5469; 66.955; -18.5378; 66.956; -18.5293; 66.957; -18.5212; 66.958; -18.5136; 66.959; -18.5064; 66.96; -18.4995; 66.961; -18.4929; 66.962; -18.4865; 66.963; -18.4804; 66.964; -18.4744; 66.965; -18.4687; 66.966; -18.4632; 66.967; -18.4578; 66.968; -18.4526; 66.969; -18.4475; 66.97; -18.4425; 66.971; -18.4377; 66.972; -18.433; 66.973; -18.4284; 66.974; -18.424; 66.975; -18.4196; 66.976; -18.4153; 66.977; -18.4111; 66.978; -18.407; 66.979; -18.403; 66.98; -18.3991; 66.981; -18.3952; 66.982; -18.3914; 66.983; -18.3877; 66.984; -18.3841; 66.985; -18.3805; 66.986; -18.3769; 66.987; -18.3735; 66.988; -18.37; 66.989; -18.3666; 66.99; -18.3633; 66.991; -18.36; 66.992; -18.3567; 66.993; -18.3536; 66.994; -18.3504; 66.995; -18.3474; 66.996; -18.3443; 66.997; -18.3413; 66.998; -18.3384; 66.999; -18.3355; 67; -18.3327; 67.001; -18.3298; 67.002; -18.3271; 67.003; -18.3243; 67.004; -18.3216; 67.005; -18.3189; 67.006; -18.3162; 67.007; -18.3136; 67.008; -18.3111; 67.009; -18.3085; 67.01; -18.306; 67.011; -18.3035; 67.012; -18.3011; 67.013; -18.2987; 67.014; -18.2963; 67.015; -18.294; 67.016; -18.2917; 67.017; -18.2894; 67.018; -18.2871; 67.019; -18.2849; 67.02; -18.2827; 67.021; -18.2806; 67.022; -18.2784; 67.023; -18.2763; 67.024; -18.2743; 67.025; -18.2722; 67.026; -18.2702; 67.027; -18.2682; 67.028; -18.2662; 67.029; -18.2643; 67.03; -18.2623; 67.031; -18.2604; 67.032; -18.2586; 67.033; -18.2567; 67.034; -18.2549; 67.035; -18.2531; 67.036; -18.2513; 67.037; -18.2496; 67.038; -18.2478; 67.039; -18.2461; 67.04; -18.2444; 67.041; -18.2427; 67.042; -18.2411; 67.043; -18.2395; 67.044; -18.2379; 67.045; -18.2363; 67.046; -18.2347; 67.047; -18.2332; 67.048; -18.2317; 67.049; -18.2302; 67.05; -18.2287; 67.051; -18.2272; 67.052; -18.2258; 67.053; -18.2243; 67.054; -18.2229; 67.055; -18.2215; 67.056; -18.2202; 67.057; -18.2188; 67.058; -18.2175; 67.059; -18.2162; 67.06; -18.2149; 67.061; -18.2124; 67.063; -18.2099; 67.065; -18.2075; 67.067; -18.2052; 67.069; -18.2029; 67.071; -18.2007; 67.073; -18.1986; 67.075; -18.1965; 67.077; -18.1945; 67.079; -18.1925; 67.081; -18.1907; 67.083; -18.1889; 67.085; -18.1871; 67.087; -18.1854; 67.089; -18.1838; 67.091; -18.1822; 67.093; -18.1807; 67.095; -18.1792; 67.097; -18.1778; 67.099; -18.1764; 67.101; -18.1751; 67.103; -18.1739; 67.105; -18.1727; 67.107; -18.1716; 67.109; -18.1705; 67.111; -18.1695; 67.113; -18.1686; 67.115; -18.1676; 67.117; -18.1668; 67.119; -18.166; 67.121; -18.1652; 67.123; -18.1645; 67.125; -18.1639; 67.127; -18.1633; 67.129; -18.1628; 67.131; -18.1623; 67.133; -18.1618; 67.135; -18.1615; 67.137; -18.1611; 67.139; -18.1609; 67.141; -18.1606; 67.143; -18.1605; 67.145; -18.1603; 67.147; -18.1603; 67.149; -18.1602; 67.151; -18.1603; 67.153; -18.1603; 67.155; -18.1605; 67.157; -18.1607; 67.159; -18.1609; 67.161; -18.1612; 67.163; -18.1615; 67.165; -18.1619; 67.167; -18.1624; 67.169; -18.1629; 67.171; -18.1634; 67.173; -18.164; 67.175; -18.1647; 67.177; -18.1654; 67.179; -18.1661; 67.181; -18.167; 67.183; -18.1678; 67.185; -18.1687; 67.187; -18.1697; 67.189; -18.1707; 67.191; -18.1718; 67.193; -18.173; 67.195; -18.1742; 67.197; -18.1754; 67.199; -18.1766; 67.201; -18.1779; 67.203; -18.1793; 67.205; -18.1807; 67.207; -18.1822; 67.209; -18.1837; 67.211; -18.1853; 67.213; -18.187; 67.215; -18.1887; 67.217; -18.1905; 67.219; -18.1923; 67.221; -18.1943; 67.223; -18.1962; 67.225; -18.1983; 67.227; -18.2004; 67.229; -18.2025; 67.231; -18.2048; 67.233; -18.2071; 67.235; -18.2094; 67.237; -18.2119; 67.239; -18.2144; 67.241; -18.2157; 67.242; -18.217; 67.243; -18.2183; 67.244; -18.2196; 67.245; -18.221; 67.246; -18.2223; 67.247; -18.2237; 67.248; -18.2251; 67.249; -18.2266; 67.25; -18.228; 67.251; -18.2295; 67.252; -18.231; 67.253; -18.2325; 67.254; -18.234; 67.255; -18.2356; 67.256; -18.2371; 67.257; -18.2387; 67.258; -18.2404; 67.259; -18.242; 67.26; -18.2436; 67.261; -18.2453; 67.262; -18.247; 67.263; -18.2488; 67.264; -18.2505; 67.265; -18.2523; 67.266; -18.2541; 67.267; -18.2559; 67.268; -18.2577; 67.269; -18.2596; 67.27; -18.2615; 67.271; -18.2634; 67.272; -18.2653; 67.273; -18.2673; 67.274; -18.2693; 67.275; -18.2713; 67.276; -18.2734; 67.277; -18.2754; 67.278; -18.2775; 67.279; -18.2797; 67.28; -18.2818; 67.281; -18.284; 67.282; -18.2862; 67.283; -18.2885; 67.284; -18.2907; 67.285; -18.293; 67.286; -18.2954; 67.287; -18.2978; 67.288; -18.3002; 67.289; -18.3026; 67.29; -18.3051; 67.291; -18.3076; 67.292; -18.3101; 67.293; -18.3127; 67.294; -18.3153; 67.295; -18.318; 67.296; -18.3206; 67.297; -18.3234; 67.298; -18.3262; 67.299; -18.329; 67.3; -18.3318; 67.301; -18.3347; 67.302; -18.3377; 67.303; -18.3407; 67.304; -18.3437; 67.305; -18.3468; 67.306; -18.3499; 67.307; -18.3531; 67.308; -18.3563; 67.309; -18.3595; 67.31; -18.3628; 67.311; -18.3662; 67.312; -18.3696; 67.313; -18.373; 67.314; -18.3766; 67.315; -18.3802; 67.316; -18.3838; 67.317; -18.3876; 67.318; -18.3914; 67.319; -18.3952; 67.32; -18.3992; 67.321; -18.4032; 67.322; -18.4073; 67.323; -18.4116; 67.324; -18.4159; 67.325; -18.4203; 67.326; -18.4248; 67.327; -18.4294; 67.328; -18.4341; 67.329; -18.4389; 67.33; -18.4439; 67.331; -18.449; 67.332; -18.4543; 67.333; -18.4597; 67.334; -18.4653; 67.335; -18.471; 67.336; -18.477; 67.337; -18.4831; 67.338; -18.4896; 67.339; -18.4962; 67.34; -18.5032; 67.341; -18.5105; 67.342; -18.5181; 67.343; -18.5262; 67.344; -18.5348; 67.345; -18.5439; 67.346; -18.5538; 67.347; -18.5646; 67.348; -18.5766; 67.349; -18.5902; 67.35; -18.6065; 67.351; -18.6277; 67.352; -18.6732; 67.353; -18.6879; 67.353; -18.7334; 67.352; -18.7546; 67.351; -18.7708; 67.35; -18.7845; 67.349; -18.7964; 67.348; -18.8072; 67.347; -18.8171; 67.346; -18.8263; 67.345; -18.8348; 67.344; -18.8429; 67.343; -18.8506; 67.342; -18.8579; 67.341; -18.8648; 67.34; -18.8715; 67.339; -18.8779; 67.338; -18.8841; 67.337; -18.89; 67.336; -18.8958; 67.335; -18.9014; 67.334; -18.9068; 67.333; -18.912; 67.332; -18.9171; 67.331; -18.9221; 67.33; -18.927; 67.329; -18.9317; 67.328; -18.9363; 67.327; -18.9408; 67.326; -18.9452; 67.325; -18.9495; 67.324; -18.9537; 67.323; -18.9578; 67.322; -18.9619; 67.321; -18.9658; 67.32; -18.9697; 67.319; -18.9735; 67.318; -18.9772; 67.317; -18.9809; 67.316; -18.9845; 67.315; -18.988; 67.314; -18.9915; 67.313; -18.9949; 67.312; -18.9982; 67.311; -19.0015; 67.31; -19.0048; 67.309; -19.008; 67.308; -19.0111; 67.307; -19.0142; 67.306; -19.0172; 67.305; -19.0202; 67.304; -19.0232; 67.303; -19.0261; 67.302; -19.0289; 67.301; -19.0317; 67.3; -19.0345; 67.299; -19.0372; 67.298; -19.0399; 67.297; -19.0426; 67.296; -19.0452; 67.295; -19.0478; 67.294; -19.0503; 67.293; -19.0528; 67.292; -19.0553; 67.291; -19.0577; 67.29; -19.0601; 67.289; -19.0625; 67.288; -19.0648; 67.287; -19.0671; 67.286; -19.0694; 67.285; -19.0717; 67.284; -19.0739; 67.283; -19.0761; 67.282; -19.0782; 67.281; -19.0803; 67.28; -19.0824; 67.279; -19.0845; 67.278; -19.0866; 67.277; -19.0886; 67.276; -19.0906; 67.275; -19.0925; 67.274; -19.0945; 67.273; -19.0964; 67.272; -19.0983; 67.271; -19.1002; 67.27; -19.102; 67.269; -19.1038; 67.268; -19.1056; 67.267; -19.1074; 67.266; -19.1091; 67.265; -19.1108; 67.264; -19.1125; 67.263; -19.1142; 67.262; -19.1159; 67.261; -19.1175; 67.26; -19.1191; 67.259; -19.1207; 67.258; -19.1223; 67.257; -19.1239; 67.256; -19.1254; 67.255; -19.1269; 67.254; -19.1284; 67.253; -19.1299; 67.252; -19.1314; 67.251; -19.1329; 67.25; -19.1343; 67.249; -19.1357; 67.248; -19.1372; 67.247; -19.1385; 67.246; -19.1399; 67.245; -19.1413; 67.244; -19.1426; 67.243; -19.1439; 67.242; -19.1452; 67.241; -19.1478; 67.239; -19.1502; 67.237; -19.1526; 67.235; -19.155; 67.233; -19.1572; 67.231; -19.1594; 67.229; -19.1616; 67.227; -19.1636; 67.225; -19.1656; 67.223; -19.1676; 67.221; -19.1695; 67.219; -19.1713; 67.217; -19.173; 67.215; -19.1747; 67.213; -19.1763; 67.211; -19.1779; 67.209; -19.1794; 67.207; -19.1809; 67.205; -19.1823; 67.203; -19.1836; 67.201; -19.1849; 67.199; -19.1861; 67.197; -19.1873; 67.195; -19.1884; 67.193; -19.1895; 67.191; -19.1905; 67.189; -19.1914; 67.187; -19.1923; 67.185; -19.1932; 67.183; -19.1939; 67.181; -19.1947; 67.179; -19.1954; 67.177; -19.196; 67.175; -19.1966; 67.173; -19.1971; 67.171; -19.1976; 67.169; -19.198; 67.167; -19.1983; 67.165; -19.1987; 67.163; -19.1989; 67.161; -19.1991; 67.159; -19.1993; 67.157; -19.1994; 67.155; -19.1995; 67.153; -19.1995; 67.151</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Iceland</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>study_site</t>
-        </is>
-      </c>
-      <c r="Q24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>96dc0855-1faa-4b76-b276-825d9bc6a8fe</t>
-        </is>
-      </c>
-      <c r="C25">
-        <v>10</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Range shifts of montane mammals under projected warming in the Andes</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Gutierrez MJ; Blanco VF; Quispe RR</t>
-        </is>
-      </c>
-      <c r="F25">
-        <v>2020</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>10.1111/geb.13094</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>reviewed</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>564c9186-f70d-47f2-b285-55baee74f705</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>2026-02-28T09:29:11+00:00</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Honolulu County, Hawaii, United States; 21.4682; -157.9605; 3861844; MultiPolygon; -178.4436; 28.419; -178.4405; 28.4052; -178.4332; 28.3978; -178.4159; 28.3801; -178.4137; 28.375; -178.4141; 28.375; -178.4153; 28.375; -178.4157; 28.375; -178.4123; 28.3633; -178.4115; 28.3607; -178.3956; 28.3419; -178.3867; 28.3391; -178.375; 28.3354; -178.375; 28.3358; -178.375; 28.3371; -178.375; 28.3375; -178.3489; 28.3347; -178.3417; 28.3339; -178.3014; 28.3283; -178.2889; 28.3288; -178.2719; 28.3353; -178.2703; 28.3359; -178.2575; 28.3428; -178.25; 28.3494; -178.25; 28.349; -178.25; 28.3476; -178.25; 28.3472; -178.2461; 28.3524; -178.2389; 28.362; -178.2357; 28.369; -178.233; 28.375; -178.2338; 28.375; -178.2363; 28.375; -178.2371; 28.375; -178.2325; 28.3836; -178.2311; 28.3937; -178.2305; 28.3977; -178.2322; 28.4273; -178.2378; 28.4529; -178.2385; 28.4562; -178.25; 28.4682; -178.25; 28.4679; -178.25; 28.467; -178.25; 28.4667; -178.256; 28.4751; -178.257; 28.4765; -178.2712; 28.4886; -178.2801; 28.4944; -178.2888; 28.5; -178.2873; 28.5; -178.2826; 28.5; -178.2811; 28.5; -178.2915; 28.5072; -178.2979; 28.5102; -178.3043; 28.5133; -178.3151; 28.5163; -178.3337; 28.5172; -178.3405; 28.5173; -178.3558; 28.5146; -178.3606; 28.5138; -178.375; 28.5101; -178.375; 28.5096; -178.375; 28.5083; -178.375; 28.5078; -178.3773; 28.5063; -178.3813; 28.5036; -178.3842; 28.5016; -178.3864; 28.5; -178.3883; 28.5; -178.3939; 28.5; -178.3958; 28.5; -178.4118; 28.4837; -178.4168; 28.4782; -178.4276; 28.4661; -178.4383; 28.4441; -178.4436; 28.419; -176.0434; 27.7959; -176.0429; 27.7784; -176.0396; 27.7582; -176.0344; 27.75; -176.0293; 27.7427; -176.0249; 27.738; -176.0235; 27.7367; -176.0055; 27.7203; -176; 27.7161; -176; 27.7147; -176; 27.7107; -176; 27.7093; -175.9763; 27.6969; -175.9696; 27.6934; -175.9395; 27.6882; -175.8988; 27.6983; -175.8952; 27.6992; -175.875; 27.7102; -175.875; 27.7098; -175.875; 27.7088; -175.875; 27.7084; -175.8649; 27.7145; -175.845; 27.7285; -175.8175; 27.723; -175.8029; 27.7235; -175.7791; 27.7257; -175.75; 27.7333; -175.75; 27.7323; -175.7461; 27.7327; -175.7341; 27.7389; -175.7262; 27.75; -175.7248; 27.7526; -175.6784; 27.8432; -175.6766; 27.8468; -175.6665; 27.875; -175.6663; 27.875; -175.6658; 27.875; -175.6656; 27.875; -175.6641; 27.8941; -175.6645; 27.9061; -175.6648; 27.9144; -175.6701; 27.9416; -175.6815; 27.9586; -175.7044; 27.9827; -175.7078; 27.9847; -175.7349; 28; -175.736; 28; -175.739; 28; -175.74; 28; -175.7411; 28.0003; -175.7444; 28.001; -175.7445; 28.001; -175.7455; 28.0013; -175.7457; 28.0014; -175.7463; 28.0016; -175.7466; 28.0016; -175.75; 28.003; -175.7544; 28.004; -175.7697; 28.0075; -175.7786; 28.0081; -175.7863; 28.0086; -175.7868; 28.0086; -175.7999; 28.0082; -175.806; 28.0073; -175.8067; 28.0072; -175.8101; 28.0059; -175.8174; 28.0022; -175.8231; 28; -175.8579; 27.9821; -175.875; 27.9733; -175.875; 27.9738; -175.875; 27.9754; -175.875; 27.9759; -175.9044; 27.9606; -175.9088; 27.9583; -175.9357; 27.9406; -175.9505; 27.9362; -175.9663; 27.9299; -175.9814; 27.9132; -175.9847; 27.9065; -175.9876; 27.9005; -175.9921; 27.8895; -175.9938; 27.875; -175.9931; 27.875; -175.9913; 27.875; -175.9907; 27.875; -175.9889; 27.8619; -175.9782; 27.848; -175.9735; 27.8449; -175.9558; 27.8331; -175.9395; 27.8275; -175.9254; 27.8234; -175.921; 27.8214; -175.9243; 27.8137; -175.9325; 27.8145; -175.9388; 27.8186; -175.9645; 27.827; -175.9746; 27.8302; -175.9832; 27.8314; -175.9907; 27.8326; -176; 27.8305; -176; 27.8315; -176; 27.8344; -176; 27.8353; -176.0062; 27.8326; -176.0108; 27.8303; -176.025; 27.8216; -176.0268; 27.8195; -176.0287; 27.8173; -176.0366; 27.8071; -176.0426; 27.7981; -176.0434; 27.7959; -174.0675; 26.0525; -174.0659; 26.0394; -174.0599; 26.0227; -174.0592; 26.0207; -174.0461; 26.0023; -174.0431; 26; -174.042; 26; -174.0387; 26; -174.0375; 26; -174.0309; 25.9957; -174.0272; 25.9933; -174.0079; 25.9905; -174.0064; 25.9903; -174; 25.9902; -174; 25.9907; -174; 25.9923; -174; 25.9929; -173.9959; 25.994; -173.9918; 25.9951; -173.9845; 25.9976; -173.984; 25.9979; -173.9803; 26; -173.9796; 26; -173.9777; 26; -173.977; 26; -173.9649; 26.0066; -173.9431; 26.0107; -173.9428; 26.0107; -173.926; 26.0196; -173.9131; 26.036; -173.9034; 26.0601; -173.9038; 26.0668; -173.9085; 26.0819; -173.9134; 26.0994; -173.914; 26.1005; -173.9186; 26.1097; -173.926; 26.1172; -173.9291; 26.1201; -173.9389; 26.125; -173.9361; 26.125; -173.9503; 26.1332; -173.9579; 26.1357; -173.9696; 26.1354; -173.9814; 26.1332; -173.9919; 26.1366; -174; 26.1369; -174; 26.1355; -174.0007; 26.1357; -174.0028; 26.1363; -174.0035; 26.1365; -174.0071; 26.1371; -174.0109; 26.1366; -174.011; 26.1366; -174.0189; 26.134; -174.0311; 26.1291; -174.0318; 26.1287; -174.0383; 26.125; -174.0379; 26.125; -174.037; 26.125; -174.0366; 26.125; -174.0407; 26.1226; -174.0496; 26.1166; -174.0525; 26.113; -174.0548; 26.1077; -174.0556; 26.1053; -174.0591; 26.0942; -174.0615; 26.082; -174.0674; 26.0596; -174.0675; 26.0525; -171.8096; 25.7813; -171.8081; 25.7729; -171.807; 25.7671; -171.8004; 25.75; -171.8006; 25.75; -171.797; 25.7405; -171.7947; 25.7386; -171.7829; 25.7283; -171.7702; 25.7182; -171.7626; 25.7148; -171.7553; 25.7115; -171.75; 25.7103; -171.75; 25.7101; -171.75; 25.7094; -171.75; 25.7092; -171.7375; 25.7065; -171.7314; 25.7075; -171.7184; 25.7095; -171.6998; 25.7169; -171.6869; 25.7279; -171.6829; 25.7333; -171.6805; 25.7368; -171.6777; 25.75; -171.669; 25.7777; -171.6679; 25.7812; -171.6694; 25.7939; -171.6766; 25.8109; -171.6883; 25.8238; -171.7106; 25.8332; -171.7211; 25.8339; -171.7315; 25.8346; -171.75; 25.8379; -171.7681; 25.8337; -171.7719; 25.8314; -171.7729; 25.8308; -171.787; 25.8223; -171.8001; 25.8058; -171.8065; 25.7934; -171.8096; 25.7813; -170.6849; 25.5064; -170.6848; 25.5048; -170.6847; 25.5031; -170.6846; 25.5014; -170.6843; 25.4998; -170.6841; 25.4981; -170.6837; 25.4965; -170.6833; 25.4949; -170.6828; 25.4932; -170.6823; 25.4916; -170.6817; 25.4901; -170.6811; 25.4885; -170.6804; 25.4869; -170.6797; 25.4854; -170.6789; 25.4839; -170.6781; 25.4824; -170.6772; 25.4809; -170.6762; 25.4795; -170.6752; 25.4781; -170.6741; 25.4767; -170.673; 25.4754; -170.6719; 25.4741; -170.6707; 25.4729; -170.6694; 25.4716; -170.6681; 25.4704; -170.6674; 25.4698; -170.6663; 25.4689; -170.665; 25.4678; -170.6635; 25.4668; -170.6621; 25.4657; -170.6606; 25.4648; -170.6591; 25.4638; -170.6575; 25.4629; -170.6559; 25.4621; -170.6543; 25.4613; -170.6526; 25.4606; -170.6509; 25.4599; -170.6492; 25.4593; -170.6475; 25.4587; -170.6458; 25.4582; -170.644; 25.4577; -170.6422; 25.4573; -170.6404; 25.4569; -170.6386; 25.4566; -170.6368; 25.4563; -170.635; 25.4561; -170.6331; 25.456; -170.6313; 25.4559; -170.6295; 25.4558; -170.6276; 25.4558; -170.6258; 25.4559; -170.6239; 25.456; -170.6221; 25.4562; -170.6203; 25.4564; -170.6185; 25.4567; -170.6167; 25.4571; -170.6149; 25.4575; -170.6131; 25.4579; -170.6113; 25.4584; -170.6096; 25.459; -170.6079; 25.4596; -170.6062; 25.4602; -170.6045; 25.461; -170.6029; 25.4617; -170.6013; 25.4625; -170.5997; 25.4634; -170.5982; 25.4643; -170.5967; 25.4652; -170.5952; 25.4662; -170.5937; 25.4673; -170.5923; 25.4684; -170.591; 25.4695; -170.5897; 25.4706; -170.5884; 25.4719; -170.5871; 25.4731; -170.5859; 25.4744; -170.5848; 25.4757; -170.5837; 25.477; -170.5827; 25.4784; -170.5817; 25.4798; -170.5807; 25.4812; -170.5798; 25.4827; -170.579; 25.4842; -170.5782; 25.4857; -170.5775; 25.4872; -170.5768; 25.4888; -170.5762; 25.4904; -170.5757; 25.492; -170.5752; 25.4936; -170.5747; 25.4952; -170.5744; 25.4968; -170.5741; 25.4985; -170.5738; 25.5002; -170.5736; 25.5018; -170.5735; 25.5035; -170.5734; 25.5051; -170.5734; 25.5068; -170.5735; 25.5085; -170.5736; 25.5101; -170.5737; 25.5118; -170.574; 25.5135; -170.5743; 25.5151; -170.5746; 25.5168; -170.5751; 25.5184; -170.5755; 25.52; -170.5761; 25.5216; -170.5767; 25.5232; -170.5773; 25.5248; -170.578; 25.5263; -170.5787; 25.5278; -170.5795; 25.5293; -170.5804; 25.5308; -170.5813; 25.5323; -170.5823; 25.5337; -170.5833; 25.5351; -170.5844; 25.5364; -170.5855; 25.5378; -170.5866; 25.5391; -170.5879; 25.5403; -170.5891; 25.5415; -170.5904; 25.5427; -170.5917; 25.5439; -170.5931; 25.545; -170.5945; 25.5461; -170.596; 25.5471; -170.5975; 25.5481; -170.599; 25.549; -170.6005; 25.5499; -170.6021; 25.5507; -170.6038; 25.5515; -170.6054; 25.5523; -170.6071; 25.5529; -170.6088; 25.5536; -170.6105; 25.5542; -170.6122; 25.5547; -170.614; 25.5552; -170.6158; 25.5556; -170.6176; 25.556; -170.6194; 25.5563; -170.6212; 25.5566; -170.623; 25.5568; -170.6249; 25.557; -170.6267; 25.5571; -170.6285; 25.5571; -170.6304; 25.5571; -170.6322; 25.5571; -170.6341; 25.557; -170.6359; 25.5568; -170.6377; 25.5566; -170.6395; 25.5563; -170.6413; 25.556; -170.6431; 25.5556; -170.6449; 25.5551; -170.6467; 25.5546; -170.6484; 25.5541; -170.6501; 25.5535; -170.6518; 25.5528; -170.6535; 25.5522; -170.6551; 25.5514; -170.6567; 25.5506; -170.6583; 25.5497; -170.6599; 25.5489; -170.6614; 25.5479; -170.6629; 25.5469; -170.6644; 25.5459; -170.6658; 25.5448; -170.6671; 25.5437; -170.6685; 25.5425; -170.6697; 25.5413; -170.671; 25.5401; -170.6722; 25.5388; -170.6733; 25.5375; -170.6744; 25.5362; -170.6755; 25.5348; -170.6764; 25.5334; -170.6774; 25.532; -170.6783; 25.5305; -170.6791; 25.529; -170.6799; 25.5275; -170.6807; 25.526; -170.6813; 25.5244; -170.682; 25.5229; -170.6825; 25.5213; -170.683; 25.5197; -170.6835; 25.518; -170.6839; 25.5164; -170.6842; 25.5148; -170.6844; 25.5131; -170.6846; 25.5114; -170.6848; 25.5098; -170.6849; 25.5081; -170.6849; 25.5064; -168.0584; 24.9879; -168.0503; 24.9745; -168.0378; 24.9597; -168.0236; 24.9545; -168; 24.9507; -168; 24.9502; -168; 24.9486; -168; 24.9481; -167.9835; 24.9493; -167.9825; 24.9496; -167.9668; 24.9549; -167.9586; 24.9614; -167.9537; 24.9644; -167.949; 24.9736; -167.9473; 24.9814; -167.9467; 24.9829; -167.9442; 24.9898; -167.9446; 25; -167.9449; 25; -167.946; 25; -167.9463; 25; -167.9479; 25.0095; -167.9499; 25.0157; -167.9524; 25.0235; -167.962; 25.0332; -167.9725; 25.0412; -167.9847; 25.047; -167.9889; 25.049; -168; 25.0522; -168; 25.0503; -168.0017; 25.0502; -168.0064; 25.05; -168.0085; 25.0499; -168.0097; 25.0498; -168.0132; 25.0492; -168.016; 25.0486; -168.0222; 25.0467; -168.027; 25.0448; -168.03; 25.0431; -168.0355; 25.04; -168.0421; 25.0354; -168.0466; 25.0313; -168.0506; 25.0259; -168.0526; 25.0213; -168.0547; 25.0153; -168.0562; 25.0105; -168.0572; 25.0059; -168.058; 25.0026; -168.0582; 25; -168.0584; 24.9879; -166.3865; 23.8464; -166.3845; 23.832; -166.3829; 23.8297; -166.3788; 23.8236; -166.375; 23.8216; -166.375; 23.8222; -166.375; 23.824; -166.375; 23.8246; -166.3692; 23.8155; -166.3573; 23.8066; -166.3563; 23.8059; -166.3368; 23.7996; -166.3226; 23.7991; -166.3136; 23.8037; -166.3192; 23.791; -166.323; 23.7744; -166.3237; 23.771; -166.3202; 23.7585; -166.3167; 23.75; -166.3173; 23.75; -166.3191; 23.75; -166.3197; 23.75; -166.3158; 23.7401; -166.3111; 23.736; -166.3026; 23.7287; -166.286; 23.7181; -166.2668; 23.7134; -166.2656; 23.7131; -166.25; 23.7139; -166.25; 23.7148; -166.25; 23.7173; -166.25; 23.7182; -166.2412; 23.7197; -166.2315; 23.7236; -166.2268; 23.7274; -166.2262; 23.7235; -166.2249; 23.7152; -166.2228; 23.7049; -166.2148; 23.6967; -166.2054; 23.6916; -166.212; 23.6855; -166.224; 23.6725; -166.2299; 23.6544; -166.2302; 23.6526; -166.2323; 23.6416; -166.2288; 23.6318; -166.2248; 23.625; -166.2256; 23.625; -166.2281; 23.625; -166.2289; 23.625; -166.2242; 23.6148; -166.2149; 23.6042; -166.2111; 23.5998; -166.1944; 23.5895; -166.1722; 23.5871; -166.1512; 23.5905; -166.1452; 23.5942; -166.1313; 23.603; -166.125; 23.6093; -166.125; 23.6088; -166.125; 23.6075; -166.125; 23.6071; -166.1214; 23.6088; -166.1206; 23.6093; -166.1168; 23.6113; -166.1126; 23.6166; -166.1118; 23.6202; -166.1107; 23.625; -166.112; 23.625; -166.1158; 23.625; -166.1171; 23.625; -166.1139; 23.6346; -166.1131; 23.637; -166.1138; 23.6523; -166.1175; 23.6641; -166.1177; 23.6646; -166.125; 23.6707; -166.125; 23.6714; -166.125; 23.6734; -166.125; 23.6741; -166.1279; 23.6776; -166.1307; 23.681; -166.133; 23.6847; -166.1288; 23.6876; -166.125; 23.6901; -166.125; 23.6893; -166.125; 23.6869; -166.125; 23.6861; -166.1145; 23.6962; -166.1135; 23.6971; -166.1059; 23.7135; -166.1046; 23.7289; -166.106; 23.7379; -166.1068; 23.7425; -166.1133; 23.75; -166.1135; 23.75; -166.1143; 23.75; -166.1146; 23.75; -166.1167; 23.7542; -166.1166; 23.7548; -166.1165; 23.7574; -166.1169; 23.7617; -166.1185; 23.7667; -166.1212; 23.7692; -166.125; 23.7729; -166.125; 23.7715; -166.125; 23.7675; -166.125; 23.7661; -166.1294; 23.7702; -166.1368; 23.7785; -166.1426; 23.7844; -166.143; 23.7845; -166.1482; 23.7855; -166.1502; 23.7997; -166.1535; 23.8189; -166.1649; 23.8354; -166.1697; 23.8374; -166.1683; 23.8401; -166.1653; 23.8496; -166.1648; 23.851; -166.1655; 23.8648; -166.1683; 23.875; -166.1678; 23.875; -166.1664; 23.875; -166.1659; 23.875; -166.1704; 23.8885; -166.1752; 23.894; -166.1823; 23.9023; -166.2043; 23.9172; -166.2293; 23.927; -166.2331; 23.9285; -166.25; 23.9324; -166.25; 23.9289; -166.2647; 23.9285; -166.2785; 23.9259; -166.288; 23.9242; -166.2884; 23.929; -166.3071; 23.9249; -166.3247; 23.918; -166.3301; 23.9083; -166.3514; 23.9029; -166.352; 23.9025; -166.3656; 23.8942; -166.375; 23.8854; -166.375; 23.886; -166.375; 23.8877; -166.375; 23.8883; -166.3776; 23.8862; -166.3805; 23.884; -166.3822; 23.8782; -166.3822; 23.8781; -166.3833; 23.875; -166.3819; 23.875; -166.384; 23.8656; -166.3843; 23.8637; -166.3865; 23.8464; -164.7649; 23.575; -164.7647; 23.5664; -164.7626; 23.5585; -164.7591; 23.5527; -164.7576; 23.5502; -164.7531; 23.5453; -164.75; 23.5411; -164.75; 23.5401; -164.75; 23.5371; -164.75; 23.5361; -164.7394; 23.5302; -164.723; 23.5218; -164.7013; 23.517; -164.6963; 23.517; -164.6852; 23.5171; -164.6733; 23.5211; -164.6639; 23.527; -164.654; 23.5352; -164.6453; 23.5515; -164.64; 23.5761; -164.6446; 23.5945; -164.6541; 23.6071; -164.6688; 23.6166; -164.6826; 23.6228; -164.6889; 23.6234; -164.6974; 23.6233; -164.7023; 23.6233; -164.7098; 23.6232; -164.7246; 23.6211; -164.7401; 23.6144; -164.75; 23.6051; -164.7538; 23.6035; -164.7555; 23.6017; -164.7581; 23.599; -164.7603; 23.5951; -164.7612; 23.5935; -164.7635; 23.5867; -164.7648; 23.5817; -164.7649; 23.575; -161.9876; 23.0699; -161.9872; 23.0567; -161.9854; 23.0411; -161.9761; 23.0256; -161.9552; 23.0092; -161.9319; 23.0053; -161.9311; 23.0054; -161.8942; 23.0094; -161.875; 23.0201; -161.875; 23.0199; -161.875; 23.0194; -161.875; 23.0192; -161.8714; 23.0235; -161.8686; 23.0277; -161.8665; 23.0328; -161.8655; 23.034; -161.8633; 23.0366; -161.8608; 23.0444; -161.8589; 23.0526; -161.8581; 23.0608; -161.8589; 23.0681; -161.86; 23.0757; -161.863; 23.0851; -161.863; 23.0852; -161.8677; 23.0911; -161.8704; 23.0954; -161.8736; 23.0969; -161.875; 23.0975; -161.875; 23.0984; -161.875; 23.1008; -161.875; 23.1016; -161.8876; 23.1104; -161.9194; 23.114; -161.9311; 23.113; -161.9447; 23.1119; -161.9654; 23.105; -161.9825; 23.0913; -161.9876; 23.0699; -158.3447; 21.5777; -158.3441; 21.5698; -158.3422; 21.5643; -158.3401; 21.5611; -158.3396; 21.5603; -158.3351; 21.554; -158.3287; 21.546; -158.3176; 21.5391; -158.3173; 21.5389; -158.2987; 21.5247; -158.3001; 21.5097; -158.301; 21.5; -158.3012; 21.4984; -158.3014; 21.4968; -158.2933; 21.4968; -158.2902; 21.4968; -158.2915; 21.4894; -158.2906; 21.4794; -158.2905; 21.4784; -158.2903; 21.476; -158.2901; 21.4756; -158.2898; 21.4747; -158.2879; 21.4702; -158.2859; 21.4652; -158.2814; 21.4572; -158.2813; 21.457; -158.2786; 21.4529; -158.2764; 21.4496; -158.2762; 21.4493; -158.275; 21.4482; -158.2683; 21.442; -158.268; 21.4414; -158.2662; 21.4379; -158.2638; 21.433; -158.2637; 21.433; -158.2576; 21.4255; -158.2529; 21.4223; -158.252; 21.4217; -158.249; 21.4197; -158.2473; 21.419; -158.2465; 21.4165; -158.2458; 21.4145; -158.2414; 21.4122; -158.2401; 21.4115; -158.24; 21.4114; -158.2397; 21.4097; -158.2388; 21.4049; -158.2386; 21.4032; -158.2371; 21.3977; -158.2356; 21.3894; -158.2352; 21.3887; -158.2319; 21.3811; -158.2289; 21.3756; -158.2283; 21.375; -158.2222; 21.3682; -158.2178; 21.3645; -158.2126; 21.3618; -158.2066; 21.359; -158.2045; 21.3583; -158.2014; 21.3572; -158.1933; 21.3544; -158.1902; 21.3538; -158.1888; 21.3535; -158.1887; 21.3535; -158.1886; 21.3534; -158.1886; 21.3533; -158.187; 21.3511; -158.1833; 21.3459; -158.1827; 21.344; -158.182; 21.3412; -158.1768; 21.3208; -158.1644; 21.2723; -158.1612; 21.2674; -158.1596; 21.2634; -158.1576; 21.2611; -158.1541; 21.2566; -158.15; 21.2525; -158.1493; 21.2517; -158.1468; 21.25; -158.1445; 21.2484; -158.1423; 21.2468; -158.1421; 21.2468; -158.1348; 21.2424; -158.1223; 21.2386; -158.1101; 21.2371; -158.0916; 21.2379; -158.0849; 21.2393; -158.0769; 21.241; -158.0725; 21.2419; -158.0598; 21.2413; -158.0526; 21.2421; -158.0492; 21.2425; -158.0444; 21.2429; -158.039; 21.2432; -158.0326; 21.2445; -158.0281; 21.2468; -158.0272; 21.2478; -158.0257; 21.2483; -158.0241; 21.2485; -158.022; 21.2487; -158.0191; 21.2487; -158.0183; 21.2487; -158.0134; 21.2492; -158.0094; 21.2492; -158.0045; 21.2492; -158.0044; 21.2492; -158.0001; 21.2496; -157.9995; 21.2496; -157.997; 21.2496; -157.9956; 21.2496; -157.9929; 21.25; -157.9919; 21.2501; -157.9907; 21.25; -157.9898; 21.2499; -157.9878; 21.2496; -157.9873; 21.2497; -157.9866; 21.2499; -157.9859; 21.25; -157.9852; 21.2501; -157.9844; 21.2501; -157.9834; 21.2501; -157.98; 21.2507; -157.9768; 21.2514; -157.9756; 21.2517; -157.9744; 21.252; -157.9727; 21.2526; -157.9723; 21.2527; -157.9707; 21.2533; -157.9707; 21.2533; -157.9683; 21.2543; -157.9667; 21.2553; -157.9653; 21.2565; -157.9652; 21.2565; -157.9636; 21.2577; -157.9614; 21.257; -157.9588; 21.256; -157.9566; 21.2556; -157.9534; 21.2546; -157.9527; 21.2546; -157.9471; 21.2538; -157.942; 21.253; -157.9395; 21.2513; -157.9368; 21.25; -157.9367; 21.2499; -157.9337; 21.2488; -157.9315; 21.2483; -157.9279; 21.248; -157.9251; 21.2478; -157.9225; 21.2478; -157.9201; 21.2473; -157.9199; 21.2472; -157.9174; 21.2475; -157.9156; 21.2475; -157.9135; 21.2475; -157.9118; 21.2478; -157.91; 21.2478; -157.9088; 21.2478; -157.9079; 21.2478; -157.9053; 21.248; -157.9036; 21.2483; -157.9019; 21.2488; -157.9002; 21.2496; -157.8987; 21.2499; -157.898; 21.2488; -157.896; 21.2468; -157.8948; 21.2468; -157.8896; 21.2446; -157.8861; 21.2432; -157.8813; 21.2394; -157.8749; 21.2305; -157.8737; 21.2288; -157.8723; 21.2283; -157.8697; 21.2249; -157.869; 21.2239; -157.8666; 21.2208; -157.8658; 21.2197; -157.8656; 21.2194; -157.8641; 21.218; -157.8591; 21.2131; -157.8589; 21.2131; -157.8568; 21.212; -157.8545; 21.2109; -157.851; 21.2091; -157.8477; 21.2078; -157.8453; 21.207; -157.8387; 21.2045; -157.8291; 21.2009; -157.8281; 21.2008; -157.8213; 21.2002; -157.812; 21.1994; -157.8102; 21.1992; -157.8079; 21.1995; -157.7955; 21.2011; -157.7914; 21.2016; -157.7909; 21.2017; -157.7883; 21.2025; -157.779; 21.2054; -157.776; 21.2064; -157.7746; 21.2068; -157.7714; 21.2078; -157.7705; 21.2083; -157.7693; 21.2091; -157.7683; 21.2096; -157.7654; 21.2113; -157.7644; 21.2119; -157.7636; 21.2124; -157.761; 21.2139; -157.7601; 21.2144; -157.758; 21.2156; -157.7555; 21.2176; -157.7533; 21.2194; -157.7508; 21.22; -157.7473; 21.2209; -157.7453; 21.2217; -157.7411; 21.2179; -157.74; 21.2169; -157.7363; 21.2151; -157.7338; 21.2139; -157.7309; 21.2125; -157.7259; 21.2111; -157.7232; 21.2104; -157.7204; 21.2097; -157.7197; 21.2095; -157.7116; 21.2086; -157.7087; 21.2082; -157.7083; 21.2082; -157.6926; 21.209; -157.6894; 21.2092; -157.6758; 21.2138; -157.6651; 21.2199; -157.6535; 21.2291; -157.6513; 21.232; -157.6481; 21.2362; -157.6459; 21.2406; -157.6405; 21.2433; -157.6389; 21.2441; -157.6341; 21.2468; -157.632; 21.2485; -157.6242; 21.254; -157.6223; 21.2553; -157.6161; 21.2604; -157.6147; 21.2619; -157.6077; 21.2691; -157.6009; 21.2829; -157.6; 21.2866; -157.5979; 21.2951; -157.5973; 21.3107; -157.5976; 21.3138; -157.598; 21.3185; -157.5987; 21.3261; -157.6002; 21.3324; -157.6012; 21.3369; -157.6014; 21.3376; -157.6018; 21.3395; -157.602; 21.3402; -157.6022; 21.3411; -157.6023; 21.3415; -157.6035; 21.3438; -157.6039; 21.3446; -157.6047; 21.3462; -157.6071; 21.3508; -157.6079; 21.3524; -157.6082; 21.3531; -157.6153; 21.3616; -157.6201; 21.3677; -157.6223; 21.3718; -157.6223; 21.3727; -157.6254; 21.3746; -157.626; 21.375; -157.6285; 21.3766; -157.6285; 21.3814; -157.6293; 21.3852; -157.6312; 21.3883; -157.6324; 21.39; -157.6324; 21.3915; -157.6324; 21.3929; -157.6332; 21.3976; -157.6342; 21.4022; -157.6347; 21.4044; -157.6351; 21.4057; -157.6358; 21.4078; -157.6363; 21.4091; -157.6378; 21.4139; -157.6378; 21.414; -157.6382; 21.4161; -157.6386; 21.4178; -157.6409; 21.4226; -157.6409; 21.4228; -157.6425; 21.4264; -157.6456; 21.4302; -157.6464; 21.4313; -157.6486; 21.4341; -157.65; 21.4361; -157.6522; 21.4391; -157.65; 21.4418; -157.6496; 21.4423; -157.6495; 21.4424; -157.6474; 21.4455; -157.6455; 21.4487; -157.6433; 21.4538; -157.6418; 21.4582; -157.6407; 21.4627; -157.6412; 21.4672; -157.6428; 21.4723; -157.6454; 21.4768; -157.6477; 21.4805; -157.6485; 21.4819; -157.65; 21.4842; -157.6505; 21.4851; -157.6536; 21.4889; -157.6557; 21.4919; -157.6557; 21.4921; -157.6567; 21.4929; -157.6588; 21.4947; -157.6599; 21.4958; -157.6609; 21.4968; -157.673; 21.5; -157.6778; 21.5019; -157.6835; 21.5078; -157.6927; 21.5135; -157.7026; 21.5187; -157.7065; 21.5196; -157.7122; 21.5208; -157.7126; 21.5208; -157.7277; 21.5198; -157.7411; 21.5174; -157.7473; 21.5153; -157.7509; 21.5165; -157.7619; 21.5264; -157.765; 21.5293; -157.7683; 21.5324; -157.7737; 21.5373; -157.7744; 21.538; -157.775; 21.5386; -157.7762; 21.5397; -157.7774; 21.541; -157.7774; 21.541; -157.7776; 21.5411; -157.7776; 21.5412; -157.7786; 21.5421; -157.78; 21.5436; -157.781; 21.5446; -157.783; 21.5488; -157.7844; 21.5518; -157.7848; 21.5525; -157.7863; 21.5555; -157.7868; 21.5562; -157.7881; 21.5582; -157.7884; 21.5585; -157.7886; 21.5589; -157.7902; 21.5615; -157.7912; 21.5646; -157.7917; 21.5654; -157.7933; 21.5682; -157.7937; 21.5719; -157.7952; 21.5761; -157.7971; 21.581; -157.7986; 21.5852; -157.7991; 21.5859; -157.802; 21.5901; -157.8035; 21.5916; -157.8043; 21.5924; -157.8049; 21.5931; -157.8066; 21.5945; -157.8074; 21.5952; -157.8082; 21.5959; -157.8098; 21.5973; -157.8106; 21.5978; -157.8116; 21.5983; -157.8142; 21.5998; -157.817; 21.6021; -157.8186; 21.6034; -157.8245; 21.6071; -157.8319; 21.6113; -157.8341; 21.6124; -157.8343; 21.6125; -157.8372; 21.6137; -157.8394; 21.6162; -157.8403; 21.6173; -157.8432; 21.6207; -157.8441; 21.6218; -157.8474; 21.6314; -157.8515; 21.6427; -157.8538; 21.6492; -157.8542; 21.6503; -157.8602; 21.6655; -157.8617; 21.6681; -157.865; 21.6741; -157.8655; 21.675; -157.8664; 21.6765; -157.8708; 21.6835; -157.8722; 21.6859; -157.8763; 21.6962; -157.8768; 21.697; -157.8814; 21.7052; -157.8847; 21.7079; -157.8881; 21.71; -157.8914; 21.7121; -157.8942; 21.7148; -157.8964; 21.7183; -157.8981; 21.721; -157.9; 21.7227; -157.9004; 21.7231; -157.9004; 21.7231; -157.9053; 21.7255; -157.9092; 21.728; -157.9105; 21.7293; -157.9139; 21.7329; -157.9219; 21.7414; -157.9242; 21.7435; -157.9279; 21.746; -157.9302; 21.7468; -157.9316; 21.7482; -157.9418; 21.7546; -157.9551; 21.7586; -157.9783; 21.763; -157.9917; 21.763; -157.9972; 21.7616; -158.0082; 21.7553; -158.024; 21.7468; -158.0251; 21.7462; -158.0309; 21.7431; -158.0353; 21.7431; -158.0405; 21.742; -158.0449; 21.7409; -158.0501; 21.7399; -158.0571; 21.7355; -158.0623; 21.7301; -158.0676; 21.7247; -158.0719; 21.7192; -158.0789; 21.716; -158.0818; 21.7139; -158.0833; 21.7127; -158.0885; 21.7095; -158.0886; 21.7095; -158.0955; 21.703; -158.0998; 21.6975; -158.1033; 21.6921; -158.104; 21.6909; -158.1068; 21.6856; -158.1078; 21.6838; -158.1089; 21.6819; -158.1103; 21.6791; -158.1116; 21.6759; -158.1124; 21.6739; -158.1127; 21.6731; -158.1129; 21.6726; -158.1135; 21.6708; -158.1138; 21.67; -158.1143; 21.6687; -158.1147; 21.6672; -158.1165; 21.665; -158.1173; 21.6639; -158.1182; 21.6623; -158.119; 21.6607; -158.1202; 21.6573; -158.1206; 21.6638; -158.1213; 21.6646; -158.1222; 21.6657; -158.1261; 21.6635; -158.1281; 21.6625; -158.1283; 21.6623; -158.1334; 21.6586; -158.1342; 21.658; -158.1351; 21.6571; -158.1392; 21.6532; -158.1445; 21.6469; -158.1488; 21.642; -158.1555; 21.6397; -158.1665; 21.636; -158.175; 21.632; -158.187; 21.6326; -158.1996; 21.6345; -158.215; 21.6331; -158.2302; 21.6308; -158.2472; 21.6311; -158.2677; 21.6281; -158.2782; 21.6278; -158.2896; 21.6254; -158.3019; 21.6218; -158.3097; 21.6218; -158.3119; 21.6218; -158.3197; 21.6173; -158.3242; 21.6157; -158.3277; 21.6118; -158.3299; 21.6094; -158.335; 21.6046; -158.3395; 21.5967; -158.3421; 21.5912; -158.3447; 21.5832; -158.3447; 21.5777</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Wetland</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>simple_group</t>
-        </is>
-      </c>
-      <c r="Q25">
-        <v>1</v>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>96dc0855-1faa-4b76-b276-825d9bc6a8fe</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
-        </is>
-      </c>
-      <c r="C26">
-        <v>10</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Range shifts of montane mammals under projected warming in the Andes</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Gutierrez MJ; Blanco VF; Quispe RR</t>
-        </is>
-      </c>
-      <c r="F26">
-        <v>2020</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>10.1111/geb.13094</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>reviewed</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>564c9186-f70d-47f2-b285-55baee74f705</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>2026-02-28T09:29:11+00:00</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Honolulu County, Hawaii, United States; 21.4682; -157.9605; 3861844; MultiPolygon; -178.4436; 28.419; -178.4405; 28.4052; -178.4332; 28.3978; -178.4159; 28.3801; -178.4137; 28.375; -178.4141; 28.375; -178.4153; 28.375; -178.4157; 28.375; -178.4123; 28.3633; -178.4115; 28.3607; -178.3956; 28.3419; -178.3867; 28.3391; -178.375; 28.3354; -178.375; 28.3358; -178.375; 28.3371; -178.375; 28.3375; -178.3489; 28.3347; -178.3417; 28.3339; -178.3014; 28.3283; -178.2889; 28.3288; -178.2719; 28.3353; -178.2703; 28.3359; -178.2575; 28.3428; -178.25; 28.3494; -178.25; 28.349; -178.25; 28.3476; -178.25; 28.3472; -178.2461; 28.3524; -178.2389; 28.362; -178.2357; 28.369; -178.233; 28.375; -178.2338; 28.375; -178.2363; 28.375; -178.2371; 28.375; -178.2325; 28.3836; -178.2311; 28.3937; -178.2305; 28.3977; -178.2322; 28.4273; -178.2378; 28.4529; -178.2385; 28.4562; -178.25; 28.4682; -178.25; 28.4679; -178.25; 28.467; -178.25; 28.4667; -178.256; 28.4751; -178.257; 28.4765; -178.2712; 28.4886; -178.2801; 28.4944; -178.2888; 28.5; -178.2873; 28.5; -178.2826; 28.5; -178.2811; 28.5; -178.2915; 28.5072; -178.2979; 28.5102; -178.3043; 28.5133; -178.3151; 28.5163; -178.3337; 28.5172; -178.3405; 28.5173; -178.3558; 28.5146; -178.3606; 28.5138; -178.375; 28.5101; -178.375; 28.5096; -178.375; 28.5083; -178.375; 28.5078; -178.3773; 28.5063; -178.3813; 28.5036; -178.3842; 28.5016; -178.3864; 28.5; -178.3883; 28.5; -178.3939; 28.5; -178.3958; 28.5; -178.4118; 28.4837; -178.4168; 28.4782; -178.4276; 28.4661; -178.4383; 28.4441; -178.4436; 28.419; -176.0434; 27.7959; -176.0429; 27.7784; -176.0396; 27.7582; -176.0344; 27.75; -176.0293; 27.7427; -176.0249; 27.738; -176.0235; 27.7367; -176.0055; 27.7203; -176; 27.7161; -176; 27.7147; -176; 27.7107; -176; 27.7093; -175.9763; 27.6969; -175.9696; 27.6934; -175.9395; 27.6882; -175.8988; 27.6983; -175.8952; 27.6992; -175.875; 27.7102; -175.875; 27.7098; -175.875; 27.7088; -175.875; 27.7084; -175.8649; 27.7145; -175.845; 27.7285; -175.8175; 27.723; -175.8029; 27.7235; -175.7791; 27.7257; -175.75; 27.7333; -175.75; 27.7323; -175.7461; 27.7327; -175.7341; 27.7389; -175.7262; 27.75; -175.7248; 27.7526; -175.6784; 27.8432; -175.6766; 27.8468; -175.6665; 27.875; -175.6663; 27.875; -175.6658; 27.875; -175.6656; 27.875; -175.6641; 27.8941; -175.6645; 27.9061; -175.6648; 27.9144; -175.6701; 27.9416; -175.6815; 27.9586; -175.7044; 27.9827; -175.7078; 27.9847; -175.7349; 28; -175.736; 28; -175.739; 28; -175.74; 28; -175.7411; 28.0003; -175.7444; 28.001; -175.7445; 28.001; -175.7455; 28.0013; -175.7457; 28.0014; -175.7463; 28.0016; -175.7466; 28.0016; -175.75; 28.003; -175.7544; 28.004; -175.7697; 28.0075; -175.7786; 28.0081; -175.7863; 28.0086; -175.7868; 28.0086; -175.7999; 28.0082; -175.806; 28.0073; -175.8067; 28.0072; -175.8101; 28.0059; -175.8174; 28.0022; -175.8231; 28; -175.8579; 27.9821; -175.875; 27.9733; -175.875; 27.9738; -175.875; 27.9754; -175.875; 27.9759; -175.9044; 27.9606; -175.9088; 27.9583; -175.9357; 27.9406; -175.9505; 27.9362; -175.9663; 27.9299; -175.9814; 27.9132; -175.9847; 27.9065; -175.9876; 27.9005; -175.9921; 27.8895; -175.9938; 27.875; -175.9931; 27.875; -175.9913; 27.875; -175.9907; 27.875; -175.9889; 27.8619; -175.9782; 27.848; -175.9735; 27.8449; -175.9558; 27.8331; -175.9395; 27.8275; -175.9254; 27.8234; -175.921; 27.8214; -175.9243; 27.8137; -175.9325; 27.8145; -175.9388; 27.8186; -175.9645; 27.827; -175.9746; 27.8302; -175.9832; 27.8314; -175.9907; 27.8326; -176; 27.8305; -176; 27.8315; -176; 27.8344; -176; 27.8353; -176.0062; 27.8326; -176.0108; 27.8303; -176.025; 27.8216; -176.0268; 27.8195; -176.0287; 27.8173; -176.0366; 27.8071; -176.0426; 27.7981; -176.0434; 27.7959; -174.0675; 26.0525; -174.0659; 26.0394; -174.0599; 26.0227; -174.0592; 26.0207; -174.0461; 26.0023; -174.0431; 26; -174.042; 26; -174.0387; 26; -174.0375; 26; -174.0309; 25.9957; -174.0272; 25.9933; -174.0079; 25.9905; -174.0064; 25.9903; -174; 25.9902; -174; 25.9907; -174; 25.9923; -174; 25.9929; -173.9959; 25.994; -173.9918; 25.9951; -173.9845; 25.9976; -173.984; 25.9979; -173.9803; 26; -173.9796; 26; -173.9777; 26; -173.977; 26; -173.9649; 26.0066; -173.9431; 26.0107; -173.9428; 26.0107; -173.926; 26.0196; -173.9131; 26.036; -173.9034; 26.0601; -173.9038; 26.0668; -173.9085; 26.0819; -173.9134; 26.0994; -173.914; 26.1005; -173.9186; 26.1097; -173.926; 26.1172; -173.9291; 26.1201; -173.9389; 26.125; -173.9361; 26.125; -173.9503; 26.1332; -173.9579; 26.1357; -173.9696; 26.1354; -173.9814; 26.1332; -173.9919; 26.1366; -174; 26.1369; -174; 26.1355; -174.0007; 26.1357; -174.0028; 26.1363; -174.0035; 26.1365; -174.0071; 26.1371; -174.0109; 26.1366; -174.011; 26.1366; -174.0189; 26.134; -174.0311; 26.1291; -174.0318; 26.1287; -174.0383; 26.125; -174.0379; 26.125; -174.037; 26.125; -174.0366; 26.125; -174.0407; 26.1226; -174.0496; 26.1166; -174.0525; 26.113; -174.0548; 26.1077; -174.0556; 26.1053; -174.0591; 26.0942; -174.0615; 26.082; -174.0674; 26.0596; -174.0675; 26.0525; -171.8096; 25.7813; -171.8081; 25.7729; -171.807; 25.7671; -171.8004; 25.75; -171.8006; 25.75; -171.797; 25.7405; -171.7947; 25.7386; -171.7829; 25.7283; -171.7702; 25.7182; -171.7626; 25.7148; -171.7553; 25.7115; -171.75; 25.7103; -171.75; 25.7101; -171.75; 25.7094; -171.75; 25.7092; -171.7375; 25.7065; -171.7314; 25.7075; -171.7184; 25.7095; -171.6998; 25.7169; -171.6869; 25.7279; -171.6829; 25.7333; -171.6805; 25.7368; -171.6777; 25.75; -171.669; 25.7777; -171.6679; 25.7812; -171.6694; 25.7939; -171.6766; 25.8109; -171.6883; 25.8238; -171.7106; 25.8332; -171.7211; 25.8339; -171.7315; 25.8346; -171.75; 25.8379; -171.7681; 25.8337; -171.7719; 25.8314; -171.7729; 25.8308; -171.787; 25.8223; -171.8001; 25.8058; -171.8065; 25.7934; -171.8096; 25.7813; -170.6849; 25.5064; -170.6848; 25.5048; -170.6847; 25.5031; -170.6846; 25.5014; -170.6843; 25.4998; -170.6841; 25.4981; -170.6837; 25.4965; -170.6833; 25.4949; -170.6828; 25.4932; -170.6823; 25.4916; -170.6817; 25.4901; -170.6811; 25.4885; -170.6804; 25.4869; -170.6797; 25.4854; -170.6789; 25.4839; -170.6781; 25.4824; -170.6772; 25.4809; -170.6762; 25.4795; -170.6752; 25.4781; -170.6741; 25.4767; -170.673; 25.4754; -170.6719; 25.4741; -170.6707; 25.4729; -170.6694; 25.4716; -170.6681; 25.4704; -170.6674; 25.4698; -170.6663; 25.4689; -170.665; 25.4678; -170.6635; 25.4668; -170.6621; 25.4657; -170.6606; 25.4648; -170.6591; 25.4638; -170.6575; 25.4629; -170.6559; 25.4621; -170.6543; 25.4613; -170.6526; 25.4606; -170.6509; 25.4599; -170.6492; 25.4593; -170.6475; 25.4587; -170.6458; 25.4582; -170.644; 25.4577; -170.6422; 25.4573; -170.6404; 25.4569; -170.6386; 25.4566; -170.6368; 25.4563; -170.635; 25.4561; -170.6331; 25.456; -170.6313; 25.4559; -170.6295; 25.4558; -170.6276; 25.4558; -170.6258; 25.4559; -170.6239; 25.456; -170.6221; 25.4562; -170.6203; 25.4564; -170.6185; 25.4567; -170.6167; 25.4571; -170.6149; 25.4575; -170.6131; 25.4579; -170.6113; 25.4584; -170.6096; 25.459; -170.6079; 25.4596; -170.6062; 25.4602; -170.6045; 25.461; -170.6029; 25.4617; -170.6013; 25.4625; -170.5997; 25.4634; -170.5982; 25.4643; -170.5967; 25.4652; -170.5952; 25.4662; -170.5937; 25.4673; -170.5923; 25.4684; -170.591; 25.4695; -170.5897; 25.4706; -170.5884; 25.4719; -170.5871; 25.4731; -170.5859; 25.4744; -170.5848; 25.4757; -170.5837; 25.477; -170.5827; 25.4784; -170.5817; 25.4798; -170.5807; 25.4812; -170.5798; 25.4827; -170.579; 25.4842; -170.5782; 25.4857; -170.5775; 25.4872; -170.5768; 25.4888; -170.5762; 25.4904; -170.5757; 25.492; -170.5752; 25.4936; -170.5747; 25.4952; -170.5744; 25.4968; -170.5741; 25.4985; -170.5738; 25.5002; -170.5736; 25.5018; -170.5735; 25.5035; -170.5734; 25.5051; -170.5734; 25.5068; -170.5735; 25.5085; -170.5736; 25.5101; -170.5737; 25.5118; -170.574; 25.5135; -170.5743; 25.5151; -170.5746; 25.5168; -170.5751; 25.5184; -170.5755; 25.52; -170.5761; 25.5216; -170.5767; 25.5232; -170.5773; 25.5248; -170.578; 25.5263; -170.5787; 25.5278; -170.5795; 25.5293; -170.5804; 25.5308; -170.5813; 25.5323; -170.5823; 25.5337; -170.5833; 25.5351; -170.5844; 25.5364; -170.5855; 25.5378; -170.5866; 25.5391; -170.5879; 25.5403; -170.5891; 25.5415; -170.5904; 25.5427; -170.5917; 25.5439; -170.5931; 25.545; -170.5945; 25.5461; -170.596; 25.5471; -170.5975; 25.5481; -170.599; 25.549; -170.6005; 25.5499; -170.6021; 25.5507; -170.6038; 25.5515; -170.6054; 25.5523; -170.6071; 25.5529; -170.6088; 25.5536; -170.6105; 25.5542; -170.6122; 25.5547; -170.614; 25.5552; -170.6158; 25.5556; -170.6176; 25.556; -170.6194; 25.5563; -170.6212; 25.5566; -170.623; 25.5568; -170.6249; 25.557; -170.6267; 25.5571; -170.6285; 25.5571; -170.6304; 25.5571; -170.6322; 25.5571; -170.6341; 25.557; -170.6359; 25.5568; -170.6377; 25.5566; -170.6395; 25.5563; -170.6413; 25.556; -170.6431; 25.5556; -170.6449; 25.5551; -170.6467; 25.5546; -170.6484; 25.5541; -170.6501; 25.5535; -170.6518; 25.5528; -170.6535; 25.5522; -170.6551; 25.5514; -170.6567; 25.5506; -170.6583; 25.5497; -170.6599; 25.5489; -170.6614; 25.5479; -170.6629; 25.5469; -170.6644; 25.5459; -170.6658; 25.5448; -170.6671; 25.5437; -170.6685; 25.5425; -170.6697; 25.5413; -170.671; 25.5401; -170.6722; 25.5388; -170.6733; 25.5375; -170.6744; 25.5362; -170.6755; 25.5348; -170.6764; 25.5334; -170.6774; 25.532; -170.6783; 25.5305; -170.6791; 25.529; -170.6799; 25.5275; -170.6807; 25.526; -170.6813; 25.5244; -170.682; 25.5229; -170.6825; 25.5213; -170.683; 25.5197; -170.6835; 25.518; -170.6839; 25.5164; -170.6842; 25.5148; -170.6844; 25.5131; -170.6846; 25.5114; -170.6848; 25.5098; -170.6849; 25.5081; -170.6849; 25.5064; -168.0584; 24.9879; -168.0503; 24.9745; -168.0378; 24.9597; -168.0236; 24.9545; -168; 24.9507; -168; 24.9502; -168; 24.9486; -168; 24.9481; -167.9835; 24.9493; -167.9825; 24.9496; -167.9668; 24.9549; -167.9586; 24.9614; -167.9537; 24.9644; -167.949; 24.9736; -167.9473; 24.9814; -167.9467; 24.9829; -167.9442; 24.9898; -167.9446; 25; -167.9449; 25; -167.946; 25; -167.9463; 25; -167.9479; 25.0095; -167.9499; 25.0157; -167.9524; 25.0235; -167.962; 25.0332; -167.9725; 25.0412; -167.9847; 25.047; -167.9889; 25.049; -168; 25.0522; -168; 25.0503; -168.0017; 25.0502; -168.0064; 25.05; -168.0085; 25.0499; -168.0097; 25.0498; -168.0132; 25.0492; -168.016; 25.0486; -168.0222; 25.0467; -168.027; 25.0448; -168.03; 25.0431; -168.0355; 25.04; -168.0421; 25.0354; -168.0466; 25.0313; -168.0506; 25.0259; -168.0526; 25.0213; -168.0547; 25.0153; -168.0562; 25.0105; -168.0572; 25.0059; -168.058; 25.0026; -168.0582; 25; -168.0584; 24.9879; -166.3865; 23.8464; -166.3845; 23.832; -166.3829; 23.8297; -166.3788; 23.8236; -166.375; 23.8216; -166.375; 23.8222; -166.375; 23.824; -166.375; 23.8246; -166.3692; 23.8155; -166.3573; 23.8066; -166.3563; 23.8059; -166.3368; 23.7996; -166.3226; 23.7991; -166.3136; 23.8037; -166.3192; 23.791; -166.323; 23.7744; -166.3237; 23.771; -166.3202; 23.7585; -166.3167; 23.75; -166.3173; 23.75; -166.3191; 23.75; -166.3197; 23.75; -166.3158; 23.7401; -166.3111; 23.736; -166.3026; 23.7287; -166.286; 23.7181; -166.2668; 23.7134; -166.2656; 23.7131; -166.25; 23.7139; -166.25; 23.7148; -166.25; 23.7173; -166.25; 23.7182; -166.2412; 23.7197; -166.2315; 23.7236; -166.2268; 23.7274; -166.2262; 23.7235; -166.2249; 23.7152; -166.2228; 23.7049; -166.2148; 23.6967; -166.2054; 23.6916; -166.212; 23.6855; -166.224; 23.6725; -166.2299; 23.6544; -166.2302; 23.6526; -166.2323; 23.6416; -166.2288; 23.6318; -166.2248; 23.625; -166.2256; 23.625; -166.2281; 23.625; -166.2289; 23.625; -166.2242; 23.6148; -166.2149; 23.6042; -166.2111; 23.5998; -166.1944; 23.5895; -166.1722; 23.5871; -166.1512; 23.5905; -166.1452; 23.5942; -166.1313; 23.603; -166.125; 23.6093; -166.125; 23.6088; -166.125; 23.6075; -166.125; 23.6071; -166.1214; 23.6088; -166.1206; 23.6093; -166.1168; 23.6113; -166.1126; 23.6166; -166.1118; 23.6202; -166.1107; 23.625; -166.112; 23.625; -166.1158; 23.625; -166.1171; 23.625; -166.1139; 23.6346; -166.1131; 23.637; -166.1138; 23.6523; -166.1175; 23.6641; -166.1177; 23.6646; -166.125; 23.6707; -166.125; 23.6714; -166.125; 23.6734; -166.125; 23.6741; -166.1279; 23.6776; -166.1307; 23.681; -166.133; 23.6847; -166.1288; 23.6876; -166.125; 23.6901; -166.125; 23.6893; -166.125; 23.6869; -166.125; 23.6861; -166.1145; 23.6962; -166.1135; 23.6971; -166.1059; 23.7135; -166.1046; 23.7289; -166.106; 23.7379; -166.1068; 23.7425; -166.1133; 23.75; -166.1135; 23.75; -166.1143; 23.75; -166.1146; 23.75; -166.1167; 23.7542; -166.1166; 23.7548; -166.1165; 23.7574; -166.1169; 23.7617; -166.1185; 23.7667; -166.1212; 23.7692; -166.125; 23.7729; -166.125; 23.7715; -166.125; 23.7675; -166.125; 23.7661; -166.1294; 23.7702; -166.1368; 23.7785; -166.1426; 23.7844; -166.143; 23.7845; -166.1482; 23.7855; -166.1502; 23.7997; -166.1535; 23.8189; -166.1649; 23.8354; -166.1697; 23.8374; -166.1683; 23.8401; -166.1653; 23.8496; -166.1648; 23.851; -166.1655; 23.8648; -166.1683; 23.875; -166.1678; 23.875; -166.1664; 23.875; -166.1659; 23.875; -166.1704; 23.8885; -166.1752; 23.894; -166.1823; 23.9023; -166.2043; 23.9172; -166.2293; 23.927; -166.2331; 23.9285; -166.25; 23.9324; -166.25; 23.9289; -166.2647; 23.9285; -166.2785; 23.9259; -166.288; 23.9242; -166.2884; 23.929; -166.3071; 23.9249; -166.3247; 23.918; -166.3301; 23.9083; -166.3514; 23.9029; -166.352; 23.9025; -166.3656; 23.8942; -166.375; 23.8854; -166.375; 23.886; -166.375; 23.8877; -166.375; 23.8883; -166.3776; 23.8862; -166.3805; 23.884; -166.3822; 23.8782; -166.3822; 23.8781; -166.3833; 23.875; -166.3819; 23.875; -166.384; 23.8656; -166.3843; 23.8637; -166.3865; 23.8464; -164.7649; 23.575; -164.7647; 23.5664; -164.7626; 23.5585; -164.7591; 23.5527; -164.7576; 23.5502; -164.7531; 23.5453; -164.75; 23.5411; -164.75; 23.5401; -164.75; 23.5371; -164.75; 23.5361; -164.7394; 23.5302; -164.723; 23.5218; -164.7013; 23.517; -164.6963; 23.517; -164.6852; 23.5171; -164.6733; 23.5211; -164.6639; 23.527; -164.654; 23.5352; -164.6453; 23.5515; -164.64; 23.5761; -164.6446; 23.5945; -164.6541; 23.6071; -164.6688; 23.6166; -164.6826; 23.6228; -164.6889; 23.6234; -164.6974; 23.6233; -164.7023; 23.6233; -164.7098; 23.6232; -164.7246; 23.6211; -164.7401; 23.6144; -164.75; 23.6051; -164.7538; 23.6035; -164.7555; 23.6017; -164.7581; 23.599; -164.7603; 23.5951; -164.7612; 23.5935; -164.7635; 23.5867; -164.7648; 23.5817; -164.7649; 23.575; -161.9876; 23.0699; -161.9872; 23.0567; -161.9854; 23.0411; -161.9761; 23.0256; -161.9552; 23.0092; -161.9319; 23.0053; -161.9311; 23.0054; -161.8942; 23.0094; -161.875; 23.0201; -161.875; 23.0199; -161.875; 23.0194; -161.875; 23.0192; -161.8714; 23.0235; -161.8686; 23.0277; -161.8665; 23.0328; -161.8655; 23.034; -161.8633; 23.0366; -161.8608; 23.0444; -161.8589; 23.0526; -161.8581; 23.0608; -161.8589; 23.0681; -161.86; 23.0757; -161.863; 23.0851; -161.863; 23.0852; -161.8677; 23.0911; -161.8704; 23.0954; -161.8736; 23.0969; -161.875; 23.0975; -161.875; 23.0984; -161.875; 23.1008; -161.875; 23.1016; -161.8876; 23.1104; -161.9194; 23.114; -161.9311; 23.113; -161.9447; 23.1119; -161.9654; 23.105; -161.9825; 23.0913; -161.9876; 23.0699; -158.3447; 21.5777; -158.3441; 21.5698; -158.3422; 21.5643; -158.3401; 21.5611; -158.3396; 21.5603; -158.3351; 21.554; -158.3287; 21.546; -158.3176; 21.5391; -158.3173; 21.5389; -158.2987; 21.5247; -158.3001; 21.5097; -158.301; 21.5; -158.3012; 21.4984; -158.3014; 21.4968; -158.2933; 21.4968; -158.2902; 21.4968; -158.2915; 21.4894; -158.2906; 21.4794; -158.2905; 21.4784; -158.2903; 21.476; -158.2901; 21.4756; -158.2898; 21.4747; -158.2879; 21.4702; -158.2859; 21.4652; -158.2814; 21.4572; -158.2813; 21.457; -158.2786; 21.4529; -158.2764; 21.4496; -158.2762; 21.4493; -158.275; 21.4482; -158.2683; 21.442; -158.268; 21.4414; -158.2662; 21.4379; -158.2638; 21.433; -158.2637; 21.433; -158.2576; 21.4255; -158.2529; 21.4223; -158.252; 21.4217; -158.249; 21.4197; -158.2473; 21.419; -158.2465; 21.4165; -158.2458; 21.4145; -158.2414; 21.4122; -158.2401; 21.4115; -158.24; 21.4114; -158.2397; 21.4097; -158.2388; 21.4049; -158.2386; 21.4032; -158.2371; 21.3977; -158.2356; 21.3894; -158.2352; 21.3887; -158.2319; 21.3811; -158.2289; 21.3756; -158.2283; 21.375; -158.2222; 21.3682; -158.2178; 21.3645; -158.2126; 21.3618; -158.2066; 21.359; -158.2045; 21.3583; -158.2014; 21.3572; -158.1933; 21.3544; -158.1902; 21.3538; -158.1888; 21.3535; -158.1887; 21.3535; -158.1886; 21.3534; -158.1886; 21.3533; -158.187; 21.3511; -158.1833; 21.3459; -158.1827; 21.344; -158.182; 21.3412; -158.1768; 21.3208; -158.1644; 21.2723; -158.1612; 21.2674; -158.1596; 21.2634; -158.1576; 21.2611; -158.1541; 21.2566; -158.15; 21.2525; -158.1493; 21.2517; -158.1468; 21.25; -158.1445; 21.2484; -158.1423; 21.2468; -158.1421; 21.2468; -158.1348; 21.2424; -158.1223; 21.2386; -158.1101; 21.2371; -158.0916; 21.2379; -158.0849; 21.2393; -158.0769; 21.241; -158.0725; 21.2419; -158.0598; 21.2413; -158.0526; 21.2421; -158.0492; 21.2425; -158.0444; 21.2429; -158.039; 21.2432; -158.0326; 21.2445; -158.0281; 21.2468; -158.0272; 21.2478; -158.0257; 21.2483; -158.0241; 21.2485; -158.022; 21.2487; -158.0191; 21.2487; -158.0183; 21.2487; -158.0134; 21.2492; -158.0094; 21.2492; -158.0045; 21.2492; -158.0044; 21.2492; -158.0001; 21.2496; -157.9995; 21.2496; -157.997; 21.2496; -157.9956; 21.2496; -157.9929; 21.25; -157.9919; 21.2501; -157.9907; 21.25; -157.9898; 21.2499; -157.9878; 21.2496; -157.9873; 21.2497; -157.9866; 21.2499; -157.9859; 21.25; -157.9852; 21.2501; -157.9844; 21.2501; -157.9834; 21.2501; -157.98; 21.2507; -157.9768; 21.2514; -157.9756; 21.2517; -157.9744; 21.252; -157.9727; 21.2526; -157.9723; 21.2527; -157.9707; 21.2533; -157.9707; 21.2533; -157.9683; 21.2543; -157.9667; 21.2553; -157.9653; 21.2565; -157.9652; 21.2565; -157.9636; 21.2577; -157.9614; 21.257; -157.9588; 21.256; -157.9566; 21.2556; -157.9534; 21.2546; -157.9527; 21.2546; -157.9471; 21.2538; -157.942; 21.253; -157.9395; 21.2513; -157.9368; 21.25; -157.9367; 21.2499; -157.9337; 21.2488; -157.9315; 21.2483; -157.9279; 21.248; -157.9251; 21.2478; -157.9225; 21.2478; -157.9201; 21.2473; -157.9199; 21.2472; -157.9174; 21.2475; -157.9156; 21.2475; -157.9135; 21.2475; -157.9118; 21.2478; -157.91; 21.2478; -157.9088; 21.2478; -157.9079; 21.2478; -157.9053; 21.248; -157.9036; 21.2483; -157.9019; 21.2488; -157.9002; 21.2496; -157.8987; 21.2499; -157.898; 21.2488; -157.896; 21.2468; -157.8948; 21.2468; -157.8896; 21.2446; -157.8861; 21.2432; -157.8813; 21.2394; -157.8749; 21.2305; -157.8737; 21.2288; -157.8723; 21.2283; -157.8697; 21.2249; -157.869; 21.2239; -157.8666; 21.2208; -157.8658; 21.2197; -157.8656; 21.2194; -157.8641; 21.218; -157.8591; 21.2131; -157.8589; 21.2131; -157.8568; 21.212; -157.8545; 21.2109; -157.851; 21.2091; -157.8477; 21.2078; -157.8453; 21.207; -157.8387; 21.2045; -157.8291; 21.2009; -157.8281; 21.2008; -157.8213; 21.2002; -157.812; 21.1994; -157.8102; 21.1992; -157.8079; 21.1995; -157.7955; 21.2011; -157.7914; 21.2016; -157.7909; 21.2017; -157.7883; 21.2025; -157.779; 21.2054; -157.776; 21.2064; -157.7746; 21.2068; -157.7714; 21.2078; -157.7705; 21.2083; -157.7693; 21.2091; -157.7683; 21.2096; -157.7654; 21.2113; -157.7644; 21.2119; -157.7636; 21.2124; -157.761; 21.2139; -157.7601; 21.2144; -157.758; 21.2156; -157.7555; 21.2176; -157.7533; 21.2194; -157.7508; 21.22; -157.7473; 21.2209; -157.7453; 21.2217; -157.7411; 21.2179; -157.74; 21.2169; -157.7363; 21.2151; -157.7338; 21.2139; -157.7309; 21.2125; -157.7259; 21.2111; -157.7232; 21.2104; -157.7204; 21.2097; -157.7197; 21.2095; -157.7116; 21.2086; -157.7087; 21.2082; -157.7083; 21.2082; -157.6926; 21.209; -157.6894; 21.2092; -157.6758; 21.2138; -157.6651; 21.2199; -157.6535; 21.2291; -157.6513; 21.232; -157.6481; 21.2362; -157.6459; 21.2406; -157.6405; 21.2433; -157.6389; 21.2441; -157.6341; 21.2468; -157.632; 21.2485; -157.6242; 21.254; -157.6223; 21.2553; -157.6161; 21.2604; -157.6147; 21.2619; -157.6077; 21.2691; -157.6009; 21.2829; -157.6; 21.2866; -157.5979; 21.2951; -157.5973; 21.3107; -157.5976; 21.3138; -157.598; 21.3185; -157.5987; 21.3261; -157.6002; 21.3324; -157.6012; 21.3369; -157.6014; 21.3376; -157.6018; 21.3395; -157.602; 21.3402; -157.6022; 21.3411; -157.6023; 21.3415; -157.6035; 21.3438; -157.6039; 21.3446; -157.6047; 21.3462; -157.6071; 21.3508; -157.6079; 21.3524; -157.6082; 21.3531; -157.6153; 21.3616; -157.6201; 21.3677; -157.6223; 21.3718; -157.6223; 21.3727; -157.6254; 21.3746; -157.626; 21.375; -157.6285; 21.3766; -157.6285; 21.3814; -157.6293; 21.3852; -157.6312; 21.3883; -157.6324; 21.39; -157.6324; 21.3915; -157.6324; 21.3929; -157.6332; 21.3976; -157.6342; 21.4022; -157.6347; 21.4044; -157.6351; 21.4057; -157.6358; 21.4078; -157.6363; 21.4091; -157.6378; 21.4139; -157.6378; 21.414; -157.6382; 21.4161; -157.6386; 21.4178; -157.6409; 21.4226; -157.6409; 21.4228; -157.6425; 21.4264; -157.6456; 21.4302; -157.6464; 21.4313; -157.6486; 21.4341; -157.65; 21.4361; -157.6522; 21.4391; -157.65; 21.4418; -157.6496; 21.4423; -157.6495; 21.4424; -157.6474; 21.4455; -157.6455; 21.4487; -157.6433; 21.4538; -157.6418; 21.4582; -157.6407; 21.4627; -157.6412; 21.4672; -157.6428; 21.4723; -157.6454; 21.4768; -157.6477; 21.4805; -157.6485; 21.4819; -157.65; 21.4842; -157.6505; 21.4851; -157.6536; 21.4889; -157.6557; 21.4919; -157.6557; 21.4921; -157.6567; 21.4929; -157.6588; 21.4947; -157.6599; 21.4958; -157.6609; 21.4968; -157.673; 21.5; -157.6778; 21.5019; -157.6835; 21.5078; -157.6927; 21.5135; -157.7026; 21.5187; -157.7065; 21.5196; -157.7122; 21.5208; -157.7126; 21.5208; -157.7277; 21.5198; -157.7411; 21.5174; -157.7473; 21.5153; -157.7509; 21.5165; -157.7619; 21.5264; -157.765; 21.5293; -157.7683; 21.5324; -157.7737; 21.5373; -157.7744; 21.538; -157.775; 21.5386; -157.7762; 21.5397; -157.7774; 21.541; -157.7774; 21.541; -157.7776; 21.5411; -157.7776; 21.5412; -157.7786; 21.5421; -157.78; 21.5436; -157.781; 21.5446; -157.783; 21.5488; -157.7844; 21.5518; -157.7848; 21.5525; -157.7863; 21.5555; -157.7868; 21.5562; -157.7881; 21.5582; -157.7884; 21.5585; -157.7886; 21.5589; -157.7902; 21.5615; -157.7912; 21.5646; -157.7917; 21.5654; -157.7933; 21.5682; -157.7937; 21.5719; -157.7952; 21.5761; -157.7971; 21.581; -157.7986; 21.5852; -157.7991; 21.5859; -157.802; 21.5901; -157.8035; 21.5916; -157.8043; 21.5924; -157.8049; 21.5931; -157.8066; 21.5945; -157.8074; 21.5952; -157.8082; 21.5959; -157.8098; 21.5973; -157.8106; 21.5978; -157.8116; 21.5983; -157.8142; 21.5998; -157.817; 21.6021; -157.8186; 21.6034; -157.8245; 21.6071; -157.8319; 21.6113; -157.8341; 21.6124; -157.8343; 21.6125; -157.8372; 21.6137; -157.8394; 21.6162; -157.8403; 21.6173; -157.8432; 21.6207; -157.8441; 21.6218; -157.8474; 21.6314; -157.8515; 21.6427; -157.8538; 21.6492; -157.8542; 21.6503; -157.8602; 21.6655; -157.8617; 21.6681; -157.865; 21.6741; -157.8655; 21.675; -157.8664; 21.6765; -157.8708; 21.6835; -157.8722; 21.6859; -157.8763; 21.6962; -157.8768; 21.697; -157.8814; 21.7052; -157.8847; 21.7079; -157.8881; 21.71; -157.8914; 21.7121; -157.8942; 21.7148; -157.8964; 21.7183; -157.8981; 21.721; -157.9; 21.7227; -157.9004; 21.7231; -157.9004; 21.7231; -157.9053; 21.7255; -157.9092; 21.728; -157.9105; 21.7293; -157.9139; 21.7329; -157.9219; 21.7414; -157.9242; 21.7435; -157.9279; 21.746; -157.9302; 21.7468; -157.9316; 21.7482; -157.9418; 21.7546; -157.9551; 21.7586; -157.9783; 21.763; -157.9917; 21.763; -157.9972; 21.7616; -158.0082; 21.7553; -158.024; 21.7468; -158.0251; 21.7462; -158.0309; 21.7431; -158.0353; 21.7431; -158.0405; 21.742; -158.0449; 21.7409; -158.0501; 21.7399; -158.0571; 21.7355; -158.0623; 21.7301; -158.0676; 21.7247; -158.0719; 21.7192; -158.0789; 21.716; -158.0818; 21.7139; -158.0833; 21.7127; -158.0885; 21.7095; -158.0886; 21.7095; -158.0955; 21.703; -158.0998; 21.6975; -158.1033; 21.6921; -158.104; 21.6909; -158.1068; 21.6856; -158.1078; 21.6838; -158.1089; 21.6819; -158.1103; 21.6791; -158.1116; 21.6759; -158.1124; 21.6739; -158.1127; 21.6731; -158.1129; 21.6726; -158.1135; 21.6708; -158.1138; 21.67; -158.1143; 21.6687; -158.1147; 21.6672; -158.1165; 21.665; -158.1173; 21.6639; -158.1182; 21.6623; -158.119; 21.6607; -158.1202; 21.6573; -158.1206; 21.6638; -158.1213; 21.6646; -158.1222; 21.6657; -158.1261; 21.6635; -158.1281; 21.6625; -158.1283; 21.6623; -158.1334; 21.6586; -158.1342; 21.658; -158.1351; 21.6571; -158.1392; 21.6532; -158.1445; 21.6469; -158.1488; 21.642; -158.1555; 21.6397; -158.1665; 21.636; -158.175; 21.632; -158.187; 21.6326; -158.1996; 21.6345; -158.215; 21.6331; -158.2302; 21.6308; -158.2472; 21.6311; -158.2677; 21.6281; -158.2782; 21.6278; -158.2896; 21.6254; -158.3019; 21.6218; -158.3097; 21.6218; -158.3119; 21.6218; -158.3197; 21.6173; -158.3242; 21.6157; -158.3277; 21.6118; -158.3299; 21.6094; -158.335; 21.6046; -158.3395; 21.5967; -158.3421; 21.5912; -158.3447; 21.5832; -158.3447; 21.5777</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>Wetland</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="P26" t="inlineStr">
-        <is>
-          <t>study_site</t>
-        </is>
-      </c>
-      <c r="Q26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>6a2f0c6a-b4f6-430e-8281-e4adbd7de258</t>
-        </is>
-      </c>
-      <c r="C27">
-        <v>11</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Mycorrhizal network connectivity shapes seedling recruitment under closed canopy</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>MacPherson DL; Simard SW; Heinrich BR</t>
-        </is>
-      </c>
-      <c r="F27">
-        <v>2021</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>10.1038/s41559-021-01569-0</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>reviewed</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>564c9186-f70d-47f2-b285-55baee74f705</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>2026-02-28T09:30:02+00:00</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Hobart, City of Hobart, Tasmania, Australia; -42.8825; 147.3281; 10632745</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="P27" t="inlineStr">
-        <is>
-          <t>simple_group</t>
-        </is>
-      </c>
-      <c r="Q27">
-        <v>1</v>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>6a2f0c6a-b4f6-430e-8281-e4adbd7de258</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>study_site_1</t>
-        </is>
-      </c>
-      <c r="C28">
-        <v>11</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Mycorrhizal network connectivity shapes seedling recruitment under closed canopy</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>MacPherson DL; Simard SW; Heinrich BR</t>
-        </is>
-      </c>
-      <c r="F28">
-        <v>2021</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>10.1038/s41559-021-01569-0</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>reviewed</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>564c9186-f70d-47f2-b285-55baee74f705</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>2026-02-28T09:30:02+00:00</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Hobart, City of Hobart, Tasmania, Australia; -42.8825; 147.3281; 10632745</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>Forest</t>
-        </is>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>study_site</t>
-        </is>
-      </c>
-      <c r="Q28">
         <v>1</v>
       </c>
     </row>

</xml_diff>